<commit_message>
IDD Update (WDATA Forward)
</commit_message>
<xml_diff>
--- a/Document/IDD.xlsx
+++ b/Document/IDD.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="V:\SoC_Design\Document\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C9644CE-B4C7-46A8-9CB2-BE0B6BEBB16E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC941B3F-7F6D-47C9-B9E9-D04C64D437AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="15585" activeTab="1" xr2:uid="{813C5046-60F0-40FF-AAC7-48B46C31F73B}"/>
+    <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{813C5046-60F0-40FF-AAC7-48B46C31F73B}"/>
   </bookViews>
   <sheets>
     <sheet name="CPU" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="819" uniqueCount="366">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="828" uniqueCount="377">
   <si>
     <t>top_cpu</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -1121,11 +1121,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>u_alusrc_mux
-u_ex_mem_bridge</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>w_mem_reg_rdata2</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -1404,15 +1399,6 @@
   </si>
   <si>
     <t>엑셀 복붙용</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>w_mem_ctr_regwrite</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>u_mem_wb_bridge
-u_forward_regdst_mux</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
@@ -1443,17 +1429,9 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>u_forward_unit</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>w_mem_regdst_mux_reg</t>
   </si>
   <si>
-    <t>u_forward_regdst_mux</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>rt or rd Register (MEM)</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -1470,34 +1448,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>w_ctr_forward_a</t>
-  </si>
-  <si>
-    <t>w_ctr_forward_b</t>
-  </si>
-  <si>
-    <t>w_ex_forward_mux_data_a</t>
-  </si>
-  <si>
-    <t>w_ex_forward_mux_data_b</t>
-  </si>
-  <si>
-    <t>ForwardA Output</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>ForwardB Output</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>u_forward_a_mux</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>u_forward_b_mux</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>ForwardA MUX Data</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -1506,40 +1456,106 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
+    <t>u_alu_forwarding_unit</t>
+  </si>
+  <si>
+    <t>u_mem_wb_bridge
+u_alu_forward_mem_regdst_mux</t>
+  </si>
+  <si>
+    <t>u_alu_forward_mem_regdst_mux</t>
+  </si>
+  <si>
+    <t>w_ctr_alu_forward_a</t>
+  </si>
+  <si>
+    <t>w_ctr_alu_forward_b</t>
+  </si>
+  <si>
+    <t>ALU ForwardA Output</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>ALU ForwardB Output</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>u_alu_forward_a_mux</t>
+  </si>
+  <si>
+    <t>u_alu_forward_b_mux</t>
+  </si>
+  <si>
+    <t>u_mem_wb_bridge
+o_d_mem_addr
+u_alu_forward_a_mux
+u_alu_forward_b_mux</t>
+  </si>
+  <si>
     <t>u_ex_mem_bridge
-u_forward_unit</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">u_mem_wb_bridge
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="맑은 고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">o_d_mem_addr
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="맑은 고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>u_forward_a_mux
-u_forward_b_mux</t>
-    </r>
+u_alu_forwarding_unit</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>u_alu_forward_b_mux
+u_ex_mem_bridge</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>w_mem_regwrite</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>u_mem_wb_bridge
+u_alu_forwarding_unit</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>WDATA Forward Output</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>u_mem_wb_bridge
+u_alu_forward_mem_regdst_mux
+u_wdata_forward_unit</t>
+  </si>
+  <si>
+    <t>u_registers
+u_wdata_forwarding_unit</t>
+  </si>
+  <si>
+    <t>w_ctr_wdata_forward</t>
+  </si>
+  <si>
+    <t>u_wdata_forwarding_unit</t>
+  </si>
+  <si>
+    <t>w_ex_alu_forward_mux_data_a</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>w_ex_alu_forward_mux_data_b</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>u_alu_src_mux</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>w_mem_wdata_forward_mux_data</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>u_wdata_forward_mux</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>WDATA Forward MUX Data</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>u_memtoreg_mux
+u_wdata_forward_mux</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -2165,7 +2181,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="149">
+  <cellXfs count="147">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -2493,18 +2509,6 @@
     <xf numFmtId="176" fontId="2" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="3" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="2" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="2" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -2529,16 +2533,58 @@
     <xf numFmtId="3" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="6" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="6" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2556,62 +2602,26 @@
     <xf numFmtId="0" fontId="0" fillId="6" borderId="28" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="6" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="176" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2973,32 +2983,32 @@
   <sheetData>
     <row r="1" spans="2:19" ht="17.25" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="2" spans="2:19" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B2" s="143" t="s">
-        <v>0</v>
-      </c>
-      <c r="C2" s="144"/>
-      <c r="D2" s="144"/>
-      <c r="E2" s="144"/>
-      <c r="F2" s="144"/>
-      <c r="G2" s="145"/>
-      <c r="I2" s="122" t="s">
+      <c r="B2" s="131" t="s">
+        <v>0</v>
+      </c>
+      <c r="C2" s="132"/>
+      <c r="D2" s="132"/>
+      <c r="E2" s="132"/>
+      <c r="F2" s="132"/>
+      <c r="G2" s="133"/>
+      <c r="I2" s="117" t="s">
         <v>104</v>
       </c>
-      <c r="J2" s="123"/>
-      <c r="K2" s="122" t="s">
+      <c r="J2" s="119"/>
+      <c r="K2" s="117" t="s">
         <v>98</v>
       </c>
-      <c r="L2" s="124"/>
-      <c r="M2" s="123"/>
-      <c r="O2" s="122" t="s">
+      <c r="L2" s="118"/>
+      <c r="M2" s="119"/>
+      <c r="O2" s="117" t="s">
         <v>104</v>
       </c>
-      <c r="P2" s="123"/>
-      <c r="Q2" s="122" t="s">
+      <c r="P2" s="119"/>
+      <c r="Q2" s="117" t="s">
         <v>151</v>
       </c>
-      <c r="R2" s="124"/>
-      <c r="S2" s="123"/>
+      <c r="R2" s="118"/>
+      <c r="S2" s="119"/>
     </row>
     <row r="3" spans="2:19" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B3" s="34" t="s">
@@ -3019,24 +3029,24 @@
       <c r="G3" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="I3" s="132" t="s">
+      <c r="I3" s="126" t="s">
         <v>110</v>
       </c>
-      <c r="J3" s="133"/>
-      <c r="K3" s="134" t="s">
+      <c r="J3" s="127"/>
+      <c r="K3" s="128" t="s">
         <v>111</v>
       </c>
-      <c r="L3" s="135"/>
-      <c r="M3" s="136"/>
-      <c r="O3" s="132" t="s">
+      <c r="L3" s="129"/>
+      <c r="M3" s="130"/>
+      <c r="O3" s="126" t="s">
         <v>110</v>
       </c>
-      <c r="P3" s="133"/>
-      <c r="Q3" s="134" t="s">
+      <c r="P3" s="127"/>
+      <c r="Q3" s="128" t="s">
         <v>239</v>
       </c>
-      <c r="R3" s="135"/>
-      <c r="S3" s="136"/>
+      <c r="R3" s="129"/>
+      <c r="S3" s="130"/>
     </row>
     <row r="4" spans="2:19" x14ac:dyDescent="0.3">
       <c r="B4" s="35">
@@ -3057,24 +3067,24 @@
       <c r="G4" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="I4" s="132" t="s">
+      <c r="I4" s="126" t="s">
         <v>108</v>
       </c>
-      <c r="J4" s="133"/>
-      <c r="K4" s="132" t="s">
+      <c r="J4" s="127"/>
+      <c r="K4" s="126" t="s">
         <v>65</v>
       </c>
-      <c r="L4" s="137"/>
-      <c r="M4" s="133"/>
-      <c r="O4" s="132" t="s">
+      <c r="L4" s="140"/>
+      <c r="M4" s="127"/>
+      <c r="O4" s="126" t="s">
         <v>108</v>
       </c>
-      <c r="P4" s="133"/>
-      <c r="Q4" s="132" t="s">
+      <c r="P4" s="127"/>
+      <c r="Q4" s="126" t="s">
         <v>65</v>
       </c>
-      <c r="R4" s="137"/>
-      <c r="S4" s="133"/>
+      <c r="R4" s="140"/>
+      <c r="S4" s="127"/>
     </row>
     <row r="5" spans="2:19" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B5" s="54">
@@ -3095,24 +3105,24 @@
       <c r="G5" s="14" t="s">
         <v>9</v>
       </c>
-      <c r="I5" s="138" t="s">
+      <c r="I5" s="120" t="s">
         <v>8</v>
       </c>
-      <c r="J5" s="139"/>
-      <c r="K5" s="140" t="s">
+      <c r="J5" s="121"/>
+      <c r="K5" s="122" t="s">
         <v>103</v>
       </c>
-      <c r="L5" s="121"/>
-      <c r="M5" s="141"/>
-      <c r="O5" s="138" t="s">
+      <c r="L5" s="123"/>
+      <c r="M5" s="124"/>
+      <c r="O5" s="120" t="s">
         <v>8</v>
       </c>
-      <c r="P5" s="139"/>
-      <c r="Q5" s="140" t="s">
+      <c r="P5" s="121"/>
+      <c r="Q5" s="122" t="s">
         <v>152</v>
       </c>
-      <c r="R5" s="121"/>
-      <c r="S5" s="141"/>
+      <c r="R5" s="123"/>
+      <c r="S5" s="124"/>
     </row>
     <row r="6" spans="2:19" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B6" s="55">
@@ -3136,22 +3146,22 @@
       <c r="I6" s="67" t="s">
         <v>41</v>
       </c>
-      <c r="J6" s="130" t="s">
+      <c r="J6" s="125" t="s">
         <v>99</v>
       </c>
-      <c r="K6" s="130"/>
-      <c r="L6" s="130"/>
+      <c r="K6" s="125"/>
+      <c r="L6" s="125"/>
       <c r="M6" s="69" t="s">
         <v>8</v>
       </c>
       <c r="O6" s="67" t="s">
         <v>41</v>
       </c>
-      <c r="P6" s="130" t="s">
+      <c r="P6" s="125" t="s">
         <v>99</v>
       </c>
-      <c r="Q6" s="130"/>
-      <c r="R6" s="130"/>
+      <c r="Q6" s="125"/>
+      <c r="R6" s="125"/>
       <c r="S6" s="69" t="s">
         <v>8</v>
       </c>
@@ -3178,22 +3188,22 @@
       <c r="I7" s="70">
         <v>1</v>
       </c>
-      <c r="J7" s="142" t="s">
+      <c r="J7" s="134" t="s">
         <v>21</v>
       </c>
-      <c r="K7" s="142"/>
-      <c r="L7" s="142"/>
+      <c r="K7" s="134"/>
+      <c r="L7" s="134"/>
       <c r="M7" s="71" t="s">
         <v>134</v>
       </c>
       <c r="O7" s="87">
         <v>1</v>
       </c>
-      <c r="P7" s="131" t="s">
+      <c r="P7" s="141" t="s">
         <v>21</v>
       </c>
-      <c r="Q7" s="131"/>
-      <c r="R7" s="131"/>
+      <c r="Q7" s="141"/>
+      <c r="R7" s="141"/>
       <c r="S7" s="88" t="s">
         <v>134</v>
       </c>
@@ -3235,11 +3245,11 @@
       <c r="O8" s="80">
         <v>2</v>
       </c>
-      <c r="P8" s="121" t="s">
+      <c r="P8" s="123" t="s">
         <v>20</v>
       </c>
-      <c r="Q8" s="121"/>
-      <c r="R8" s="121"/>
+      <c r="Q8" s="123"/>
+      <c r="R8" s="123"/>
       <c r="S8" s="82" t="s">
         <v>135</v>
       </c>
@@ -3413,15 +3423,15 @@
       <c r="G12" s="30" t="s">
         <v>29</v>
       </c>
-      <c r="I12" s="125" t="s">
+      <c r="I12" s="135" t="s">
         <v>106</v>
       </c>
-      <c r="J12" s="126"/>
-      <c r="K12" s="127" t="s">
+      <c r="J12" s="136"/>
+      <c r="K12" s="137" t="s">
         <v>107</v>
       </c>
-      <c r="L12" s="128"/>
-      <c r="M12" s="129"/>
+      <c r="L12" s="138"/>
+      <c r="M12" s="139"/>
       <c r="O12" s="72">
         <v>3</v>
       </c>
@@ -3544,15 +3554,15 @@
       </c>
     </row>
     <row r="16" spans="2:19" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="O16" s="125" t="s">
+      <c r="O16" s="135" t="s">
         <v>106</v>
       </c>
-      <c r="P16" s="126"/>
-      <c r="Q16" s="127" t="s">
+      <c r="P16" s="136"/>
+      <c r="Q16" s="137" t="s">
         <v>242</v>
       </c>
-      <c r="R16" s="128"/>
-      <c r="S16" s="129"/>
+      <c r="R16" s="138"/>
+      <c r="S16" s="139"/>
     </row>
     <row r="17" spans="2:19" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B17" s="90" t="s">
@@ -3586,32 +3596,32 @@
         <v>1</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>347</v>
+        <v>351</v>
       </c>
       <c r="F18" s="2" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
       <c r="G18" s="5" t="s">
-        <v>358</v>
-      </c>
-      <c r="I18" s="122" t="s">
+        <v>356</v>
+      </c>
+      <c r="I18" s="117" t="s">
         <v>104</v>
       </c>
-      <c r="J18" s="123"/>
-      <c r="K18" s="122" t="s">
+      <c r="J18" s="119"/>
+      <c r="K18" s="117" t="s">
         <v>105</v>
       </c>
-      <c r="L18" s="124"/>
-      <c r="M18" s="123"/>
-      <c r="O18" s="122" t="s">
+      <c r="L18" s="118"/>
+      <c r="M18" s="119"/>
+      <c r="O18" s="117" t="s">
         <v>104</v>
       </c>
-      <c r="P18" s="123"/>
-      <c r="Q18" s="122" t="s">
+      <c r="P18" s="119"/>
+      <c r="Q18" s="117" t="s">
         <v>161</v>
       </c>
-      <c r="R18" s="124"/>
-      <c r="S18" s="123"/>
+      <c r="R18" s="118"/>
+      <c r="S18" s="119"/>
     </row>
     <row r="19" spans="2:19" x14ac:dyDescent="0.3">
       <c r="B19" s="33">
@@ -3625,32 +3635,32 @@
         <v>1</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>347</v>
+        <v>351</v>
       </c>
       <c r="F19" s="2" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="G19" s="5" t="s">
-        <v>359</v>
-      </c>
-      <c r="I19" s="132" t="s">
+        <v>357</v>
+      </c>
+      <c r="I19" s="126" t="s">
         <v>110</v>
       </c>
-      <c r="J19" s="133"/>
-      <c r="K19" s="134" t="s">
+      <c r="J19" s="127"/>
+      <c r="K19" s="128" t="s">
         <v>112</v>
       </c>
-      <c r="L19" s="135"/>
-      <c r="M19" s="136"/>
-      <c r="O19" s="132" t="s">
+      <c r="L19" s="129"/>
+      <c r="M19" s="130"/>
+      <c r="O19" s="126" t="s">
         <v>110</v>
       </c>
-      <c r="P19" s="133"/>
-      <c r="Q19" s="134" t="s">
+      <c r="P19" s="127"/>
+      <c r="Q19" s="128" t="s">
         <v>239</v>
       </c>
-      <c r="R19" s="135"/>
-      <c r="S19" s="136"/>
+      <c r="R19" s="129"/>
+      <c r="S19" s="130"/>
     </row>
     <row r="20" spans="2:19" ht="33" x14ac:dyDescent="0.3">
       <c r="B20" s="33">
@@ -3672,24 +3682,24 @@
       <c r="G20" s="99" t="s">
         <v>199</v>
       </c>
-      <c r="I20" s="132" t="s">
+      <c r="I20" s="126" t="s">
         <v>108</v>
       </c>
-      <c r="J20" s="133"/>
-      <c r="K20" s="134" t="s">
+      <c r="J20" s="127"/>
+      <c r="K20" s="128" t="s">
         <v>109</v>
       </c>
-      <c r="L20" s="135"/>
-      <c r="M20" s="136"/>
-      <c r="O20" s="132" t="s">
+      <c r="L20" s="129"/>
+      <c r="M20" s="130"/>
+      <c r="O20" s="126" t="s">
         <v>108</v>
       </c>
-      <c r="P20" s="133"/>
-      <c r="Q20" s="132" t="s">
+      <c r="P20" s="127"/>
+      <c r="Q20" s="126" t="s">
         <v>65</v>
       </c>
-      <c r="R20" s="137"/>
-      <c r="S20" s="133"/>
+      <c r="R20" s="140"/>
+      <c r="S20" s="127"/>
     </row>
     <row r="21" spans="2:19" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B21" s="33">
@@ -3697,7 +3707,7 @@
         <v>4</v>
       </c>
       <c r="C21" s="3" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="D21" s="1">
         <v>1</v>
@@ -3711,24 +3721,24 @@
       <c r="G21" s="5" t="s">
         <v>85</v>
       </c>
-      <c r="I21" s="138" t="s">
+      <c r="I21" s="120" t="s">
         <v>8</v>
       </c>
-      <c r="J21" s="139"/>
-      <c r="K21" s="140" t="s">
+      <c r="J21" s="121"/>
+      <c r="K21" s="122" t="s">
         <v>126</v>
       </c>
-      <c r="L21" s="121"/>
-      <c r="M21" s="141"/>
-      <c r="O21" s="138" t="s">
+      <c r="L21" s="123"/>
+      <c r="M21" s="124"/>
+      <c r="O21" s="120" t="s">
         <v>8</v>
       </c>
-      <c r="P21" s="139"/>
-      <c r="Q21" s="140" t="s">
+      <c r="P21" s="121"/>
+      <c r="Q21" s="122" t="s">
         <v>162</v>
       </c>
-      <c r="R21" s="121"/>
-      <c r="S21" s="141"/>
+      <c r="R21" s="123"/>
+      <c r="S21" s="124"/>
     </row>
     <row r="22" spans="2:19" ht="33.75" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B22" s="33">
@@ -3736,7 +3746,7 @@
         <v>5</v>
       </c>
       <c r="C22" s="3" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="D22" s="1">
         <v>4</v>
@@ -3753,22 +3763,22 @@
       <c r="I22" s="67" t="s">
         <v>41</v>
       </c>
-      <c r="J22" s="130" t="s">
+      <c r="J22" s="125" t="s">
         <v>99</v>
       </c>
-      <c r="K22" s="130"/>
-      <c r="L22" s="130"/>
+      <c r="K22" s="125"/>
+      <c r="L22" s="125"/>
       <c r="M22" s="69" t="s">
         <v>8</v>
       </c>
       <c r="O22" s="67" t="s">
         <v>41</v>
       </c>
-      <c r="P22" s="130" t="s">
+      <c r="P22" s="125" t="s">
         <v>99</v>
       </c>
-      <c r="Q22" s="130"/>
-      <c r="R22" s="130"/>
+      <c r="Q22" s="125"/>
+      <c r="R22" s="125"/>
       <c r="S22" s="69" t="s">
         <v>8</v>
       </c>
@@ -3796,22 +3806,22 @@
       <c r="I23" s="70">
         <v>1</v>
       </c>
-      <c r="J23" s="142" t="s">
+      <c r="J23" s="134" t="s">
         <v>20</v>
       </c>
-      <c r="K23" s="142"/>
-      <c r="L23" s="142"/>
+      <c r="K23" s="134"/>
+      <c r="L23" s="134"/>
       <c r="M23" s="71" t="s">
         <v>135</v>
       </c>
       <c r="O23" s="87">
         <v>1</v>
       </c>
-      <c r="P23" s="131" t="s">
+      <c r="P23" s="141" t="s">
         <v>21</v>
       </c>
-      <c r="Q23" s="131"/>
-      <c r="R23" s="131"/>
+      <c r="Q23" s="141"/>
+      <c r="R23" s="141"/>
       <c r="S23" s="88" t="s">
         <v>134</v>
       </c>
@@ -3822,7 +3832,7 @@
         <v>7</v>
       </c>
       <c r="C24" s="3" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="D24" s="1">
         <v>1</v>
@@ -3831,7 +3841,7 @@
         <v>80</v>
       </c>
       <c r="F24" s="2" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="G24" s="5" t="s">
         <v>86</v>
@@ -3854,11 +3864,11 @@
       <c r="O24" s="80">
         <v>2</v>
       </c>
-      <c r="P24" s="121" t="s">
+      <c r="P24" s="123" t="s">
         <v>20</v>
       </c>
-      <c r="Q24" s="121"/>
-      <c r="R24" s="121"/>
+      <c r="Q24" s="123"/>
+      <c r="R24" s="123"/>
       <c r="S24" s="82" t="s">
         <v>135</v>
       </c>
@@ -3914,13 +3924,13 @@
         <v>8</v>
       </c>
     </row>
-    <row r="26" spans="2:19" x14ac:dyDescent="0.3">
+    <row r="26" spans="2:19" ht="33" x14ac:dyDescent="0.3">
       <c r="B26" s="33">
         <f t="shared" si="0"/>
         <v>9</v>
       </c>
       <c r="C26" s="3" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="D26" s="90" t="s">
         <v>20</v>
@@ -3929,7 +3939,7 @@
         <v>81</v>
       </c>
       <c r="F26" s="103" t="s">
-        <v>361</v>
+        <v>77</v>
       </c>
       <c r="G26" s="5" t="s">
         <v>83</v>
@@ -3971,7 +3981,7 @@
         <v>10</v>
       </c>
       <c r="C27" s="3" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="D27" s="1">
         <v>1</v>
@@ -3980,10 +3990,10 @@
         <v>243</v>
       </c>
       <c r="F27" s="2" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="G27" s="5" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="I27" s="83">
         <v>3</v>
@@ -4022,7 +4032,7 @@
         <v>11</v>
       </c>
       <c r="C28" s="3" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="D28" s="90" t="s">
         <v>20</v>
@@ -4073,7 +4083,7 @@
         <v>12</v>
       </c>
       <c r="C29" s="3" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="D29" s="90" t="s">
         <v>21</v>
@@ -4175,13 +4185,13 @@
         <v>14</v>
       </c>
       <c r="C31" s="3" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="D31" s="1">
         <v>1</v>
       </c>
       <c r="E31" s="102" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="F31" s="2" t="s">
         <v>53</v>
@@ -4226,7 +4236,7 @@
         <v>15</v>
       </c>
       <c r="C32" s="3" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="D32" s="1">
         <v>1</v>
@@ -4238,17 +4248,17 @@
         <v>36</v>
       </c>
       <c r="G32" s="5" t="s">
-        <v>272</v>
-      </c>
-      <c r="I32" s="125" t="s">
+        <v>271</v>
+      </c>
+      <c r="I32" s="135" t="s">
         <v>106</v>
       </c>
-      <c r="J32" s="126"/>
-      <c r="K32" s="127" t="s">
+      <c r="J32" s="136"/>
+      <c r="K32" s="137" t="s">
         <v>80</v>
       </c>
-      <c r="L32" s="128"/>
-      <c r="M32" s="129"/>
+      <c r="L32" s="138"/>
+      <c r="M32" s="139"/>
       <c r="O32" s="83">
         <v>7</v>
       </c>
@@ -4271,7 +4281,7 @@
         <v>16</v>
       </c>
       <c r="C33" s="3" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="D33" s="1">
         <v>1</v>
@@ -4283,7 +4293,7 @@
         <v>244</v>
       </c>
       <c r="G33" s="5" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="O33" s="83">
         <v>8</v>
@@ -4343,7 +4353,7 @@
         <v>18</v>
       </c>
       <c r="C35" s="3" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="D35" s="90" t="s">
         <v>56</v>
@@ -4355,7 +4365,7 @@
         <v>244</v>
       </c>
       <c r="G35" s="5" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="O35" s="80">
         <v>10</v>
@@ -4379,7 +4389,7 @@
         <v>19</v>
       </c>
       <c r="C36" s="3" t="s">
-        <v>343</v>
+        <v>340</v>
       </c>
       <c r="D36" s="90" t="s">
         <v>56</v>
@@ -4388,20 +4398,20 @@
         <v>243</v>
       </c>
       <c r="F36" s="2" t="s">
-        <v>347</v>
+        <v>351</v>
       </c>
       <c r="G36" s="5" t="s">
-        <v>344</v>
-      </c>
-      <c r="O36" s="125" t="s">
+        <v>341</v>
+      </c>
+      <c r="O36" s="135" t="s">
         <v>106</v>
       </c>
-      <c r="P36" s="126"/>
-      <c r="Q36" s="127" t="s">
+      <c r="P36" s="136"/>
+      <c r="Q36" s="137" t="s">
         <v>243</v>
       </c>
-      <c r="R36" s="128"/>
-      <c r="S36" s="129"/>
+      <c r="R36" s="138"/>
+      <c r="S36" s="139"/>
     </row>
     <row r="37" spans="2:19" ht="33.75" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B37" s="33">
@@ -4409,7 +4419,7 @@
         <v>20</v>
       </c>
       <c r="C37" s="3" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="D37" s="90" t="s">
         <v>56</v>
@@ -4418,10 +4428,10 @@
         <v>243</v>
       </c>
       <c r="F37" s="103" t="s">
-        <v>364</v>
+        <v>361</v>
       </c>
       <c r="G37" s="5" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
     </row>
     <row r="38" spans="2:19" ht="33" x14ac:dyDescent="0.3">
@@ -4430,77 +4440,77 @@
         <v>21</v>
       </c>
       <c r="C38" s="3" t="s">
-        <v>356</v>
+        <v>370</v>
       </c>
       <c r="D38" s="90" t="s">
         <v>20</v>
       </c>
       <c r="E38" s="1" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
       <c r="F38" s="103" t="s">
         <v>77</v>
       </c>
       <c r="G38" s="5" t="s">
-        <v>362</v>
-      </c>
-      <c r="I38" s="122" t="s">
+        <v>349</v>
+      </c>
+      <c r="I38" s="117" t="s">
         <v>104</v>
       </c>
-      <c r="J38" s="123"/>
-      <c r="K38" s="122" t="s">
+      <c r="J38" s="119"/>
+      <c r="K38" s="117" t="s">
         <v>124</v>
       </c>
-      <c r="L38" s="124"/>
-      <c r="M38" s="123"/>
-      <c r="O38" s="122" t="s">
+      <c r="L38" s="118"/>
+      <c r="M38" s="119"/>
+      <c r="O38" s="117" t="s">
         <v>104</v>
       </c>
-      <c r="P38" s="123"/>
-      <c r="Q38" s="122" t="s">
+      <c r="P38" s="119"/>
+      <c r="Q38" s="117" t="s">
         <v>175</v>
       </c>
-      <c r="R38" s="124"/>
-      <c r="S38" s="123"/>
-    </row>
-    <row r="39" spans="2:19" ht="33" x14ac:dyDescent="0.3">
+      <c r="R38" s="118"/>
+      <c r="S38" s="119"/>
+    </row>
+    <row r="39" spans="2:19" x14ac:dyDescent="0.3">
       <c r="B39" s="33">
         <f t="shared" si="0"/>
         <v>22</v>
       </c>
       <c r="C39" s="3" t="s">
-        <v>357</v>
+        <v>371</v>
       </c>
       <c r="D39" s="90" t="s">
         <v>20</v>
       </c>
       <c r="E39" s="1" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="F39" s="103" t="s">
-        <v>77</v>
+        <v>372</v>
       </c>
       <c r="G39" s="5" t="s">
-        <v>363</v>
-      </c>
-      <c r="I39" s="132" t="s">
+        <v>350</v>
+      </c>
+      <c r="I39" s="126" t="s">
         <v>110</v>
       </c>
-      <c r="J39" s="133"/>
-      <c r="K39" s="134" t="s">
+      <c r="J39" s="127"/>
+      <c r="K39" s="128" t="s">
         <v>125</v>
       </c>
-      <c r="L39" s="135"/>
-      <c r="M39" s="136"/>
-      <c r="O39" s="132" t="s">
+      <c r="L39" s="129"/>
+      <c r="M39" s="130"/>
+      <c r="O39" s="126" t="s">
         <v>110</v>
       </c>
-      <c r="P39" s="133"/>
-      <c r="Q39" s="134" t="s">
+      <c r="P39" s="127"/>
+      <c r="Q39" s="128" t="s">
         <v>239</v>
       </c>
-      <c r="R39" s="135"/>
-      <c r="S39" s="136"/>
+      <c r="R39" s="129"/>
+      <c r="S39" s="130"/>
     </row>
     <row r="40" spans="2:19" x14ac:dyDescent="0.3">
       <c r="B40" s="33">
@@ -4508,7 +4518,7 @@
         <v>23</v>
       </c>
       <c r="C40" s="3" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="D40" s="90" t="s">
         <v>20</v>
@@ -4522,24 +4532,24 @@
       <c r="G40" s="5" t="s">
         <v>88</v>
       </c>
-      <c r="I40" s="132" t="s">
+      <c r="I40" s="126" t="s">
         <v>108</v>
       </c>
-      <c r="J40" s="133"/>
-      <c r="K40" s="134" t="s">
+      <c r="J40" s="127"/>
+      <c r="K40" s="128" t="s">
         <v>109</v>
       </c>
-      <c r="L40" s="135"/>
-      <c r="M40" s="136"/>
-      <c r="O40" s="132" t="s">
+      <c r="L40" s="129"/>
+      <c r="M40" s="130"/>
+      <c r="O40" s="126" t="s">
         <v>108</v>
       </c>
-      <c r="P40" s="133"/>
-      <c r="Q40" s="132" t="s">
+      <c r="P40" s="127"/>
+      <c r="Q40" s="126" t="s">
         <v>65</v>
       </c>
-      <c r="R40" s="137"/>
-      <c r="S40" s="133"/>
+      <c r="R40" s="140"/>
+      <c r="S40" s="127"/>
     </row>
     <row r="41" spans="2:19" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B41" s="33">
@@ -4561,24 +4571,24 @@
       <c r="G41" s="5" t="s">
         <v>237</v>
       </c>
-      <c r="I41" s="138" t="s">
+      <c r="I41" s="120" t="s">
         <v>8</v>
       </c>
-      <c r="J41" s="139"/>
-      <c r="K41" s="140" t="s">
+      <c r="J41" s="121"/>
+      <c r="K41" s="122" t="s">
         <v>127</v>
       </c>
-      <c r="L41" s="121"/>
-      <c r="M41" s="141"/>
-      <c r="O41" s="138" t="s">
+      <c r="L41" s="123"/>
+      <c r="M41" s="124"/>
+      <c r="O41" s="120" t="s">
         <v>8</v>
       </c>
-      <c r="P41" s="139"/>
-      <c r="Q41" s="140" t="s">
+      <c r="P41" s="121"/>
+      <c r="Q41" s="122" t="s">
         <v>176</v>
       </c>
-      <c r="R41" s="121"/>
-      <c r="S41" s="141"/>
+      <c r="R41" s="123"/>
+      <c r="S41" s="124"/>
     </row>
     <row r="42" spans="2:19" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B42" s="33">
@@ -4586,7 +4596,7 @@
         <v>25</v>
       </c>
       <c r="C42" s="97" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="D42" s="90" t="s">
         <v>21</v>
@@ -4598,27 +4608,27 @@
         <v>35</v>
       </c>
       <c r="G42" s="99" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="I42" s="67" t="s">
         <v>41</v>
       </c>
-      <c r="J42" s="130" t="s">
+      <c r="J42" s="125" t="s">
         <v>99</v>
       </c>
-      <c r="K42" s="130"/>
-      <c r="L42" s="130"/>
+      <c r="K42" s="125"/>
+      <c r="L42" s="125"/>
       <c r="M42" s="69" t="s">
         <v>8</v>
       </c>
       <c r="O42" s="67" t="s">
         <v>41</v>
       </c>
-      <c r="P42" s="130" t="s">
+      <c r="P42" s="125" t="s">
         <v>99</v>
       </c>
-      <c r="Q42" s="130"/>
-      <c r="R42" s="130"/>
+      <c r="Q42" s="125"/>
+      <c r="R42" s="125"/>
       <c r="S42" s="69" t="s">
         <v>8</v>
       </c>
@@ -4629,7 +4639,7 @@
         <v>26</v>
       </c>
       <c r="C43" s="3" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="D43" s="90" t="s">
         <v>20</v>
@@ -4646,22 +4656,22 @@
       <c r="I43" s="70">
         <v>1</v>
       </c>
-      <c r="J43" s="142" t="s">
+      <c r="J43" s="134" t="s">
         <v>20</v>
       </c>
-      <c r="K43" s="142"/>
-      <c r="L43" s="142"/>
+      <c r="K43" s="134"/>
+      <c r="L43" s="134"/>
       <c r="M43" s="71" t="s">
         <v>135</v>
       </c>
       <c r="O43" s="87">
         <v>1</v>
       </c>
-      <c r="P43" s="131" t="s">
+      <c r="P43" s="141" t="s">
         <v>21</v>
       </c>
-      <c r="Q43" s="131"/>
-      <c r="R43" s="131"/>
+      <c r="Q43" s="141"/>
+      <c r="R43" s="141"/>
       <c r="S43" s="88" t="s">
         <v>134</v>
       </c>
@@ -4677,10 +4687,10 @@
       <c r="D44" s="1">
         <v>1</v>
       </c>
-      <c r="E44" s="118" t="s">
+      <c r="E44" s="114" t="s">
         <v>243</v>
       </c>
-      <c r="F44" s="118" t="s">
+      <c r="F44" s="114" t="s">
         <v>244</v>
       </c>
       <c r="G44" s="5" t="s">
@@ -4704,11 +4714,11 @@
       <c r="O44" s="80">
         <v>2</v>
       </c>
-      <c r="P44" s="121" t="s">
+      <c r="P44" s="123" t="s">
         <v>20</v>
       </c>
-      <c r="Q44" s="121"/>
-      <c r="R44" s="121"/>
+      <c r="Q44" s="123"/>
+      <c r="R44" s="123"/>
       <c r="S44" s="82" t="s">
         <v>135</v>
       </c>
@@ -4719,7 +4729,7 @@
         <v>28</v>
       </c>
       <c r="C45" s="3" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="D45" s="1">
         <v>1</v>
@@ -4731,7 +4741,7 @@
         <v>244</v>
       </c>
       <c r="G45" s="5" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="I45" s="72">
         <v>1</v>
@@ -4775,10 +4785,10 @@
       <c r="D46" s="1">
         <v>1</v>
       </c>
-      <c r="E46" s="118" t="s">
+      <c r="E46" s="114" t="s">
         <v>243</v>
       </c>
-      <c r="F46" s="118" t="s">
+      <c r="F46" s="114" t="s">
         <v>244</v>
       </c>
       <c r="G46" s="5" t="s">
@@ -4830,7 +4840,7 @@
         <v>240</v>
       </c>
       <c r="F47" s="103" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
       <c r="G47" s="5" t="s">
         <v>226</v>
@@ -4871,30 +4881,30 @@
         <f t="shared" si="0"/>
         <v>31</v>
       </c>
-      <c r="C48" s="116" t="s">
+      <c r="C48" s="112" t="s">
         <v>225</v>
       </c>
-      <c r="D48" s="117" t="s">
+      <c r="D48" s="113" t="s">
         <v>20</v>
       </c>
-      <c r="E48" s="115" t="s">
+      <c r="E48" s="111" t="s">
         <v>240</v>
       </c>
-      <c r="F48" s="119" t="s">
-        <v>266</v>
-      </c>
-      <c r="G48" s="116" t="s">
+      <c r="F48" s="115" t="s">
+        <v>362</v>
+      </c>
+      <c r="G48" s="112" t="s">
         <v>227</v>
       </c>
-      <c r="I48" s="125" t="s">
+      <c r="I48" s="135" t="s">
         <v>106</v>
       </c>
-      <c r="J48" s="126"/>
-      <c r="K48" s="127" t="s">
+      <c r="J48" s="136"/>
+      <c r="K48" s="137" t="s">
         <v>66</v>
       </c>
-      <c r="L48" s="128"/>
-      <c r="M48" s="129"/>
+      <c r="L48" s="138"/>
+      <c r="M48" s="139"/>
       <c r="O48" s="83">
         <v>3</v>
       </c>
@@ -4917,7 +4927,7 @@
         <v>32</v>
       </c>
       <c r="C49" s="3" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="D49" s="1">
         <v>1</v>
@@ -4925,11 +4935,11 @@
       <c r="E49" s="2" t="s">
         <v>243</v>
       </c>
-      <c r="F49" s="2" t="s">
+      <c r="F49" s="103" t="s">
         <v>244</v>
       </c>
       <c r="G49" s="5" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="O49" s="83">
         <v>4</v>
@@ -4948,12 +4958,12 @@
       </c>
     </row>
     <row r="50" spans="2:19" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B50" s="120">
+      <c r="B50" s="116">
         <f t="shared" si="0"/>
         <v>33</v>
       </c>
       <c r="C50" s="3" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="D50" s="90" t="s">
         <v>49</v>
@@ -4962,7 +4972,7 @@
         <v>47</v>
       </c>
       <c r="F50" s="1" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="G50" s="5" t="s">
         <v>54</v>
@@ -4989,13 +4999,13 @@
         <v>34</v>
       </c>
       <c r="C51" s="3" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="D51" s="90" t="s">
         <v>20</v>
       </c>
       <c r="E51" s="1" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="F51" s="2" t="s">
         <v>40</v>
@@ -5003,15 +5013,15 @@
       <c r="G51" s="5" t="s">
         <v>52</v>
       </c>
-      <c r="I51" s="122" t="s">
+      <c r="I51" s="117" t="s">
         <v>104</v>
       </c>
-      <c r="J51" s="123"/>
-      <c r="K51" s="122" t="s">
+      <c r="J51" s="119"/>
+      <c r="K51" s="117" t="s">
         <v>131</v>
       </c>
-      <c r="L51" s="124"/>
-      <c r="M51" s="123"/>
+      <c r="L51" s="118"/>
+      <c r="M51" s="119"/>
       <c r="O51" s="83">
         <v>6</v>
       </c>
@@ -5048,15 +5058,15 @@
       <c r="G52" s="5" t="s">
         <v>230</v>
       </c>
-      <c r="I52" s="132" t="s">
+      <c r="I52" s="126" t="s">
         <v>110</v>
       </c>
-      <c r="J52" s="133"/>
-      <c r="K52" s="134" t="s">
+      <c r="J52" s="127"/>
+      <c r="K52" s="128" t="s">
         <v>132</v>
       </c>
-      <c r="L52" s="135"/>
-      <c r="M52" s="136"/>
+      <c r="L52" s="129"/>
+      <c r="M52" s="130"/>
       <c r="O52" s="83">
         <v>7</v>
       </c>
@@ -5093,15 +5103,15 @@
       <c r="G53" s="5" t="s">
         <v>195</v>
       </c>
-      <c r="I53" s="132" t="s">
+      <c r="I53" s="126" t="s">
         <v>108</v>
       </c>
-      <c r="J53" s="133"/>
-      <c r="K53" s="134" t="s">
+      <c r="J53" s="127"/>
+      <c r="K53" s="128" t="s">
         <v>109</v>
       </c>
-      <c r="L53" s="135"/>
-      <c r="M53" s="136"/>
+      <c r="L53" s="129"/>
+      <c r="M53" s="130"/>
       <c r="O53" s="83">
         <v>8</v>
       </c>
@@ -5138,15 +5148,15 @@
       <c r="G54" s="99" t="s">
         <v>196</v>
       </c>
-      <c r="I54" s="138" t="s">
+      <c r="I54" s="120" t="s">
         <v>8</v>
       </c>
-      <c r="J54" s="139"/>
-      <c r="K54" s="140" t="s">
+      <c r="J54" s="121"/>
+      <c r="K54" s="122" t="s">
         <v>133</v>
       </c>
-      <c r="L54" s="121"/>
-      <c r="M54" s="141"/>
+      <c r="L54" s="123"/>
+      <c r="M54" s="124"/>
       <c r="O54" s="83">
         <v>9</v>
       </c>
@@ -5186,11 +5196,11 @@
       <c r="I55" s="67" t="s">
         <v>41</v>
       </c>
-      <c r="J55" s="130" t="s">
+      <c r="J55" s="125" t="s">
         <v>99</v>
       </c>
-      <c r="K55" s="130"/>
-      <c r="L55" s="130"/>
+      <c r="K55" s="125"/>
+      <c r="L55" s="125"/>
       <c r="M55" s="69" t="s">
         <v>8</v>
       </c>
@@ -5233,23 +5243,23 @@
       <c r="I56" s="87">
         <v>1</v>
       </c>
-      <c r="J56" s="131" t="s">
+      <c r="J56" s="141" t="s">
         <v>20</v>
       </c>
-      <c r="K56" s="131"/>
-      <c r="L56" s="131"/>
+      <c r="K56" s="141"/>
+      <c r="L56" s="141"/>
       <c r="M56" s="88" t="s">
         <v>135</v>
       </c>
-      <c r="O56" s="125" t="s">
+      <c r="O56" s="135" t="s">
         <v>106</v>
       </c>
-      <c r="P56" s="126"/>
-      <c r="Q56" s="127" t="s">
+      <c r="P56" s="136"/>
+      <c r="Q56" s="137" t="s">
         <v>244</v>
       </c>
-      <c r="R56" s="128"/>
-      <c r="S56" s="129"/>
+      <c r="R56" s="138"/>
+      <c r="S56" s="139"/>
     </row>
     <row r="57" spans="2:19" ht="33.75" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B57" s="33">
@@ -5274,11 +5284,11 @@
       <c r="I57" s="80">
         <v>2</v>
       </c>
-      <c r="J57" s="121" t="s">
+      <c r="J57" s="123" t="s">
         <v>55</v>
       </c>
-      <c r="K57" s="121"/>
-      <c r="L57" s="121"/>
+      <c r="K57" s="123"/>
+      <c r="L57" s="123"/>
       <c r="M57" s="89" t="s">
         <v>136</v>
       </c>
@@ -5318,15 +5328,15 @@
       <c r="M58" s="69" t="s">
         <v>8</v>
       </c>
-      <c r="O58" s="122" t="s">
+      <c r="O58" s="117" t="s">
         <v>104</v>
       </c>
-      <c r="P58" s="123"/>
-      <c r="Q58" s="122" t="s">
+      <c r="P58" s="119"/>
+      <c r="Q58" s="117" t="s">
         <v>186</v>
       </c>
-      <c r="R58" s="124"/>
-      <c r="S58" s="123"/>
+      <c r="R58" s="118"/>
+      <c r="S58" s="119"/>
     </row>
     <row r="59" spans="2:19" x14ac:dyDescent="0.3">
       <c r="B59" s="33">
@@ -5363,15 +5373,15 @@
       <c r="M59" s="75" t="s">
         <v>59</v>
       </c>
-      <c r="O59" s="132" t="s">
+      <c r="O59" s="126" t="s">
         <v>110</v>
       </c>
-      <c r="P59" s="133"/>
-      <c r="Q59" s="134" t="s">
+      <c r="P59" s="127"/>
+      <c r="Q59" s="128" t="s">
         <v>239</v>
       </c>
-      <c r="R59" s="135"/>
-      <c r="S59" s="136"/>
+      <c r="R59" s="129"/>
+      <c r="S59" s="130"/>
     </row>
     <row r="60" spans="2:19" x14ac:dyDescent="0.3">
       <c r="B60" s="33">
@@ -5379,7 +5389,7 @@
         <v>43</v>
       </c>
       <c r="C60" s="3" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="D60" s="90" t="s">
         <v>57</v>
@@ -5408,15 +5418,15 @@
       <c r="M60" s="79" t="s">
         <v>67</v>
       </c>
-      <c r="O60" s="132" t="s">
+      <c r="O60" s="126" t="s">
         <v>108</v>
       </c>
-      <c r="P60" s="133"/>
-      <c r="Q60" s="132" t="s">
+      <c r="P60" s="127"/>
+      <c r="Q60" s="126" t="s">
         <v>65</v>
       </c>
-      <c r="R60" s="137"/>
-      <c r="S60" s="133"/>
+      <c r="R60" s="140"/>
+      <c r="S60" s="127"/>
     </row>
     <row r="61" spans="2:19" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B61" s="33">
@@ -5453,15 +5463,15 @@
       <c r="M61" s="85" t="s">
         <v>147</v>
       </c>
-      <c r="O61" s="138" t="s">
+      <c r="O61" s="120" t="s">
         <v>8</v>
       </c>
-      <c r="P61" s="139"/>
-      <c r="Q61" s="140" t="s">
+      <c r="P61" s="121"/>
+      <c r="Q61" s="122" t="s">
         <v>187</v>
       </c>
-      <c r="R61" s="121"/>
-      <c r="S61" s="141"/>
+      <c r="R61" s="123"/>
+      <c r="S61" s="124"/>
     </row>
     <row r="62" spans="2:19" ht="33.75" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B62" s="33">
@@ -5469,7 +5479,7 @@
         <v>45</v>
       </c>
       <c r="C62" s="97" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="D62" s="101" t="s">
         <v>45</v>
@@ -5501,11 +5511,11 @@
       <c r="O62" s="67" t="s">
         <v>41</v>
       </c>
-      <c r="P62" s="130" t="s">
+      <c r="P62" s="125" t="s">
         <v>99</v>
       </c>
-      <c r="Q62" s="130"/>
-      <c r="R62" s="130"/>
+      <c r="Q62" s="125"/>
+      <c r="R62" s="125"/>
       <c r="S62" s="69" t="s">
         <v>8</v>
       </c>
@@ -5516,7 +5526,7 @@
         <v>46</v>
       </c>
       <c r="C63" s="3" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="D63" s="90" t="s">
         <v>55</v>
@@ -5548,11 +5558,11 @@
       <c r="O63" s="87">
         <v>1</v>
       </c>
-      <c r="P63" s="131" t="s">
+      <c r="P63" s="141" t="s">
         <v>21</v>
       </c>
-      <c r="Q63" s="131"/>
-      <c r="R63" s="131"/>
+      <c r="Q63" s="141"/>
+      <c r="R63" s="141"/>
       <c r="S63" s="88" t="s">
         <v>134</v>
       </c>
@@ -5563,7 +5573,7 @@
         <v>47</v>
       </c>
       <c r="C64" s="3" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="D64" s="90" t="s">
         <v>56</v>
@@ -5575,7 +5585,7 @@
         <v>243</v>
       </c>
       <c r="G64" s="5" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="I64" s="83">
         <v>6</v>
@@ -5595,11 +5605,11 @@
       <c r="O64" s="80">
         <v>2</v>
       </c>
-      <c r="P64" s="121" t="s">
+      <c r="P64" s="123" t="s">
         <v>20</v>
       </c>
-      <c r="Q64" s="121"/>
-      <c r="R64" s="121"/>
+      <c r="Q64" s="123"/>
+      <c r="R64" s="123"/>
       <c r="S64" s="82" t="s">
         <v>135</v>
       </c>
@@ -5610,7 +5620,7 @@
         <v>48</v>
       </c>
       <c r="C65" s="3" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="D65" s="90" t="s">
         <v>56</v>
@@ -5619,10 +5629,10 @@
         <v>44</v>
       </c>
       <c r="F65" s="103" t="s">
-        <v>346</v>
+        <v>343</v>
       </c>
       <c r="G65" s="5" t="s">
-        <v>345</v>
+        <v>342</v>
       </c>
       <c r="I65" s="83">
         <v>7</v>
@@ -5661,7 +5671,7 @@
         <v>49</v>
       </c>
       <c r="C66" s="3" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="D66" s="90" t="s">
         <v>56</v>
@@ -5673,7 +5683,7 @@
         <v>62</v>
       </c>
       <c r="G66" s="5" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="I66" s="83">
         <v>8</v>
@@ -5712,7 +5722,7 @@
         <v>50</v>
       </c>
       <c r="C67" s="3" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="D67" s="1">
         <v>5</v>
@@ -5769,7 +5779,7 @@
         <v>20</v>
       </c>
       <c r="E68" s="102" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="F68" s="2" t="s">
         <v>243</v>
@@ -5822,7 +5832,7 @@
       <c r="E69" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="F69" s="118" t="s">
+      <c r="F69" s="114" t="s">
         <v>243</v>
       </c>
       <c r="G69" s="5" t="s">
@@ -5924,7 +5934,7 @@
       <c r="E71" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="F71" s="118" t="s">
+      <c r="F71" s="114" t="s">
         <v>243</v>
       </c>
       <c r="G71" s="5" t="s">
@@ -5975,49 +5985,49 @@
       <c r="E72" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="F72" s="115" t="s">
+      <c r="F72" s="111" t="s">
         <v>240</v>
       </c>
       <c r="G72" s="5" t="s">
         <v>212</v>
       </c>
-      <c r="I72" s="125" t="s">
+      <c r="I72" s="135" t="s">
         <v>106</v>
       </c>
-      <c r="J72" s="126"/>
-      <c r="K72" s="127" t="s">
+      <c r="J72" s="136"/>
+      <c r="K72" s="137" t="s">
         <v>58</v>
       </c>
-      <c r="L72" s="128"/>
-      <c r="M72" s="129"/>
-      <c r="O72" s="125" t="s">
+      <c r="L72" s="138"/>
+      <c r="M72" s="139"/>
+      <c r="O72" s="135" t="s">
         <v>106</v>
       </c>
-      <c r="P72" s="126"/>
-      <c r="Q72" s="127" t="s">
+      <c r="P72" s="136"/>
+      <c r="Q72" s="137" t="s">
         <v>245</v>
       </c>
-      <c r="R72" s="128"/>
-      <c r="S72" s="129"/>
+      <c r="R72" s="138"/>
+      <c r="S72" s="139"/>
     </row>
     <row r="73" spans="2:19" x14ac:dyDescent="0.3">
       <c r="B73" s="33">
         <f t="shared" si="1"/>
         <v>56</v>
       </c>
-      <c r="C73" s="116" t="s">
+      <c r="C73" s="112" t="s">
         <v>211</v>
       </c>
-      <c r="D73" s="117" t="s">
+      <c r="D73" s="113" t="s">
         <v>20</v>
       </c>
       <c r="E73" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="F73" s="115" t="s">
+      <c r="F73" s="111" t="s">
         <v>240</v>
       </c>
-      <c r="G73" s="116" t="s">
+      <c r="G73" s="112" t="s">
         <v>213</v>
       </c>
     </row>
@@ -6048,7 +6058,7 @@
         <v>58</v>
       </c>
       <c r="C75" s="3" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="D75" s="101" t="s">
         <v>46</v>
@@ -6132,7 +6142,7 @@
         <v>62</v>
       </c>
       <c r="C79" s="93" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="D79" s="94" t="s">
         <v>21</v>
@@ -6153,7 +6163,7 @@
         <v>63</v>
       </c>
       <c r="C80" s="93" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="D80" s="92">
         <v>1</v>
@@ -6174,19 +6184,19 @@
         <v>64</v>
       </c>
       <c r="C81" s="3" t="s">
-        <v>351</v>
+        <v>346</v>
       </c>
       <c r="D81" s="90" t="s">
         <v>21</v>
       </c>
       <c r="E81" s="1" t="s">
-        <v>352</v>
+        <v>347</v>
       </c>
       <c r="F81" s="2" t="s">
         <v>35</v>
       </c>
       <c r="G81" s="5" t="s">
-        <v>353</v>
+        <v>348</v>
       </c>
     </row>
     <row r="82" spans="2:7" ht="66" x14ac:dyDescent="0.3">
@@ -6197,14 +6207,14 @@
       <c r="C82" s="104" t="s">
         <v>262</v>
       </c>
-      <c r="D82" s="113" t="s">
+      <c r="D82" s="109" t="s">
         <v>20</v>
       </c>
       <c r="E82" s="105" t="s">
         <v>244</v>
       </c>
-      <c r="F82" s="114" t="s">
-        <v>365</v>
+      <c r="F82" s="110" t="s">
+        <v>360</v>
       </c>
       <c r="G82" s="107" t="s">
         <v>265</v>
@@ -6216,7 +6226,7 @@
         <v>66</v>
       </c>
       <c r="C83" s="3" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="D83" s="1">
         <v>1</v>
@@ -6225,10 +6235,10 @@
         <v>244</v>
       </c>
       <c r="F83" s="103" t="s">
-        <v>340</v>
+        <v>352</v>
       </c>
       <c r="G83" s="5" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
     </row>
     <row r="84" spans="2:7" ht="33" x14ac:dyDescent="0.3">
@@ -6237,7 +6247,7 @@
         <v>67</v>
       </c>
       <c r="C84" s="3" t="s">
-        <v>339</v>
+        <v>363</v>
       </c>
       <c r="D84" s="1">
         <v>1</v>
@@ -6246,10 +6256,10 @@
         <v>244</v>
       </c>
       <c r="F84" s="103" t="s">
-        <v>340</v>
+        <v>364</v>
       </c>
       <c r="G84" s="5" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
     </row>
     <row r="85" spans="2:7" ht="33" x14ac:dyDescent="0.3">
@@ -6258,7 +6268,7 @@
         <v>68</v>
       </c>
       <c r="C85" s="3" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="D85" s="90" t="s">
         <v>56</v>
@@ -6267,19 +6277,19 @@
         <v>244</v>
       </c>
       <c r="F85" s="103" t="s">
-        <v>340</v>
+        <v>352</v>
       </c>
       <c r="G85" s="5" t="s">
-        <v>323</v>
-      </c>
-    </row>
-    <row r="86" spans="2:7" ht="33" x14ac:dyDescent="0.3">
+        <v>322</v>
+      </c>
+    </row>
+    <row r="86" spans="2:7" ht="49.5" x14ac:dyDescent="0.3">
       <c r="B86" s="33">
         <f t="shared" si="2"/>
         <v>69</v>
       </c>
       <c r="C86" s="3" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="D86" s="90" t="s">
         <v>56</v>
@@ -6288,10 +6298,10 @@
         <v>244</v>
       </c>
       <c r="F86" s="103" t="s">
-        <v>340</v>
+        <v>366</v>
       </c>
       <c r="G86" s="5" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
     </row>
     <row r="87" spans="2:7" x14ac:dyDescent="0.3">
@@ -6321,7 +6331,7 @@
         <v>71</v>
       </c>
       <c r="C88" s="3" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="D88" s="1">
         <v>1</v>
@@ -6333,7 +6343,7 @@
         <v>245</v>
       </c>
       <c r="G88" s="5" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
     </row>
     <row r="89" spans="2:7" ht="33" x14ac:dyDescent="0.3">
@@ -6362,20 +6372,20 @@
         <f t="shared" si="2"/>
         <v>73</v>
       </c>
-      <c r="C90" s="109" t="s">
+      <c r="C90" s="143" t="s">
+        <v>266</v>
+      </c>
+      <c r="D90" s="144" t="s">
+        <v>20</v>
+      </c>
+      <c r="E90" s="145" t="s">
+        <v>244</v>
+      </c>
+      <c r="F90" s="146" t="s">
+        <v>374</v>
+      </c>
+      <c r="G90" s="143" t="s">
         <v>267</v>
-      </c>
-      <c r="D90" s="110" t="s">
-        <v>20</v>
-      </c>
-      <c r="E90" s="111" t="s">
-        <v>244</v>
-      </c>
-      <c r="F90" s="112" t="s">
-        <v>17</v>
-      </c>
-      <c r="G90" s="109" t="s">
-        <v>268</v>
       </c>
     </row>
     <row r="91" spans="2:7" x14ac:dyDescent="0.3">
@@ -6384,28 +6394,28 @@
         <v>74</v>
       </c>
       <c r="C91" s="3" t="s">
-        <v>348</v>
+        <v>344</v>
       </c>
       <c r="D91" s="90" t="s">
         <v>56</v>
       </c>
       <c r="E91" s="1" t="s">
-        <v>349</v>
+        <v>353</v>
       </c>
       <c r="F91" s="2" t="s">
-        <v>347</v>
+        <v>351</v>
       </c>
       <c r="G91" s="5" t="s">
-        <v>350</v>
-      </c>
-    </row>
-    <row r="92" spans="2:7" x14ac:dyDescent="0.3">
+        <v>345</v>
+      </c>
+    </row>
+    <row r="92" spans="2:7" ht="33" x14ac:dyDescent="0.3">
       <c r="B92" s="33">
         <f t="shared" si="2"/>
         <v>75</v>
       </c>
       <c r="C92" s="3" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="D92" s="90" t="s">
         <v>20</v>
@@ -6414,10 +6424,10 @@
         <v>245</v>
       </c>
       <c r="F92" s="103" t="s">
-        <v>82</v>
+        <v>376</v>
       </c>
       <c r="G92" s="5" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
     </row>
     <row r="93" spans="2:7" x14ac:dyDescent="0.3">
@@ -6426,7 +6436,7 @@
         <v>76</v>
       </c>
       <c r="C93" s="3" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="D93" s="1">
         <v>1</v>
@@ -6438,7 +6448,7 @@
         <v>64</v>
       </c>
       <c r="G93" s="5" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
     </row>
     <row r="94" spans="2:7" x14ac:dyDescent="0.3">
@@ -6447,7 +6457,7 @@
         <v>77</v>
       </c>
       <c r="C94" s="3" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="D94" s="90" t="s">
         <v>56</v>
@@ -6459,7 +6469,7 @@
         <v>64</v>
       </c>
       <c r="G94" s="5" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
     </row>
     <row r="95" spans="2:7" ht="33" x14ac:dyDescent="0.3">
@@ -6468,7 +6478,7 @@
         <v>78</v>
       </c>
       <c r="C95" s="3" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="D95" s="90" t="s">
         <v>56</v>
@@ -6480,7 +6490,7 @@
         <v>63</v>
       </c>
       <c r="G95" s="5" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
     </row>
     <row r="96" spans="2:7" x14ac:dyDescent="0.3">
@@ -6489,7 +6499,7 @@
         <v>79</v>
       </c>
       <c r="C96" s="3" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="D96" s="1">
         <v>1</v>
@@ -6501,7 +6511,7 @@
         <v>82</v>
       </c>
       <c r="G96" s="5" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
     </row>
     <row r="97" spans="2:7" x14ac:dyDescent="0.3">
@@ -6510,7 +6520,7 @@
         <v>80</v>
       </c>
       <c r="C97" s="3" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="D97" s="90" t="s">
         <v>20</v>
@@ -6522,16 +6532,16 @@
         <v>62</v>
       </c>
       <c r="G97" s="5" t="s">
-        <v>299</v>
-      </c>
-    </row>
-    <row r="98" spans="2:7" x14ac:dyDescent="0.3">
+        <v>298</v>
+      </c>
+    </row>
+    <row r="98" spans="2:7" ht="33" x14ac:dyDescent="0.3">
       <c r="B98" s="33">
         <f t="shared" si="2"/>
         <v>81</v>
       </c>
       <c r="C98" s="3" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="D98" s="90" t="s">
         <v>56</v>
@@ -6540,19 +6550,19 @@
         <v>64</v>
       </c>
       <c r="F98" s="103" t="s">
-        <v>62</v>
+        <v>367</v>
       </c>
       <c r="G98" s="5" t="s">
-        <v>333</v>
-      </c>
-    </row>
-    <row r="99" spans="2:7" x14ac:dyDescent="0.3">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="99" spans="2:7" ht="33" x14ac:dyDescent="0.3">
       <c r="B99" s="33">
         <f t="shared" si="2"/>
         <v>82</v>
       </c>
       <c r="C99" s="3" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="D99" s="1">
         <v>1</v>
@@ -6560,23 +6570,53 @@
       <c r="E99" s="2" t="s">
         <v>245</v>
       </c>
-      <c r="F99" s="2" t="s">
-        <v>62</v>
+      <c r="F99" s="103" t="s">
+        <v>367</v>
       </c>
       <c r="G99" s="5" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
     </row>
     <row r="100" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B100" s="33" t="str">
-        <f t="shared" si="2"/>
-        <v/>
+      <c r="B100" s="33">
+        <f t="shared" si="2"/>
+        <v>83</v>
+      </c>
+      <c r="C100" s="3" t="s">
+        <v>368</v>
+      </c>
+      <c r="D100" s="33">
+        <v>1</v>
+      </c>
+      <c r="E100" s="1" t="s">
+        <v>369</v>
+      </c>
+      <c r="F100" s="2" t="s">
+        <v>374</v>
+      </c>
+      <c r="G100" s="5" t="s">
+        <v>365</v>
       </c>
     </row>
     <row r="101" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B101" s="33" t="str">
-        <f t="shared" si="2"/>
-        <v/>
+      <c r="B101" s="33">
+        <f t="shared" si="2"/>
+        <v>84</v>
+      </c>
+      <c r="C101" s="104" t="s">
+        <v>373</v>
+      </c>
+      <c r="D101" s="109" t="s">
+        <v>20</v>
+      </c>
+      <c r="E101" s="142" t="s">
+        <v>374</v>
+      </c>
+      <c r="F101" s="106" t="s">
+        <v>17</v>
+      </c>
+      <c r="G101" s="107" t="s">
+        <v>375</v>
       </c>
     </row>
     <row r="102" spans="2:7" x14ac:dyDescent="0.3">
@@ -6820,39 +6860,51 @@
     </sortState>
   </autoFilter>
   <mergeCells count="102">
-    <mergeCell ref="K2:M2"/>
-    <mergeCell ref="I18:J18"/>
-    <mergeCell ref="K18:M18"/>
-    <mergeCell ref="I21:J21"/>
-    <mergeCell ref="K21:M21"/>
-    <mergeCell ref="J22:L22"/>
-    <mergeCell ref="I3:J3"/>
-    <mergeCell ref="K3:M3"/>
-    <mergeCell ref="B2:G2"/>
-    <mergeCell ref="J6:L6"/>
-    <mergeCell ref="J7:L7"/>
-    <mergeCell ref="I5:J5"/>
-    <mergeCell ref="K5:M5"/>
-    <mergeCell ref="I2:J2"/>
-    <mergeCell ref="J23:L23"/>
-    <mergeCell ref="I12:J12"/>
-    <mergeCell ref="K12:M12"/>
-    <mergeCell ref="I4:J4"/>
-    <mergeCell ref="K4:M4"/>
-    <mergeCell ref="I20:J20"/>
-    <mergeCell ref="K20:M20"/>
-    <mergeCell ref="I19:J19"/>
-    <mergeCell ref="K19:M19"/>
-    <mergeCell ref="I41:J41"/>
-    <mergeCell ref="K41:M41"/>
-    <mergeCell ref="J42:L42"/>
-    <mergeCell ref="J43:L43"/>
-    <mergeCell ref="I32:J32"/>
-    <mergeCell ref="K32:M32"/>
-    <mergeCell ref="I38:J38"/>
-    <mergeCell ref="K38:M38"/>
-    <mergeCell ref="I39:J39"/>
-    <mergeCell ref="K39:M39"/>
+    <mergeCell ref="P24:R24"/>
+    <mergeCell ref="O38:P38"/>
+    <mergeCell ref="Q38:S38"/>
+    <mergeCell ref="P44:R44"/>
+    <mergeCell ref="O56:P56"/>
+    <mergeCell ref="Q56:S56"/>
+    <mergeCell ref="P62:R62"/>
+    <mergeCell ref="P63:R63"/>
+    <mergeCell ref="P64:R64"/>
+    <mergeCell ref="O72:P72"/>
+    <mergeCell ref="Q72:S72"/>
+    <mergeCell ref="P8:R8"/>
+    <mergeCell ref="O59:P59"/>
+    <mergeCell ref="Q59:S59"/>
+    <mergeCell ref="O60:P60"/>
+    <mergeCell ref="Q60:S60"/>
+    <mergeCell ref="O61:P61"/>
+    <mergeCell ref="Q61:S61"/>
+    <mergeCell ref="P42:R42"/>
+    <mergeCell ref="P43:R43"/>
+    <mergeCell ref="O58:P58"/>
+    <mergeCell ref="Q58:S58"/>
+    <mergeCell ref="O39:P39"/>
+    <mergeCell ref="Q39:S39"/>
+    <mergeCell ref="O40:P40"/>
+    <mergeCell ref="Q40:S40"/>
+    <mergeCell ref="O41:P41"/>
+    <mergeCell ref="Q41:S41"/>
+    <mergeCell ref="P22:R22"/>
+    <mergeCell ref="P23:R23"/>
+    <mergeCell ref="O36:P36"/>
+    <mergeCell ref="Q36:S36"/>
+    <mergeCell ref="O19:P19"/>
+    <mergeCell ref="Q19:S19"/>
+    <mergeCell ref="O20:P20"/>
+    <mergeCell ref="Q20:S20"/>
+    <mergeCell ref="O21:P21"/>
+    <mergeCell ref="Q21:S21"/>
+    <mergeCell ref="Q5:S5"/>
+    <mergeCell ref="P6:R6"/>
+    <mergeCell ref="P7:R7"/>
+    <mergeCell ref="O16:P16"/>
+    <mergeCell ref="Q16:S16"/>
+    <mergeCell ref="O18:P18"/>
+    <mergeCell ref="Q18:S18"/>
     <mergeCell ref="I72:J72"/>
     <mergeCell ref="K72:M72"/>
     <mergeCell ref="J57:L57"/>
@@ -6877,51 +6929,39 @@
     <mergeCell ref="K52:M52"/>
     <mergeCell ref="I40:J40"/>
     <mergeCell ref="K40:M40"/>
-    <mergeCell ref="Q19:S19"/>
-    <mergeCell ref="O20:P20"/>
-    <mergeCell ref="Q20:S20"/>
-    <mergeCell ref="O21:P21"/>
-    <mergeCell ref="Q21:S21"/>
-    <mergeCell ref="Q5:S5"/>
-    <mergeCell ref="P6:R6"/>
-    <mergeCell ref="P7:R7"/>
-    <mergeCell ref="O16:P16"/>
-    <mergeCell ref="Q16:S16"/>
-    <mergeCell ref="O18:P18"/>
-    <mergeCell ref="Q18:S18"/>
-    <mergeCell ref="O72:P72"/>
-    <mergeCell ref="Q72:S72"/>
-    <mergeCell ref="P8:R8"/>
-    <mergeCell ref="O59:P59"/>
-    <mergeCell ref="Q59:S59"/>
-    <mergeCell ref="O60:P60"/>
-    <mergeCell ref="Q60:S60"/>
-    <mergeCell ref="O61:P61"/>
-    <mergeCell ref="Q61:S61"/>
-    <mergeCell ref="P42:R42"/>
-    <mergeCell ref="P43:R43"/>
-    <mergeCell ref="O58:P58"/>
-    <mergeCell ref="Q58:S58"/>
-    <mergeCell ref="O39:P39"/>
-    <mergeCell ref="Q39:S39"/>
-    <mergeCell ref="O40:P40"/>
-    <mergeCell ref="Q40:S40"/>
-    <mergeCell ref="O41:P41"/>
-    <mergeCell ref="Q41:S41"/>
-    <mergeCell ref="P22:R22"/>
-    <mergeCell ref="P23:R23"/>
-    <mergeCell ref="O36:P36"/>
-    <mergeCell ref="Q36:S36"/>
-    <mergeCell ref="O19:P19"/>
-    <mergeCell ref="P24:R24"/>
-    <mergeCell ref="O38:P38"/>
-    <mergeCell ref="Q38:S38"/>
-    <mergeCell ref="P44:R44"/>
-    <mergeCell ref="O56:P56"/>
-    <mergeCell ref="Q56:S56"/>
-    <mergeCell ref="P62:R62"/>
-    <mergeCell ref="P63:R63"/>
-    <mergeCell ref="P64:R64"/>
+    <mergeCell ref="I41:J41"/>
+    <mergeCell ref="K41:M41"/>
+    <mergeCell ref="J42:L42"/>
+    <mergeCell ref="J43:L43"/>
+    <mergeCell ref="I32:J32"/>
+    <mergeCell ref="K32:M32"/>
+    <mergeCell ref="I38:J38"/>
+    <mergeCell ref="K38:M38"/>
+    <mergeCell ref="I39:J39"/>
+    <mergeCell ref="K39:M39"/>
+    <mergeCell ref="J23:L23"/>
+    <mergeCell ref="I12:J12"/>
+    <mergeCell ref="K12:M12"/>
+    <mergeCell ref="I4:J4"/>
+    <mergeCell ref="K4:M4"/>
+    <mergeCell ref="I20:J20"/>
+    <mergeCell ref="K20:M20"/>
+    <mergeCell ref="I19:J19"/>
+    <mergeCell ref="K19:M19"/>
+    <mergeCell ref="K2:M2"/>
+    <mergeCell ref="I18:J18"/>
+    <mergeCell ref="K18:M18"/>
+    <mergeCell ref="I21:J21"/>
+    <mergeCell ref="K21:M21"/>
+    <mergeCell ref="J22:L22"/>
+    <mergeCell ref="I3:J3"/>
+    <mergeCell ref="K3:M3"/>
+    <mergeCell ref="B2:G2"/>
+    <mergeCell ref="J6:L6"/>
+    <mergeCell ref="J7:L7"/>
+    <mergeCell ref="I5:J5"/>
+    <mergeCell ref="K5:M5"/>
+    <mergeCell ref="I2:J2"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -6943,25 +6983,25 @@
   <sheetData>
     <row r="2" spans="2:8" ht="49.5" x14ac:dyDescent="0.3">
       <c r="B2" s="1" t="s">
+        <v>333</v>
+      </c>
+      <c r="C2" s="1" t="s">
         <v>334</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="D2" s="1" t="s">
         <v>335</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="E2" s="1" t="s">
         <v>336</v>
       </c>
-      <c r="E2" s="1" t="s">
+      <c r="F2" s="1" t="s">
         <v>337</v>
       </c>
-      <c r="F2" s="1" t="s">
+      <c r="G2" s="102" t="s">
         <v>338</v>
       </c>
-      <c r="G2" s="102" t="s">
-        <v>341</v>
-      </c>
       <c r="H2" s="102" t="s">
-        <v>342</v>
+        <v>339</v>
       </c>
     </row>
     <row r="3" spans="2:8" x14ac:dyDescent="0.3">
@@ -6977,7 +7017,6 @@
         <f>MID(B3,C3,D3-C3)</f>
         <v>#VALUE!</v>
       </c>
-      <c r="F3" s="146"/>
       <c r="G3" s="1">
         <f>COUNTIF($E$3:$E$100,F3)</f>
         <v>0</v>
@@ -7000,7 +7039,6 @@
         <f t="shared" ref="E4:E67" si="2">MID(B4,C4,D4-C4)</f>
         <v>#VALUE!</v>
       </c>
-      <c r="F4" s="146"/>
       <c r="G4" s="1">
         <f t="shared" ref="G4:G67" si="3">COUNTIF($E$3:$E$100,F4)</f>
         <v>0</v>
@@ -7023,7 +7061,6 @@
         <f t="shared" si="2"/>
         <v>#VALUE!</v>
       </c>
-      <c r="F5" s="146"/>
       <c r="G5" s="1">
         <f t="shared" si="3"/>
         <v>0</v>
@@ -7046,7 +7083,6 @@
         <f t="shared" si="2"/>
         <v>#VALUE!</v>
       </c>
-      <c r="F6" s="146"/>
       <c r="G6" s="1">
         <f t="shared" si="3"/>
         <v>0</v>
@@ -7069,7 +7105,6 @@
         <f t="shared" si="2"/>
         <v>#VALUE!</v>
       </c>
-      <c r="F7" s="146"/>
       <c r="G7" s="1">
         <f t="shared" si="3"/>
         <v>0</v>
@@ -7092,7 +7127,6 @@
         <f t="shared" si="2"/>
         <v>#VALUE!</v>
       </c>
-      <c r="F8" s="146"/>
       <c r="G8" s="1">
         <f t="shared" si="3"/>
         <v>0</v>
@@ -7115,7 +7149,6 @@
         <f t="shared" si="2"/>
         <v>#VALUE!</v>
       </c>
-      <c r="F9" s="146"/>
       <c r="G9" s="1">
         <f t="shared" si="3"/>
         <v>0</v>
@@ -7138,7 +7171,6 @@
         <f t="shared" si="2"/>
         <v>#VALUE!</v>
       </c>
-      <c r="F10" s="146"/>
       <c r="G10" s="1">
         <f t="shared" si="3"/>
         <v>0</v>
@@ -7161,7 +7193,6 @@
         <f t="shared" si="2"/>
         <v>#VALUE!</v>
       </c>
-      <c r="F11" s="146"/>
       <c r="G11" s="1">
         <f t="shared" si="3"/>
         <v>0</v>
@@ -7184,7 +7215,6 @@
         <f t="shared" si="2"/>
         <v>#VALUE!</v>
       </c>
-      <c r="F12" s="146"/>
       <c r="G12" s="1">
         <f t="shared" si="3"/>
         <v>0</v>
@@ -7207,7 +7237,6 @@
         <f t="shared" si="2"/>
         <v>#VALUE!</v>
       </c>
-      <c r="F13" s="146"/>
       <c r="G13" s="1">
         <f t="shared" si="3"/>
         <v>0</v>
@@ -7230,7 +7259,6 @@
         <f t="shared" si="2"/>
         <v>#VALUE!</v>
       </c>
-      <c r="F14" s="146"/>
       <c r="G14" s="1">
         <f t="shared" si="3"/>
         <v>0</v>
@@ -7253,7 +7281,6 @@
         <f t="shared" si="2"/>
         <v>#VALUE!</v>
       </c>
-      <c r="F15" s="146"/>
       <c r="G15" s="1">
         <f t="shared" si="3"/>
         <v>0</v>
@@ -7276,7 +7303,6 @@
         <f t="shared" si="2"/>
         <v>#VALUE!</v>
       </c>
-      <c r="F16" s="146"/>
       <c r="G16" s="1">
         <f t="shared" si="3"/>
         <v>0</v>
@@ -7299,7 +7325,6 @@
         <f t="shared" si="2"/>
         <v>#VALUE!</v>
       </c>
-      <c r="F17" s="146"/>
       <c r="G17" s="1">
         <f t="shared" si="3"/>
         <v>0</v>
@@ -7322,7 +7347,6 @@
         <f t="shared" si="2"/>
         <v>#VALUE!</v>
       </c>
-      <c r="F18" s="146"/>
       <c r="G18" s="1">
         <f t="shared" si="3"/>
         <v>0</v>
@@ -7345,7 +7369,6 @@
         <f t="shared" si="2"/>
         <v>#VALUE!</v>
       </c>
-      <c r="F19" s="146"/>
       <c r="G19" s="1">
         <f t="shared" si="3"/>
         <v>0</v>
@@ -7368,7 +7391,6 @@
         <f t="shared" si="2"/>
         <v>#VALUE!</v>
       </c>
-      <c r="F20" s="146"/>
       <c r="G20" s="1">
         <f t="shared" si="3"/>
         <v>0</v>
@@ -7391,7 +7413,6 @@
         <f t="shared" si="2"/>
         <v>#VALUE!</v>
       </c>
-      <c r="F21" s="146"/>
       <c r="G21" s="1">
         <f t="shared" si="3"/>
         <v>0</v>
@@ -7414,7 +7435,7 @@
         <f t="shared" si="2"/>
         <v>#VALUE!</v>
       </c>
-      <c r="F22" s="147"/>
+      <c r="F22" s="33"/>
       <c r="G22" s="1">
         <f t="shared" si="3"/>
         <v>0</v>
@@ -7437,7 +7458,6 @@
         <f t="shared" si="2"/>
         <v>#VALUE!</v>
       </c>
-      <c r="F23" s="146"/>
       <c r="G23" s="1">
         <f t="shared" si="3"/>
         <v>0</v>
@@ -7460,7 +7480,6 @@
         <f t="shared" si="2"/>
         <v>#VALUE!</v>
       </c>
-      <c r="F24" s="146"/>
       <c r="G24" s="1">
         <f t="shared" si="3"/>
         <v>0</v>
@@ -7483,7 +7502,6 @@
         <f t="shared" si="2"/>
         <v>#VALUE!</v>
       </c>
-      <c r="F25" s="146"/>
       <c r="G25" s="1">
         <f t="shared" si="3"/>
         <v>0</v>
@@ -7506,7 +7524,6 @@
         <f t="shared" si="2"/>
         <v>#VALUE!</v>
       </c>
-      <c r="F26" s="146"/>
       <c r="G26" s="1">
         <f t="shared" si="3"/>
         <v>0</v>
@@ -7529,7 +7546,6 @@
         <f t="shared" si="2"/>
         <v>#VALUE!</v>
       </c>
-      <c r="F27" s="146"/>
       <c r="G27" s="1">
         <f t="shared" si="3"/>
         <v>0</v>
@@ -7552,7 +7568,7 @@
         <f t="shared" si="2"/>
         <v>#VALUE!</v>
       </c>
-      <c r="F28" s="148"/>
+      <c r="F28" s="111"/>
       <c r="G28" s="1">
         <f t="shared" si="3"/>
         <v>0</v>
@@ -7575,7 +7591,6 @@
         <f t="shared" si="2"/>
         <v>#VALUE!</v>
       </c>
-      <c r="F29" s="146"/>
       <c r="G29" s="1">
         <f t="shared" si="3"/>
         <v>0</v>
@@ -7598,7 +7613,6 @@
         <f t="shared" si="2"/>
         <v>#VALUE!</v>
       </c>
-      <c r="F30" s="146"/>
       <c r="G30" s="1">
         <f t="shared" si="3"/>
         <v>0</v>
@@ -7621,7 +7635,6 @@
         <f t="shared" si="2"/>
         <v>#VALUE!</v>
       </c>
-      <c r="F31" s="146"/>
       <c r="G31" s="1">
         <f t="shared" si="3"/>
         <v>0</v>
@@ -7644,7 +7657,6 @@
         <f t="shared" si="2"/>
         <v>#VALUE!</v>
       </c>
-      <c r="F32" s="146"/>
       <c r="G32" s="1">
         <f t="shared" si="3"/>
         <v>0</v>
@@ -7667,7 +7679,6 @@
         <f t="shared" si="2"/>
         <v>#VALUE!</v>
       </c>
-      <c r="F33" s="146"/>
       <c r="G33" s="1">
         <f t="shared" si="3"/>
         <v>0</v>
@@ -7690,7 +7701,6 @@
         <f t="shared" si="2"/>
         <v>#VALUE!</v>
       </c>
-      <c r="F34" s="146"/>
       <c r="G34" s="1">
         <f t="shared" si="3"/>
         <v>0</v>
@@ -7713,7 +7723,6 @@
         <f t="shared" si="2"/>
         <v>#VALUE!</v>
       </c>
-      <c r="F35" s="146"/>
       <c r="G35" s="1">
         <f t="shared" si="3"/>
         <v>0</v>
@@ -7736,7 +7745,6 @@
         <f t="shared" si="2"/>
         <v>#VALUE!</v>
       </c>
-      <c r="F36" s="146"/>
       <c r="G36" s="1">
         <f t="shared" si="3"/>
         <v>0</v>
@@ -7759,7 +7767,6 @@
         <f t="shared" si="2"/>
         <v>#VALUE!</v>
       </c>
-      <c r="F37" s="146"/>
       <c r="G37" s="1">
         <f t="shared" si="3"/>
         <v>0</v>
@@ -7782,7 +7789,6 @@
         <f t="shared" si="2"/>
         <v>#VALUE!</v>
       </c>
-      <c r="F38" s="146"/>
       <c r="G38" s="1">
         <f t="shared" si="3"/>
         <v>0</v>
@@ -7805,7 +7811,6 @@
         <f t="shared" si="2"/>
         <v>#VALUE!</v>
       </c>
-      <c r="F39" s="146"/>
       <c r="G39" s="1">
         <f t="shared" si="3"/>
         <v>0</v>
@@ -7828,7 +7833,6 @@
         <f t="shared" si="2"/>
         <v>#VALUE!</v>
       </c>
-      <c r="F40" s="146"/>
       <c r="G40" s="1">
         <f t="shared" si="3"/>
         <v>0</v>
@@ -7851,7 +7855,6 @@
         <f t="shared" si="2"/>
         <v>#VALUE!</v>
       </c>
-      <c r="F41" s="146"/>
       <c r="G41" s="1">
         <f t="shared" si="3"/>
         <v>0</v>
@@ -7874,7 +7877,7 @@
         <f t="shared" si="2"/>
         <v>#VALUE!</v>
       </c>
-      <c r="F42" s="147"/>
+      <c r="F42" s="33"/>
       <c r="G42" s="1">
         <f t="shared" si="3"/>
         <v>0</v>
@@ -7897,7 +7900,6 @@
         <f t="shared" si="2"/>
         <v>#VALUE!</v>
       </c>
-      <c r="F43" s="146"/>
       <c r="G43" s="1">
         <f t="shared" si="3"/>
         <v>0</v>
@@ -7920,7 +7922,6 @@
         <f t="shared" si="2"/>
         <v>#VALUE!</v>
       </c>
-      <c r="F44" s="146"/>
       <c r="G44" s="1">
         <f t="shared" si="3"/>
         <v>0</v>
@@ -7943,7 +7944,6 @@
         <f t="shared" si="2"/>
         <v>#VALUE!</v>
       </c>
-      <c r="F45" s="146"/>
       <c r="G45" s="1">
         <f t="shared" si="3"/>
         <v>0</v>
@@ -7966,7 +7966,6 @@
         <f t="shared" si="2"/>
         <v>#VALUE!</v>
       </c>
-      <c r="F46" s="146"/>
       <c r="G46" s="1">
         <f t="shared" si="3"/>
         <v>0</v>
@@ -7989,7 +7988,6 @@
         <f t="shared" si="2"/>
         <v>#VALUE!</v>
       </c>
-      <c r="F47" s="146"/>
       <c r="G47" s="1">
         <f t="shared" si="3"/>
         <v>0</v>
@@ -8012,7 +8010,6 @@
         <f t="shared" si="2"/>
         <v>#VALUE!</v>
       </c>
-      <c r="F48" s="146"/>
       <c r="G48" s="1">
         <f t="shared" si="3"/>
         <v>0</v>
@@ -8035,7 +8032,6 @@
         <f t="shared" si="2"/>
         <v>#VALUE!</v>
       </c>
-      <c r="F49" s="146"/>
       <c r="G49" s="1">
         <f t="shared" si="3"/>
         <v>0</v>
@@ -8058,7 +8054,6 @@
         <f t="shared" si="2"/>
         <v>#VALUE!</v>
       </c>
-      <c r="F50" s="146"/>
       <c r="G50" s="1">
         <f t="shared" si="3"/>
         <v>0</v>
@@ -8081,7 +8076,6 @@
         <f t="shared" si="2"/>
         <v>#VALUE!</v>
       </c>
-      <c r="F51" s="146"/>
       <c r="G51" s="1">
         <f t="shared" si="3"/>
         <v>0</v>
@@ -8104,7 +8098,6 @@
         <f t="shared" si="2"/>
         <v>#VALUE!</v>
       </c>
-      <c r="F52" s="146"/>
       <c r="G52" s="1">
         <f t="shared" si="3"/>
         <v>0</v>
@@ -8127,7 +8120,7 @@
         <f t="shared" si="2"/>
         <v>#VALUE!</v>
       </c>
-      <c r="F53" s="148"/>
+      <c r="F53" s="111"/>
       <c r="G53" s="1">
         <f t="shared" si="3"/>
         <v>0</v>
@@ -8150,7 +8143,6 @@
         <f t="shared" si="2"/>
         <v>#VALUE!</v>
       </c>
-      <c r="F54" s="146"/>
       <c r="G54" s="1">
         <f t="shared" si="3"/>
         <v>0</v>
@@ -8173,7 +8165,6 @@
         <f t="shared" si="2"/>
         <v>#VALUE!</v>
       </c>
-      <c r="F55" s="146"/>
       <c r="G55" s="1">
         <f t="shared" si="3"/>
         <v>0</v>
@@ -8196,7 +8187,6 @@
         <f t="shared" si="2"/>
         <v>#VALUE!</v>
       </c>
-      <c r="F56" s="146"/>
       <c r="G56" s="1">
         <f t="shared" si="3"/>
         <v>0</v>
@@ -8219,7 +8209,6 @@
         <f t="shared" si="2"/>
         <v>#VALUE!</v>
       </c>
-      <c r="F57" s="146"/>
       <c r="G57" s="1">
         <f t="shared" si="3"/>
         <v>0</v>
@@ -8242,7 +8231,7 @@
         <f t="shared" si="2"/>
         <v>#VALUE!</v>
       </c>
-      <c r="F58" s="147"/>
+      <c r="F58" s="33"/>
       <c r="G58" s="1">
         <f t="shared" si="3"/>
         <v>0</v>
@@ -8265,7 +8254,7 @@
         <f t="shared" si="2"/>
         <v>#VALUE!</v>
       </c>
-      <c r="F59" s="147"/>
+      <c r="F59" s="33"/>
       <c r="G59" s="1">
         <f t="shared" si="3"/>
         <v>0</v>
@@ -8288,7 +8277,7 @@
         <f t="shared" si="2"/>
         <v>#VALUE!</v>
       </c>
-      <c r="F60" s="147"/>
+      <c r="F60" s="33"/>
       <c r="G60" s="1">
         <f t="shared" si="3"/>
         <v>0</v>
@@ -8311,7 +8300,6 @@
         <f t="shared" si="2"/>
         <v>#VALUE!</v>
       </c>
-      <c r="F61" s="146"/>
       <c r="G61" s="1">
         <f t="shared" si="3"/>
         <v>0</v>
@@ -8334,7 +8322,6 @@
         <f t="shared" si="2"/>
         <v>#VALUE!</v>
       </c>
-      <c r="F62" s="146"/>
       <c r="G62" s="1">
         <f t="shared" si="3"/>
         <v>0</v>
@@ -8357,7 +8344,6 @@
         <f t="shared" si="2"/>
         <v>#VALUE!</v>
       </c>
-      <c r="F63" s="146"/>
       <c r="G63" s="1">
         <f t="shared" si="3"/>
         <v>0</v>
@@ -8380,7 +8366,6 @@
         <f t="shared" si="2"/>
         <v>#VALUE!</v>
       </c>
-      <c r="F64" s="146"/>
       <c r="G64" s="1">
         <f t="shared" si="3"/>
         <v>0</v>
@@ -8403,7 +8388,6 @@
         <f t="shared" si="2"/>
         <v>#VALUE!</v>
       </c>
-      <c r="F65" s="146"/>
       <c r="G65" s="1">
         <f t="shared" si="3"/>
         <v>0</v>
@@ -8426,7 +8410,6 @@
         <f t="shared" si="2"/>
         <v>#VALUE!</v>
       </c>
-      <c r="F66" s="146"/>
       <c r="G66" s="1">
         <f t="shared" si="3"/>
         <v>0</v>
@@ -8449,7 +8432,6 @@
         <f t="shared" si="2"/>
         <v>#VALUE!</v>
       </c>
-      <c r="F67" s="146"/>
       <c r="G67" s="1">
         <f t="shared" si="3"/>
         <v>0</v>
@@ -8472,7 +8454,7 @@
         <f t="shared" ref="E68:E84" si="7">MID(B68,C68,D68-C68)</f>
         <v>#VALUE!</v>
       </c>
-      <c r="F68" s="148"/>
+      <c r="F68" s="111"/>
       <c r="G68" s="1">
         <f t="shared" ref="G68:G84" si="8">COUNTIF($E$3:$E$100,F68)</f>
         <v>0</v>
@@ -8495,7 +8477,6 @@
         <f t="shared" si="7"/>
         <v>#VALUE!</v>
       </c>
-      <c r="F69" s="146"/>
       <c r="G69" s="1">
         <f t="shared" si="8"/>
         <v>0</v>
@@ -8518,7 +8499,6 @@
         <f t="shared" si="7"/>
         <v>#VALUE!</v>
       </c>
-      <c r="F70" s="146"/>
       <c r="G70" s="1">
         <f t="shared" si="8"/>
         <v>0</v>
@@ -8541,7 +8521,6 @@
         <f t="shared" si="7"/>
         <v>#VALUE!</v>
       </c>
-      <c r="F71" s="146"/>
       <c r="G71" s="1">
         <f t="shared" si="8"/>
         <v>0</v>
@@ -8564,7 +8543,6 @@
         <f t="shared" si="7"/>
         <v>#VALUE!</v>
       </c>
-      <c r="F72" s="146"/>
       <c r="G72" s="1">
         <f t="shared" si="8"/>
         <v>0</v>
@@ -8587,7 +8565,6 @@
         <f t="shared" si="7"/>
         <v>#VALUE!</v>
       </c>
-      <c r="F73" s="146"/>
       <c r="G73" s="1">
         <f t="shared" si="8"/>
         <v>0</v>
@@ -8610,7 +8587,6 @@
         <f t="shared" si="7"/>
         <v>#VALUE!</v>
       </c>
-      <c r="F74" s="146"/>
       <c r="G74" s="1">
         <f t="shared" si="8"/>
         <v>0</v>
@@ -8633,7 +8609,6 @@
         <f t="shared" si="7"/>
         <v>#VALUE!</v>
       </c>
-      <c r="F75" s="146"/>
       <c r="G75" s="1">
         <f t="shared" si="8"/>
         <v>0</v>
@@ -8656,7 +8631,6 @@
         <f t="shared" si="7"/>
         <v>#VALUE!</v>
       </c>
-      <c r="F76" s="146"/>
       <c r="G76" s="1">
         <f t="shared" si="8"/>
         <v>0</v>
@@ -8679,7 +8653,6 @@
         <f t="shared" si="7"/>
         <v>#VALUE!</v>
       </c>
-      <c r="F77" s="146"/>
       <c r="G77" s="1">
         <f t="shared" si="8"/>
         <v>0</v>

</xml_diff>

<commit_message>
IDD Update for 2 Cycle WDATA Hazard
</commit_message>
<xml_diff>
--- a/Document/IDD.xlsx
+++ b/Document/IDD.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="V:\SoC_Design\Document\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{52B9693E-721C-41BD-A898-07F7EED66780}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7B27CCE0-E8C4-4047-BF55-54CB5B588EB6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{813C5046-60F0-40FF-AAC7-48B46C31F73B}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="841" uniqueCount="382">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="859" uniqueCount="396">
   <si>
     <t>top_cpu</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -1431,19 +1431,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>ForwardA MUX Data</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>ForwardB MUX Data</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>u_alu_forward_b_mux
-u_ex_mem_bridge</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>w_mem_regwrite</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -1453,22 +1440,7 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>u_wdata_forwarding_unit</t>
-  </si>
-  <si>
-    <t>w_ex_alu_forward_mux_data_a</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>w_ex_alu_forward_mux_data_b</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>u_alu_src_mux</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>w_mem_wdata_forward_mux_data</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
@@ -1504,11 +1476,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>u_mem_wb_bridge
-u_wdata_forward_unit</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>w_id_regdst</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -1518,42 +1485,6 @@
   </si>
   <si>
     <t>w_wb_regdst</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>w_fw_ctr_alu_1c_forward_a</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>w_fw_ctr_alu_1c_forward_b</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>WDATA Forward Output (1 Cycle)</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>ALU ForwardB Output (1 Cycle)</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>ALU ForwardA Output (1 Cycle)</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>w_fw_ctr_wdata_1c_forward</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>w_fw_ctr_alu_2c_forward_a</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>w_fw_ctr_alu_2c_forward_b</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>ALU ForwardA Output (2 Cycle)</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
@@ -1581,14 +1512,130 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>ALU ForwardB Output (2 Cycle)</t>
+    <t>w_ex_fw_ctr_wdata_2c</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>u_wdata_forwarding_unit</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>w_mem_fw_ctr_wdata_2c</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>w_fw_ctr_alu_a_1c</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>w_fw_ctr_alu_b_1c</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>w_fw_ctr_alu_a_2c</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>w_fw_ctr_alu_b_2c</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>w_fw_ctr_wdata_1c</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>w_mem_wdata_fw_mux_data</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>w_ex_alu_fw_mux_data_a</t>
+  </si>
+  <si>
+    <t>fwA MUX Data</t>
+  </si>
+  <si>
+    <t>w_ex_alu_fw_mux_data_b</t>
+  </si>
+  <si>
+    <t>fwB MUX Data</t>
+  </si>
+  <si>
+    <t>ALU fwA Output (1 Cycle)</t>
+  </si>
+  <si>
+    <t>ALU fwB Output (1 Cycle)</t>
+  </si>
+  <si>
+    <t>ALU fwA Output (2 Cycle)</t>
+  </si>
+  <si>
+    <t>ALU fwB Output (2 Cycle)</t>
+  </si>
+  <si>
+    <t>WDATA fw Output (1 Cycle)</t>
+  </si>
+  <si>
+    <t>WDATA fw Output (2 Cycle) (EX)</t>
+  </si>
+  <si>
+    <t>WDATA fw Output (2 Cycle) (MEM)</t>
+  </si>
+  <si>
+    <t>w_mem_wdata_fw_mux_data_2c</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>u_alu_forwarding_unit</t>
+  </si>
+  <si>
+    <t>u_alu_forward_a_mux</t>
+  </si>
+  <si>
+    <t>u_alu_forward_b_mux</t>
+  </si>
+  <si>
+    <t>u_mem_wb_bridge
+u_wdata_forwarding_unit</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>u_wdata_forward_2cycle_mux</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>u_ex_mem_bridge
+u_wdata_forward_mux</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>u_ex_mem_bridge
+u_wdata_forward_2cycle_mux</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>u_alu_forward_b_mux
+u_ex_mem_bridge
+u_wdata_forward_2cycle_mux</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>u_memtoreg_mux
 u_wdata_forward_mux
+u_wdata_forward_2cycle_mux
 u_alu_forward_a_mux
 u_alu_forward_b_mux</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>w_ex_wdata_fw_mux_data_2c</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>WDATA Forward MUX Data (2 Cylce) (EX)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>WDATA Forward MUX Data (2 Cylce) (MEM)</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -2569,83 +2616,83 @@
     <xf numFmtId="176" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="3" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="26" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="27" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="28" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="26" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="27" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="28" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -3007,32 +3054,32 @@
   <sheetData>
     <row r="1" spans="2:19" ht="17.25" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="2" spans="2:19" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B2" s="141" t="s">
-        <v>0</v>
-      </c>
-      <c r="C2" s="142"/>
-      <c r="D2" s="142"/>
-      <c r="E2" s="142"/>
-      <c r="F2" s="142"/>
-      <c r="G2" s="143"/>
-      <c r="I2" s="120" t="s">
+      <c r="B2" s="132" t="s">
+        <v>0</v>
+      </c>
+      <c r="C2" s="133"/>
+      <c r="D2" s="133"/>
+      <c r="E2" s="133"/>
+      <c r="F2" s="133"/>
+      <c r="G2" s="134"/>
+      <c r="I2" s="118" t="s">
         <v>103</v>
       </c>
-      <c r="J2" s="121"/>
-      <c r="K2" s="120" t="s">
+      <c r="J2" s="120"/>
+      <c r="K2" s="118" t="s">
         <v>97</v>
       </c>
-      <c r="L2" s="122"/>
-      <c r="M2" s="121"/>
-      <c r="O2" s="120" t="s">
+      <c r="L2" s="119"/>
+      <c r="M2" s="120"/>
+      <c r="O2" s="118" t="s">
         <v>103</v>
       </c>
-      <c r="P2" s="121"/>
-      <c r="Q2" s="120" t="s">
+      <c r="P2" s="120"/>
+      <c r="Q2" s="118" t="s">
         <v>150</v>
       </c>
-      <c r="R2" s="122"/>
-      <c r="S2" s="121"/>
+      <c r="R2" s="119"/>
+      <c r="S2" s="120"/>
     </row>
     <row r="3" spans="2:19" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B3" s="34" t="s">
@@ -3053,24 +3100,24 @@
       <c r="G3" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="I3" s="130" t="s">
+      <c r="I3" s="127" t="s">
         <v>109</v>
       </c>
-      <c r="J3" s="131"/>
-      <c r="K3" s="132" t="s">
+      <c r="J3" s="128"/>
+      <c r="K3" s="129" t="s">
         <v>110</v>
       </c>
-      <c r="L3" s="133"/>
-      <c r="M3" s="134"/>
-      <c r="O3" s="130" t="s">
+      <c r="L3" s="130"/>
+      <c r="M3" s="131"/>
+      <c r="O3" s="127" t="s">
         <v>109</v>
       </c>
-      <c r="P3" s="131"/>
-      <c r="Q3" s="132" t="s">
+      <c r="P3" s="128"/>
+      <c r="Q3" s="129" t="s">
         <v>237</v>
       </c>
-      <c r="R3" s="133"/>
-      <c r="S3" s="134"/>
+      <c r="R3" s="130"/>
+      <c r="S3" s="131"/>
     </row>
     <row r="4" spans="2:19" x14ac:dyDescent="0.3">
       <c r="B4" s="35">
@@ -3091,24 +3138,24 @@
       <c r="G4" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="I4" s="130" t="s">
+      <c r="I4" s="127" t="s">
         <v>107</v>
       </c>
-      <c r="J4" s="131"/>
-      <c r="K4" s="130" t="s">
+      <c r="J4" s="128"/>
+      <c r="K4" s="127" t="s">
         <v>64</v>
       </c>
-      <c r="L4" s="135"/>
-      <c r="M4" s="131"/>
-      <c r="O4" s="130" t="s">
+      <c r="L4" s="141"/>
+      <c r="M4" s="128"/>
+      <c r="O4" s="127" t="s">
         <v>107</v>
       </c>
-      <c r="P4" s="131"/>
-      <c r="Q4" s="130" t="s">
+      <c r="P4" s="128"/>
+      <c r="Q4" s="127" t="s">
         <v>64</v>
       </c>
-      <c r="R4" s="135"/>
-      <c r="S4" s="131"/>
+      <c r="R4" s="141"/>
+      <c r="S4" s="128"/>
     </row>
     <row r="5" spans="2:19" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B5" s="54">
@@ -3129,24 +3176,24 @@
       <c r="G5" s="14" t="s">
         <v>9</v>
       </c>
-      <c r="I5" s="136" t="s">
+      <c r="I5" s="121" t="s">
         <v>8</v>
       </c>
-      <c r="J5" s="137"/>
-      <c r="K5" s="138" t="s">
+      <c r="J5" s="122"/>
+      <c r="K5" s="123" t="s">
         <v>102</v>
       </c>
-      <c r="L5" s="119"/>
-      <c r="M5" s="139"/>
-      <c r="O5" s="136" t="s">
+      <c r="L5" s="124"/>
+      <c r="M5" s="125"/>
+      <c r="O5" s="121" t="s">
         <v>8</v>
       </c>
-      <c r="P5" s="137"/>
-      <c r="Q5" s="138" t="s">
+      <c r="P5" s="122"/>
+      <c r="Q5" s="123" t="s">
         <v>151</v>
       </c>
-      <c r="R5" s="119"/>
-      <c r="S5" s="139"/>
+      <c r="R5" s="124"/>
+      <c r="S5" s="125"/>
     </row>
     <row r="6" spans="2:19" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B6" s="55">
@@ -3170,22 +3217,22 @@
       <c r="I6" s="67" t="s">
         <v>41</v>
       </c>
-      <c r="J6" s="128" t="s">
+      <c r="J6" s="126" t="s">
         <v>98</v>
       </c>
-      <c r="K6" s="128"/>
-      <c r="L6" s="128"/>
+      <c r="K6" s="126"/>
+      <c r="L6" s="126"/>
       <c r="M6" s="69" t="s">
         <v>8</v>
       </c>
       <c r="O6" s="67" t="s">
         <v>41</v>
       </c>
-      <c r="P6" s="128" t="s">
+      <c r="P6" s="126" t="s">
         <v>98</v>
       </c>
-      <c r="Q6" s="128"/>
-      <c r="R6" s="128"/>
+      <c r="Q6" s="126"/>
+      <c r="R6" s="126"/>
       <c r="S6" s="69" t="s">
         <v>8</v>
       </c>
@@ -3212,22 +3259,22 @@
       <c r="I7" s="70">
         <v>1</v>
       </c>
-      <c r="J7" s="140" t="s">
+      <c r="J7" s="135" t="s">
         <v>21</v>
       </c>
-      <c r="K7" s="140"/>
-      <c r="L7" s="140"/>
+      <c r="K7" s="135"/>
+      <c r="L7" s="135"/>
       <c r="M7" s="71" t="s">
         <v>133</v>
       </c>
       <c r="O7" s="87">
         <v>1</v>
       </c>
-      <c r="P7" s="129" t="s">
+      <c r="P7" s="142" t="s">
         <v>21</v>
       </c>
-      <c r="Q7" s="129"/>
-      <c r="R7" s="129"/>
+      <c r="Q7" s="142"/>
+      <c r="R7" s="142"/>
       <c r="S7" s="88" t="s">
         <v>133</v>
       </c>
@@ -3269,11 +3316,11 @@
       <c r="O8" s="80">
         <v>2</v>
       </c>
-      <c r="P8" s="119" t="s">
+      <c r="P8" s="124" t="s">
         <v>20</v>
       </c>
-      <c r="Q8" s="119"/>
-      <c r="R8" s="119"/>
+      <c r="Q8" s="124"/>
+      <c r="R8" s="124"/>
       <c r="S8" s="82" t="s">
         <v>134</v>
       </c>
@@ -3447,15 +3494,15 @@
       <c r="G12" s="30" t="s">
         <v>29</v>
       </c>
-      <c r="I12" s="123" t="s">
+      <c r="I12" s="136" t="s">
         <v>105</v>
       </c>
-      <c r="J12" s="124"/>
-      <c r="K12" s="125" t="s">
+      <c r="J12" s="137"/>
+      <c r="K12" s="138" t="s">
         <v>106</v>
       </c>
-      <c r="L12" s="126"/>
-      <c r="M12" s="127"/>
+      <c r="L12" s="139"/>
+      <c r="M12" s="140"/>
       <c r="O12" s="72">
         <v>3</v>
       </c>
@@ -3578,15 +3625,15 @@
       </c>
     </row>
     <row r="16" spans="2:19" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="O16" s="123" t="s">
+      <c r="O16" s="136" t="s">
         <v>105</v>
       </c>
-      <c r="P16" s="124"/>
-      <c r="Q16" s="125" t="s">
+      <c r="P16" s="137"/>
+      <c r="Q16" s="138" t="s">
         <v>240</v>
       </c>
-      <c r="R16" s="126"/>
-      <c r="S16" s="127"/>
+      <c r="R16" s="139"/>
+      <c r="S16" s="140"/>
     </row>
     <row r="17" spans="2:19" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B17" s="90" t="s">
@@ -3628,24 +3675,24 @@
       <c r="G18" s="99" t="s">
         <v>198</v>
       </c>
-      <c r="I18" s="120" t="s">
+      <c r="I18" s="118" t="s">
         <v>103</v>
       </c>
-      <c r="J18" s="121"/>
-      <c r="K18" s="120" t="s">
+      <c r="J18" s="120"/>
+      <c r="K18" s="118" t="s">
         <v>104</v>
       </c>
-      <c r="L18" s="122"/>
-      <c r="M18" s="121"/>
-      <c r="O18" s="120" t="s">
+      <c r="L18" s="119"/>
+      <c r="M18" s="120"/>
+      <c r="O18" s="118" t="s">
         <v>103</v>
       </c>
-      <c r="P18" s="121"/>
-      <c r="Q18" s="120" t="s">
+      <c r="P18" s="120"/>
+      <c r="Q18" s="118" t="s">
         <v>160</v>
       </c>
-      <c r="R18" s="122"/>
-      <c r="S18" s="121"/>
+      <c r="R18" s="119"/>
+      <c r="S18" s="120"/>
     </row>
     <row r="19" spans="2:19" x14ac:dyDescent="0.3">
       <c r="B19" s="33">
@@ -3667,24 +3714,24 @@
       <c r="G19" s="5" t="s">
         <v>84</v>
       </c>
-      <c r="I19" s="130" t="s">
+      <c r="I19" s="127" t="s">
         <v>109</v>
       </c>
-      <c r="J19" s="131"/>
-      <c r="K19" s="132" t="s">
+      <c r="J19" s="128"/>
+      <c r="K19" s="129" t="s">
         <v>111</v>
       </c>
-      <c r="L19" s="133"/>
-      <c r="M19" s="134"/>
-      <c r="O19" s="130" t="s">
+      <c r="L19" s="130"/>
+      <c r="M19" s="131"/>
+      <c r="O19" s="127" t="s">
         <v>109</v>
       </c>
-      <c r="P19" s="131"/>
-      <c r="Q19" s="132" t="s">
+      <c r="P19" s="128"/>
+      <c r="Q19" s="129" t="s">
         <v>237</v>
       </c>
-      <c r="R19" s="133"/>
-      <c r="S19" s="134"/>
+      <c r="R19" s="130"/>
+      <c r="S19" s="131"/>
     </row>
     <row r="20" spans="2:19" ht="33" x14ac:dyDescent="0.3">
       <c r="B20" s="33">
@@ -3706,24 +3753,24 @@
       <c r="G20" s="5" t="s">
         <v>77</v>
       </c>
-      <c r="I20" s="130" t="s">
+      <c r="I20" s="127" t="s">
         <v>107</v>
       </c>
-      <c r="J20" s="131"/>
-      <c r="K20" s="132" t="s">
+      <c r="J20" s="128"/>
+      <c r="K20" s="129" t="s">
         <v>108</v>
       </c>
-      <c r="L20" s="133"/>
-      <c r="M20" s="134"/>
-      <c r="O20" s="130" t="s">
+      <c r="L20" s="130"/>
+      <c r="M20" s="131"/>
+      <c r="O20" s="127" t="s">
         <v>107</v>
       </c>
-      <c r="P20" s="131"/>
-      <c r="Q20" s="130" t="s">
+      <c r="P20" s="128"/>
+      <c r="Q20" s="127" t="s">
         <v>64</v>
       </c>
-      <c r="R20" s="135"/>
-      <c r="S20" s="131"/>
+      <c r="R20" s="141"/>
+      <c r="S20" s="128"/>
     </row>
     <row r="21" spans="2:19" ht="33.75" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B21" s="33">
@@ -3731,38 +3778,38 @@
         <v>4</v>
       </c>
       <c r="C21" s="3" t="s">
-        <v>351</v>
+        <v>372</v>
       </c>
       <c r="D21" s="90" t="s">
         <v>20</v>
       </c>
       <c r="E21" s="1" t="s">
-        <v>375</v>
+        <v>358</v>
       </c>
       <c r="F21" s="103" t="s">
         <v>76</v>
       </c>
       <c r="G21" s="5" t="s">
-        <v>345</v>
-      </c>
-      <c r="I21" s="136" t="s">
+        <v>373</v>
+      </c>
+      <c r="I21" s="121" t="s">
         <v>8</v>
       </c>
-      <c r="J21" s="137"/>
-      <c r="K21" s="138" t="s">
+      <c r="J21" s="122"/>
+      <c r="K21" s="123" t="s">
         <v>125</v>
       </c>
-      <c r="L21" s="119"/>
-      <c r="M21" s="139"/>
-      <c r="O21" s="136" t="s">
+      <c r="L21" s="124"/>
+      <c r="M21" s="125"/>
+      <c r="O21" s="121" t="s">
         <v>8</v>
       </c>
-      <c r="P21" s="137"/>
-      <c r="Q21" s="138" t="s">
+      <c r="P21" s="122"/>
+      <c r="Q21" s="123" t="s">
         <v>161</v>
       </c>
-      <c r="R21" s="119"/>
-      <c r="S21" s="139"/>
+      <c r="R21" s="124"/>
+      <c r="S21" s="125"/>
     </row>
     <row r="22" spans="2:19" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B22" s="33">
@@ -3770,44 +3817,44 @@
         <v>5</v>
       </c>
       <c r="C22" s="3" t="s">
-        <v>352</v>
+        <v>374</v>
       </c>
       <c r="D22" s="90" t="s">
         <v>20</v>
       </c>
       <c r="E22" s="1" t="s">
-        <v>376</v>
+        <v>359</v>
       </c>
       <c r="F22" s="103" t="s">
-        <v>353</v>
+        <v>347</v>
       </c>
       <c r="G22" s="5" t="s">
-        <v>346</v>
+        <v>375</v>
       </c>
       <c r="I22" s="67" t="s">
         <v>41</v>
       </c>
-      <c r="J22" s="128" t="s">
+      <c r="J22" s="126" t="s">
         <v>98</v>
       </c>
-      <c r="K22" s="128"/>
-      <c r="L22" s="128"/>
+      <c r="K22" s="126"/>
+      <c r="L22" s="126"/>
       <c r="M22" s="69" t="s">
         <v>8</v>
       </c>
       <c r="O22" s="67" t="s">
         <v>41</v>
       </c>
-      <c r="P22" s="128" t="s">
+      <c r="P22" s="126" t="s">
         <v>98</v>
       </c>
-      <c r="Q22" s="128"/>
-      <c r="R22" s="128"/>
+      <c r="Q22" s="126"/>
+      <c r="R22" s="126"/>
       <c r="S22" s="69" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="23" spans="2:19" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="23" spans="2:19" ht="33.75" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B23" s="33">
         <f t="shared" si="0"/>
         <v>6</v>
@@ -3822,7 +3869,7 @@
         <v>79</v>
       </c>
       <c r="F23" s="103" t="s">
-        <v>242</v>
+        <v>389</v>
       </c>
       <c r="G23" s="5" t="s">
         <v>262</v>
@@ -3830,22 +3877,22 @@
       <c r="I23" s="70">
         <v>1</v>
       </c>
-      <c r="J23" s="140" t="s">
+      <c r="J23" s="135" t="s">
         <v>20</v>
       </c>
-      <c r="K23" s="140"/>
-      <c r="L23" s="140"/>
+      <c r="K23" s="135"/>
+      <c r="L23" s="135"/>
       <c r="M23" s="71" t="s">
         <v>134</v>
       </c>
       <c r="O23" s="87">
         <v>1</v>
       </c>
-      <c r="P23" s="129" t="s">
+      <c r="P23" s="142" t="s">
         <v>21</v>
       </c>
-      <c r="Q23" s="129"/>
-      <c r="R23" s="129"/>
+      <c r="Q23" s="142"/>
+      <c r="R23" s="142"/>
       <c r="S23" s="88" t="s">
         <v>133</v>
       </c>
@@ -3888,11 +3935,11 @@
       <c r="O24" s="80">
         <v>2</v>
       </c>
-      <c r="P24" s="119" t="s">
+      <c r="P24" s="124" t="s">
         <v>20</v>
       </c>
-      <c r="Q24" s="119"/>
-      <c r="R24" s="119"/>
+      <c r="Q24" s="124"/>
+      <c r="R24" s="124"/>
       <c r="S24" s="82" t="s">
         <v>134</v>
       </c>
@@ -4274,15 +4321,15 @@
       <c r="G32" s="5" t="s">
         <v>269</v>
       </c>
-      <c r="I32" s="123" t="s">
+      <c r="I32" s="136" t="s">
         <v>105</v>
       </c>
-      <c r="J32" s="124"/>
-      <c r="K32" s="125" t="s">
+      <c r="J32" s="137"/>
+      <c r="K32" s="138" t="s">
         <v>79</v>
       </c>
-      <c r="L32" s="126"/>
-      <c r="M32" s="127"/>
+      <c r="L32" s="139"/>
+      <c r="M32" s="140"/>
       <c r="O32" s="83">
         <v>7</v>
       </c>
@@ -4314,7 +4361,7 @@
         <v>241</v>
       </c>
       <c r="F33" s="103" t="s">
-        <v>360</v>
+        <v>353</v>
       </c>
       <c r="G33" s="5" t="s">
         <v>324</v>
@@ -4386,7 +4433,7 @@
         <v>241</v>
       </c>
       <c r="F35" s="103" t="s">
-        <v>360</v>
+        <v>353</v>
       </c>
       <c r="G35" s="5" t="s">
         <v>318</v>
@@ -4422,20 +4469,20 @@
         <v>241</v>
       </c>
       <c r="F36" s="103" t="s">
-        <v>378</v>
+        <v>361</v>
       </c>
       <c r="G36" s="5" t="s">
         <v>337</v>
       </c>
-      <c r="O36" s="123" t="s">
+      <c r="O36" s="136" t="s">
         <v>105</v>
       </c>
-      <c r="P36" s="124"/>
-      <c r="Q36" s="125" t="s">
+      <c r="P36" s="137"/>
+      <c r="Q36" s="138" t="s">
         <v>241</v>
       </c>
-      <c r="R36" s="126"/>
-      <c r="S36" s="127"/>
+      <c r="R36" s="139"/>
+      <c r="S36" s="140"/>
     </row>
     <row r="37" spans="2:19" ht="50.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B37" s="33">
@@ -4452,50 +4499,50 @@
         <v>241</v>
       </c>
       <c r="F37" s="103" t="s">
-        <v>361</v>
+        <v>354</v>
       </c>
       <c r="G37" s="5" t="s">
         <v>311</v>
       </c>
     </row>
-    <row r="38" spans="2:19" x14ac:dyDescent="0.3">
+    <row r="38" spans="2:19" ht="33" x14ac:dyDescent="0.3">
       <c r="B38" s="33">
         <f t="shared" si="0"/>
         <v>21</v>
       </c>
       <c r="C38" s="3" t="s">
-        <v>300</v>
-      </c>
-      <c r="D38" s="90" t="s">
-        <v>20</v>
-      </c>
-      <c r="E38" s="1" t="s">
-        <v>86</v>
-      </c>
-      <c r="F38" s="2" t="s">
-        <v>64</v>
+        <v>363</v>
+      </c>
+      <c r="D38" s="1">
+        <v>1</v>
+      </c>
+      <c r="E38" s="102" t="s">
+        <v>364</v>
+      </c>
+      <c r="F38" s="103" t="s">
+        <v>390</v>
       </c>
       <c r="G38" s="5" t="s">
-        <v>87</v>
-      </c>
-      <c r="I38" s="120" t="s">
+        <v>381</v>
+      </c>
+      <c r="I38" s="118" t="s">
         <v>103</v>
       </c>
-      <c r="J38" s="121"/>
-      <c r="K38" s="120" t="s">
+      <c r="J38" s="120"/>
+      <c r="K38" s="118" t="s">
         <v>123</v>
       </c>
-      <c r="L38" s="122"/>
-      <c r="M38" s="121"/>
-      <c r="O38" s="120" t="s">
+      <c r="L38" s="119"/>
+      <c r="M38" s="120"/>
+      <c r="O38" s="118" t="s">
         <v>103</v>
       </c>
-      <c r="P38" s="121"/>
-      <c r="Q38" s="120" t="s">
+      <c r="P38" s="120"/>
+      <c r="Q38" s="118" t="s">
         <v>174</v>
       </c>
-      <c r="R38" s="122"/>
-      <c r="S38" s="121"/>
+      <c r="R38" s="119"/>
+      <c r="S38" s="120"/>
     </row>
     <row r="39" spans="2:19" x14ac:dyDescent="0.3">
       <c r="B39" s="33">
@@ -4503,116 +4550,116 @@
         <v>22</v>
       </c>
       <c r="C39" s="3" t="s">
-        <v>234</v>
-      </c>
-      <c r="D39" s="101" t="s">
+        <v>300</v>
+      </c>
+      <c r="D39" s="90" t="s">
         <v>20</v>
       </c>
-      <c r="E39" s="102" t="s">
-        <v>238</v>
+      <c r="E39" s="1" t="s">
+        <v>86</v>
       </c>
       <c r="F39" s="2" t="s">
-        <v>36</v>
+        <v>64</v>
       </c>
       <c r="G39" s="5" t="s">
-        <v>235</v>
-      </c>
-      <c r="I39" s="130" t="s">
+        <v>87</v>
+      </c>
+      <c r="I39" s="127" t="s">
         <v>109</v>
       </c>
-      <c r="J39" s="131"/>
-      <c r="K39" s="132" t="s">
+      <c r="J39" s="128"/>
+      <c r="K39" s="129" t="s">
         <v>124</v>
       </c>
-      <c r="L39" s="133"/>
-      <c r="M39" s="134"/>
-      <c r="O39" s="130" t="s">
+      <c r="L39" s="130"/>
+      <c r="M39" s="131"/>
+      <c r="O39" s="127" t="s">
         <v>109</v>
       </c>
-      <c r="P39" s="131"/>
-      <c r="Q39" s="132" t="s">
+      <c r="P39" s="128"/>
+      <c r="Q39" s="129" t="s">
         <v>237</v>
       </c>
-      <c r="R39" s="133"/>
-      <c r="S39" s="134"/>
+      <c r="R39" s="130"/>
+      <c r="S39" s="131"/>
     </row>
     <row r="40" spans="2:19" x14ac:dyDescent="0.3">
       <c r="B40" s="33">
         <f t="shared" si="0"/>
         <v>23</v>
       </c>
-      <c r="C40" s="97" t="s">
-        <v>278</v>
-      </c>
-      <c r="D40" s="90" t="s">
-        <v>21</v>
-      </c>
-      <c r="E40" s="33" t="s">
+      <c r="C40" s="3" t="s">
+        <v>234</v>
+      </c>
+      <c r="D40" s="101" t="s">
+        <v>20</v>
+      </c>
+      <c r="E40" s="102" t="s">
+        <v>238</v>
+      </c>
+      <c r="F40" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="F40" s="98" t="s">
-        <v>35</v>
-      </c>
-      <c r="G40" s="99" t="s">
-        <v>279</v>
-      </c>
-      <c r="I40" s="130" t="s">
+      <c r="G40" s="5" t="s">
+        <v>235</v>
+      </c>
+      <c r="I40" s="127" t="s">
         <v>107</v>
       </c>
-      <c r="J40" s="131"/>
-      <c r="K40" s="132" t="s">
+      <c r="J40" s="128"/>
+      <c r="K40" s="129" t="s">
         <v>108</v>
       </c>
-      <c r="L40" s="133"/>
-      <c r="M40" s="134"/>
-      <c r="O40" s="130" t="s">
+      <c r="L40" s="130"/>
+      <c r="M40" s="131"/>
+      <c r="O40" s="127" t="s">
         <v>107</v>
       </c>
-      <c r="P40" s="131"/>
-      <c r="Q40" s="130" t="s">
+      <c r="P40" s="128"/>
+      <c r="Q40" s="127" t="s">
         <v>64</v>
       </c>
-      <c r="R40" s="135"/>
-      <c r="S40" s="131"/>
+      <c r="R40" s="141"/>
+      <c r="S40" s="128"/>
     </row>
     <row r="41" spans="2:19" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B41" s="33">
         <f t="shared" si="0"/>
         <v>24</v>
       </c>
-      <c r="C41" s="3" t="s">
-        <v>301</v>
+      <c r="C41" s="97" t="s">
+        <v>278</v>
       </c>
       <c r="D41" s="90" t="s">
-        <v>20</v>
-      </c>
-      <c r="E41" s="1" t="s">
-        <v>86</v>
-      </c>
-      <c r="F41" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="G41" s="5" t="s">
-        <v>88</v>
-      </c>
-      <c r="I41" s="136" t="s">
+        <v>21</v>
+      </c>
+      <c r="E41" s="33" t="s">
+        <v>36</v>
+      </c>
+      <c r="F41" s="98" t="s">
+        <v>35</v>
+      </c>
+      <c r="G41" s="99" t="s">
+        <v>279</v>
+      </c>
+      <c r="I41" s="121" t="s">
         <v>8</v>
       </c>
-      <c r="J41" s="137"/>
-      <c r="K41" s="138" t="s">
+      <c r="J41" s="122"/>
+      <c r="K41" s="123" t="s">
         <v>126</v>
       </c>
-      <c r="L41" s="119"/>
-      <c r="M41" s="139"/>
-      <c r="O41" s="136" t="s">
+      <c r="L41" s="124"/>
+      <c r="M41" s="125"/>
+      <c r="O41" s="121" t="s">
         <v>8</v>
       </c>
-      <c r="P41" s="137"/>
-      <c r="Q41" s="138" t="s">
+      <c r="P41" s="122"/>
+      <c r="Q41" s="123" t="s">
         <v>175</v>
       </c>
-      <c r="R41" s="119"/>
-      <c r="S41" s="139"/>
+      <c r="R41" s="124"/>
+      <c r="S41" s="125"/>
     </row>
     <row r="42" spans="2:19" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B42" s="33">
@@ -4620,39 +4667,39 @@
         <v>25</v>
       </c>
       <c r="C42" s="3" t="s">
-        <v>250</v>
-      </c>
-      <c r="D42" s="1">
-        <v>1</v>
-      </c>
-      <c r="E42" s="114" t="s">
-        <v>241</v>
-      </c>
-      <c r="F42" s="114" t="s">
-        <v>242</v>
+        <v>301</v>
+      </c>
+      <c r="D42" s="90" t="s">
+        <v>20</v>
+      </c>
+      <c r="E42" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="F42" s="2" t="s">
+        <v>64</v>
       </c>
       <c r="G42" s="5" t="s">
-        <v>252</v>
+        <v>88</v>
       </c>
       <c r="I42" s="67" t="s">
         <v>41</v>
       </c>
-      <c r="J42" s="128" t="s">
+      <c r="J42" s="126" t="s">
         <v>98</v>
       </c>
-      <c r="K42" s="128"/>
-      <c r="L42" s="128"/>
+      <c r="K42" s="126"/>
+      <c r="L42" s="126"/>
       <c r="M42" s="69" t="s">
         <v>8</v>
       </c>
       <c r="O42" s="67" t="s">
         <v>41</v>
       </c>
-      <c r="P42" s="128" t="s">
+      <c r="P42" s="126" t="s">
         <v>98</v>
       </c>
-      <c r="Q42" s="128"/>
-      <c r="R42" s="128"/>
+      <c r="Q42" s="126"/>
+      <c r="R42" s="126"/>
       <c r="S42" s="69" t="s">
         <v>8</v>
       </c>
@@ -4663,39 +4710,39 @@
         <v>26</v>
       </c>
       <c r="C43" s="3" t="s">
-        <v>270</v>
+        <v>250</v>
       </c>
       <c r="D43" s="1">
         <v>1</v>
       </c>
-      <c r="E43" s="2" t="s">
+      <c r="E43" s="114" t="s">
         <v>241</v>
       </c>
-      <c r="F43" s="103" t="s">
+      <c r="F43" s="114" t="s">
         <v>242</v>
       </c>
       <c r="G43" s="5" t="s">
-        <v>273</v>
+        <v>252</v>
       </c>
       <c r="I43" s="70">
         <v>1</v>
       </c>
-      <c r="J43" s="140" t="s">
+      <c r="J43" s="135" t="s">
         <v>20</v>
       </c>
-      <c r="K43" s="140"/>
-      <c r="L43" s="140"/>
+      <c r="K43" s="135"/>
+      <c r="L43" s="135"/>
       <c r="M43" s="71" t="s">
         <v>134</v>
       </c>
       <c r="O43" s="87">
         <v>1</v>
       </c>
-      <c r="P43" s="129" t="s">
+      <c r="P43" s="142" t="s">
         <v>21</v>
       </c>
-      <c r="Q43" s="129"/>
-      <c r="R43" s="129"/>
+      <c r="Q43" s="142"/>
+      <c r="R43" s="142"/>
       <c r="S43" s="88" t="s">
         <v>133</v>
       </c>
@@ -4706,19 +4753,19 @@
         <v>27</v>
       </c>
       <c r="C44" s="3" t="s">
-        <v>251</v>
+        <v>270</v>
       </c>
       <c r="D44" s="1">
         <v>1</v>
       </c>
-      <c r="E44" s="114" t="s">
+      <c r="E44" s="2" t="s">
         <v>241</v>
       </c>
-      <c r="F44" s="114" t="s">
+      <c r="F44" s="103" t="s">
         <v>242</v>
       </c>
       <c r="G44" s="5" t="s">
-        <v>253</v>
+        <v>273</v>
       </c>
       <c r="I44" s="67" t="s">
         <v>41</v>
@@ -4738,11 +4785,11 @@
       <c r="O44" s="80">
         <v>2</v>
       </c>
-      <c r="P44" s="119" t="s">
+      <c r="P44" s="124" t="s">
         <v>20</v>
       </c>
-      <c r="Q44" s="119"/>
-      <c r="R44" s="119"/>
+      <c r="Q44" s="124"/>
+      <c r="R44" s="124"/>
       <c r="S44" s="82" t="s">
         <v>134</v>
       </c>
@@ -4753,19 +4800,19 @@
         <v>28</v>
       </c>
       <c r="C45" s="3" t="s">
-        <v>222</v>
-      </c>
-      <c r="D45" s="90" t="s">
-        <v>20</v>
-      </c>
-      <c r="E45" s="1" t="s">
-        <v>238</v>
-      </c>
-      <c r="F45" s="103" t="s">
-        <v>375</v>
+        <v>251</v>
+      </c>
+      <c r="D45" s="1">
+        <v>1</v>
+      </c>
+      <c r="E45" s="114" t="s">
+        <v>241</v>
+      </c>
+      <c r="F45" s="114" t="s">
+        <v>242</v>
       </c>
       <c r="G45" s="5" t="s">
-        <v>224</v>
+        <v>253</v>
       </c>
       <c r="I45" s="72">
         <v>1</v>
@@ -4798,25 +4845,25 @@
         <v>8</v>
       </c>
     </row>
-    <row r="46" spans="2:19" ht="33" x14ac:dyDescent="0.3">
+    <row r="46" spans="2:19" x14ac:dyDescent="0.3">
       <c r="B46" s="33">
         <f t="shared" si="0"/>
         <v>29</v>
       </c>
-      <c r="C46" s="112" t="s">
-        <v>223</v>
-      </c>
-      <c r="D46" s="113" t="s">
+      <c r="C46" s="3" t="s">
+        <v>222</v>
+      </c>
+      <c r="D46" s="90" t="s">
         <v>20</v>
       </c>
-      <c r="E46" s="111" t="s">
+      <c r="E46" s="1" t="s">
         <v>238</v>
       </c>
-      <c r="F46" s="115" t="s">
-        <v>347</v>
-      </c>
-      <c r="G46" s="112" t="s">
-        <v>225</v>
+      <c r="F46" s="103" t="s">
+        <v>358</v>
+      </c>
+      <c r="G46" s="5" t="s">
+        <v>224</v>
       </c>
       <c r="I46" s="76">
         <v>2</v>
@@ -4849,25 +4896,25 @@
         <v>155</v>
       </c>
     </row>
-    <row r="47" spans="2:19" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="47" spans="2:19" ht="50.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B47" s="33">
         <f t="shared" si="0"/>
         <v>30</v>
       </c>
-      <c r="C47" s="3" t="s">
-        <v>357</v>
-      </c>
-      <c r="D47" s="90" t="s">
-        <v>56</v>
-      </c>
-      <c r="E47" s="1" t="s">
-        <v>63</v>
-      </c>
-      <c r="F47" s="2" t="s">
-        <v>242</v>
-      </c>
-      <c r="G47" s="5" t="s">
-        <v>358</v>
+      <c r="C47" s="112" t="s">
+        <v>223</v>
+      </c>
+      <c r="D47" s="113" t="s">
+        <v>20</v>
+      </c>
+      <c r="E47" s="111" t="s">
+        <v>238</v>
+      </c>
+      <c r="F47" s="115" t="s">
+        <v>391</v>
+      </c>
+      <c r="G47" s="112" t="s">
+        <v>225</v>
       </c>
       <c r="I47" s="80">
         <v>3</v>
@@ -4906,29 +4953,29 @@
         <v>31</v>
       </c>
       <c r="C48" s="3" t="s">
-        <v>305</v>
-      </c>
-      <c r="D48" s="1">
-        <v>1</v>
-      </c>
-      <c r="E48" s="2" t="s">
-        <v>241</v>
-      </c>
-      <c r="F48" s="103" t="s">
+        <v>350</v>
+      </c>
+      <c r="D48" s="90" t="s">
+        <v>56</v>
+      </c>
+      <c r="E48" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="F48" s="2" t="s">
         <v>242</v>
       </c>
       <c r="G48" s="5" t="s">
-        <v>307</v>
-      </c>
-      <c r="I48" s="123" t="s">
+        <v>351</v>
+      </c>
+      <c r="I48" s="136" t="s">
         <v>105</v>
       </c>
-      <c r="J48" s="124"/>
-      <c r="K48" s="125" t="s">
+      <c r="J48" s="137"/>
+      <c r="K48" s="138" t="s">
         <v>65</v>
       </c>
-      <c r="L48" s="126"/>
-      <c r="M48" s="127"/>
+      <c r="L48" s="139"/>
+      <c r="M48" s="140"/>
       <c r="O48" s="83">
         <v>3</v>
       </c>
@@ -4951,19 +4998,19 @@
         <v>32</v>
       </c>
       <c r="C49" s="3" t="s">
-        <v>285</v>
-      </c>
-      <c r="D49" s="90" t="s">
-        <v>49</v>
-      </c>
-      <c r="E49" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="F49" s="1" t="s">
-        <v>286</v>
+        <v>305</v>
+      </c>
+      <c r="D49" s="1">
+        <v>1</v>
+      </c>
+      <c r="E49" s="2" t="s">
+        <v>241</v>
+      </c>
+      <c r="F49" s="103" t="s">
+        <v>242</v>
       </c>
       <c r="G49" s="5" t="s">
-        <v>54</v>
+        <v>307</v>
       </c>
       <c r="O49" s="83">
         <v>4</v>
@@ -4987,19 +5034,19 @@
         <v>33</v>
       </c>
       <c r="C50" s="3" t="s">
+        <v>285</v>
+      </c>
+      <c r="D50" s="90" t="s">
+        <v>49</v>
+      </c>
+      <c r="E50" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="F50" s="1" t="s">
         <v>286</v>
       </c>
-      <c r="D50" s="90" t="s">
-        <v>20</v>
-      </c>
-      <c r="E50" s="1" t="s">
-        <v>285</v>
-      </c>
-      <c r="F50" s="2" t="s">
-        <v>40</v>
-      </c>
       <c r="G50" s="5" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="O50" s="83">
         <v>5</v>
@@ -5017,35 +5064,35 @@
         <v>182</v>
       </c>
     </row>
-    <row r="51" spans="2:19" ht="33" x14ac:dyDescent="0.3">
+    <row r="51" spans="2:19" x14ac:dyDescent="0.3">
       <c r="B51" s="33">
         <f t="shared" ref="B51:B82" si="1">IF(C51="","",B50+1)</f>
         <v>34</v>
       </c>
       <c r="C51" s="3" t="s">
-        <v>226</v>
+        <v>286</v>
       </c>
       <c r="D51" s="90" t="s">
         <v>20</v>
       </c>
       <c r="E51" s="1" t="s">
-        <v>238</v>
-      </c>
-      <c r="F51" s="103" t="s">
-        <v>48</v>
+        <v>285</v>
+      </c>
+      <c r="F51" s="2" t="s">
+        <v>40</v>
       </c>
       <c r="G51" s="5" t="s">
-        <v>228</v>
-      </c>
-      <c r="I51" s="120" t="s">
+        <v>52</v>
+      </c>
+      <c r="I51" s="118" t="s">
         <v>103</v>
       </c>
-      <c r="J51" s="121"/>
-      <c r="K51" s="120" t="s">
+      <c r="J51" s="120"/>
+      <c r="K51" s="118" t="s">
         <v>130</v>
       </c>
-      <c r="L51" s="122"/>
-      <c r="M51" s="121"/>
+      <c r="L51" s="119"/>
+      <c r="M51" s="120"/>
       <c r="O51" s="83">
         <v>6</v>
       </c>
@@ -5062,35 +5109,35 @@
         <v>169</v>
       </c>
     </row>
-    <row r="52" spans="2:19" x14ac:dyDescent="0.3">
+    <row r="52" spans="2:19" ht="33" x14ac:dyDescent="0.3">
       <c r="B52" s="33">
         <f t="shared" si="1"/>
         <v>35</v>
       </c>
       <c r="C52" s="3" t="s">
-        <v>366</v>
-      </c>
-      <c r="D52" s="1">
-        <v>1</v>
-      </c>
-      <c r="E52" s="2" t="s">
-        <v>378</v>
-      </c>
-      <c r="F52" s="2" t="s">
-        <v>375</v>
+        <v>226</v>
+      </c>
+      <c r="D52" s="90" t="s">
+        <v>20</v>
+      </c>
+      <c r="E52" s="1" t="s">
+        <v>238</v>
+      </c>
+      <c r="F52" s="103" t="s">
+        <v>48</v>
       </c>
       <c r="G52" s="5" t="s">
-        <v>370</v>
-      </c>
-      <c r="I52" s="130" t="s">
+        <v>228</v>
+      </c>
+      <c r="I52" s="127" t="s">
         <v>109</v>
       </c>
-      <c r="J52" s="131"/>
-      <c r="K52" s="132" t="s">
+      <c r="J52" s="128"/>
+      <c r="K52" s="129" t="s">
         <v>131</v>
       </c>
-      <c r="L52" s="133"/>
-      <c r="M52" s="134"/>
+      <c r="L52" s="130"/>
+      <c r="M52" s="131"/>
       <c r="O52" s="83">
         <v>7</v>
       </c>
@@ -5113,29 +5160,29 @@
         <v>36</v>
       </c>
       <c r="C53" s="3" t="s">
-        <v>367</v>
-      </c>
-      <c r="D53" s="1">
-        <v>1</v>
-      </c>
-      <c r="E53" s="2" t="s">
-        <v>378</v>
-      </c>
-      <c r="F53" s="2" t="s">
-        <v>376</v>
+        <v>393</v>
+      </c>
+      <c r="D53" s="90" t="s">
+        <v>20</v>
+      </c>
+      <c r="E53" s="1" t="s">
+        <v>388</v>
+      </c>
+      <c r="F53" s="1" t="s">
+        <v>242</v>
       </c>
       <c r="G53" s="5" t="s">
-        <v>369</v>
-      </c>
-      <c r="I53" s="130" t="s">
+        <v>394</v>
+      </c>
+      <c r="I53" s="127" t="s">
         <v>107</v>
       </c>
-      <c r="J53" s="131"/>
-      <c r="K53" s="132" t="s">
+      <c r="J53" s="128"/>
+      <c r="K53" s="129" t="s">
         <v>108</v>
       </c>
-      <c r="L53" s="133"/>
-      <c r="M53" s="134"/>
+      <c r="L53" s="130"/>
+      <c r="M53" s="131"/>
       <c r="O53" s="83">
         <v>8</v>
       </c>
@@ -5158,29 +5205,29 @@
         <v>37</v>
       </c>
       <c r="C54" s="3" t="s">
-        <v>372</v>
+        <v>366</v>
       </c>
       <c r="D54" s="1">
         <v>1</v>
       </c>
       <c r="E54" s="2" t="s">
-        <v>378</v>
+        <v>384</v>
       </c>
       <c r="F54" s="2" t="s">
-        <v>375</v>
+        <v>385</v>
       </c>
       <c r="G54" s="5" t="s">
-        <v>374</v>
-      </c>
-      <c r="I54" s="136" t="s">
+        <v>376</v>
+      </c>
+      <c r="I54" s="121" t="s">
         <v>8</v>
       </c>
-      <c r="J54" s="137"/>
-      <c r="K54" s="138" t="s">
+      <c r="J54" s="122"/>
+      <c r="K54" s="123" t="s">
         <v>132</v>
       </c>
-      <c r="L54" s="119"/>
-      <c r="M54" s="139"/>
+      <c r="L54" s="124"/>
+      <c r="M54" s="125"/>
       <c r="O54" s="83">
         <v>9</v>
       </c>
@@ -5203,28 +5250,28 @@
         <v>38</v>
       </c>
       <c r="C55" s="3" t="s">
-        <v>373</v>
+        <v>368</v>
       </c>
       <c r="D55" s="1">
         <v>1</v>
       </c>
       <c r="E55" s="2" t="s">
+        <v>384</v>
+      </c>
+      <c r="F55" s="2" t="s">
+        <v>385</v>
+      </c>
+      <c r="G55" s="5" t="s">
         <v>378</v>
-      </c>
-      <c r="F55" s="2" t="s">
-        <v>376</v>
-      </c>
-      <c r="G55" s="5" t="s">
-        <v>380</v>
       </c>
       <c r="I55" s="67" t="s">
         <v>41</v>
       </c>
-      <c r="J55" s="128" t="s">
+      <c r="J55" s="126" t="s">
         <v>98</v>
       </c>
-      <c r="K55" s="128"/>
-      <c r="L55" s="128"/>
+      <c r="K55" s="126"/>
+      <c r="L55" s="126"/>
       <c r="M55" s="69" t="s">
         <v>8</v>
       </c>
@@ -5250,40 +5297,40 @@
         <v>39</v>
       </c>
       <c r="C56" s="3" t="s">
-        <v>371</v>
-      </c>
-      <c r="D56" s="33">
-        <v>1</v>
-      </c>
-      <c r="E56" s="1" t="s">
-        <v>350</v>
+        <v>367</v>
+      </c>
+      <c r="D56" s="1">
+        <v>1</v>
+      </c>
+      <c r="E56" s="2" t="s">
+        <v>384</v>
       </c>
       <c r="F56" s="2" t="s">
-        <v>355</v>
+        <v>386</v>
       </c>
       <c r="G56" s="5" t="s">
-        <v>368</v>
+        <v>377</v>
       </c>
       <c r="I56" s="87">
         <v>1</v>
       </c>
-      <c r="J56" s="129" t="s">
+      <c r="J56" s="142" t="s">
         <v>20</v>
       </c>
-      <c r="K56" s="129"/>
-      <c r="L56" s="129"/>
+      <c r="K56" s="142"/>
+      <c r="L56" s="142"/>
       <c r="M56" s="88" t="s">
         <v>134</v>
       </c>
-      <c r="O56" s="123" t="s">
+      <c r="O56" s="136" t="s">
         <v>105</v>
       </c>
-      <c r="P56" s="124"/>
-      <c r="Q56" s="125" t="s">
+      <c r="P56" s="137"/>
+      <c r="Q56" s="138" t="s">
         <v>242</v>
       </c>
-      <c r="R56" s="126"/>
-      <c r="S56" s="127"/>
+      <c r="R56" s="139"/>
+      <c r="S56" s="140"/>
     </row>
     <row r="57" spans="2:19" ht="33.75" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B57" s="33">
@@ -5291,51 +5338,51 @@
         <v>40</v>
       </c>
       <c r="C57" s="3" t="s">
-        <v>193</v>
-      </c>
-      <c r="D57" s="90" t="s">
-        <v>20</v>
-      </c>
-      <c r="E57" s="1" t="s">
-        <v>239</v>
+        <v>369</v>
+      </c>
+      <c r="D57" s="1">
+        <v>1</v>
+      </c>
+      <c r="E57" s="2" t="s">
+        <v>384</v>
       </c>
       <c r="F57" s="2" t="s">
-        <v>44</v>
+        <v>386</v>
       </c>
       <c r="G57" s="5" t="s">
-        <v>194</v>
+        <v>379</v>
       </c>
       <c r="I57" s="80">
         <v>2</v>
       </c>
-      <c r="J57" s="119" t="s">
+      <c r="J57" s="124" t="s">
         <v>55</v>
       </c>
-      <c r="K57" s="119"/>
-      <c r="L57" s="119"/>
+      <c r="K57" s="124"/>
+      <c r="L57" s="124"/>
       <c r="M57" s="89" t="s">
         <v>135</v>
       </c>
     </row>
-    <row r="58" spans="2:19" ht="33.75" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="58" spans="2:19" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B58" s="33">
         <f t="shared" si="1"/>
         <v>41</v>
       </c>
       <c r="C58" s="3" t="s">
-        <v>197</v>
-      </c>
-      <c r="D58" s="90" t="s">
-        <v>21</v>
+        <v>370</v>
+      </c>
+      <c r="D58" s="33">
+        <v>1</v>
       </c>
       <c r="E58" s="1" t="s">
-        <v>239</v>
-      </c>
-      <c r="F58" s="103" t="s">
-        <v>258</v>
-      </c>
-      <c r="G58" s="99" t="s">
-        <v>195</v>
+        <v>364</v>
+      </c>
+      <c r="F58" s="2" t="s">
+        <v>348</v>
+      </c>
+      <c r="G58" s="5" t="s">
+        <v>380</v>
       </c>
       <c r="I58" s="67" t="s">
         <v>41</v>
@@ -5352,15 +5399,15 @@
       <c r="M58" s="69" t="s">
         <v>8</v>
       </c>
-      <c r="O58" s="120" t="s">
+      <c r="O58" s="118" t="s">
         <v>103</v>
       </c>
-      <c r="P58" s="121"/>
-      <c r="Q58" s="120" t="s">
+      <c r="P58" s="120"/>
+      <c r="Q58" s="118" t="s">
         <v>185</v>
       </c>
-      <c r="R58" s="122"/>
-      <c r="S58" s="121"/>
+      <c r="R58" s="119"/>
+      <c r="S58" s="120"/>
     </row>
     <row r="59" spans="2:19" x14ac:dyDescent="0.3">
       <c r="B59" s="33">
@@ -5368,19 +5415,19 @@
         <v>42</v>
       </c>
       <c r="C59" s="3" t="s">
-        <v>199</v>
-      </c>
-      <c r="D59" s="1">
-        <v>3</v>
+        <v>193</v>
+      </c>
+      <c r="D59" s="90" t="s">
+        <v>20</v>
       </c>
       <c r="E59" s="1" t="s">
-        <v>58</v>
+        <v>239</v>
       </c>
       <c r="F59" s="2" t="s">
-        <v>241</v>
+        <v>44</v>
       </c>
       <c r="G59" s="5" t="s">
-        <v>212</v>
+        <v>194</v>
       </c>
       <c r="I59" s="72">
         <v>1</v>
@@ -5397,35 +5444,35 @@
       <c r="M59" s="75" t="s">
         <v>59</v>
       </c>
-      <c r="O59" s="130" t="s">
+      <c r="O59" s="127" t="s">
         <v>109</v>
       </c>
-      <c r="P59" s="131"/>
-      <c r="Q59" s="132" t="s">
+      <c r="P59" s="128"/>
+      <c r="Q59" s="129" t="s">
         <v>237</v>
       </c>
-      <c r="R59" s="133"/>
-      <c r="S59" s="134"/>
-    </row>
-    <row r="60" spans="2:19" x14ac:dyDescent="0.3">
+      <c r="R59" s="130"/>
+      <c r="S59" s="131"/>
+    </row>
+    <row r="60" spans="2:19" ht="33" x14ac:dyDescent="0.3">
       <c r="B60" s="33">
         <f t="shared" si="1"/>
         <v>43</v>
       </c>
       <c r="C60" s="3" t="s">
-        <v>205</v>
-      </c>
-      <c r="D60" s="1">
-        <v>1</v>
+        <v>197</v>
+      </c>
+      <c r="D60" s="90" t="s">
+        <v>21</v>
       </c>
       <c r="E60" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="F60" s="2" t="s">
-        <v>241</v>
-      </c>
-      <c r="G60" s="5" t="s">
-        <v>219</v>
+        <v>239</v>
+      </c>
+      <c r="F60" s="103" t="s">
+        <v>258</v>
+      </c>
+      <c r="G60" s="99" t="s">
+        <v>195</v>
       </c>
       <c r="I60" s="76">
         <v>2</v>
@@ -5442,15 +5489,15 @@
       <c r="M60" s="79" t="s">
         <v>66</v>
       </c>
-      <c r="O60" s="130" t="s">
+      <c r="O60" s="127" t="s">
         <v>107</v>
       </c>
-      <c r="P60" s="131"/>
-      <c r="Q60" s="130" t="s">
+      <c r="P60" s="128"/>
+      <c r="Q60" s="127" t="s">
         <v>64</v>
       </c>
-      <c r="R60" s="135"/>
-      <c r="S60" s="131"/>
+      <c r="R60" s="141"/>
+      <c r="S60" s="128"/>
     </row>
     <row r="61" spans="2:19" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B61" s="33">
@@ -5458,19 +5505,19 @@
         <v>44</v>
       </c>
       <c r="C61" s="3" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="D61" s="1">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E61" s="1" t="s">
         <v>58</v>
       </c>
       <c r="F61" s="2" t="s">
-        <v>238</v>
+        <v>241</v>
       </c>
       <c r="G61" s="5" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="I61" s="83">
         <v>3</v>
@@ -5487,15 +5534,15 @@
       <c r="M61" s="85" t="s">
         <v>146</v>
       </c>
-      <c r="O61" s="136" t="s">
+      <c r="O61" s="121" t="s">
         <v>8</v>
       </c>
-      <c r="P61" s="137"/>
-      <c r="Q61" s="138" t="s">
+      <c r="P61" s="122"/>
+      <c r="Q61" s="123" t="s">
         <v>186</v>
       </c>
-      <c r="R61" s="119"/>
-      <c r="S61" s="139"/>
+      <c r="R61" s="124"/>
+      <c r="S61" s="125"/>
     </row>
     <row r="62" spans="2:19" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B62" s="33">
@@ -5503,7 +5550,7 @@
         <v>45</v>
       </c>
       <c r="C62" s="3" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="D62" s="1">
         <v>1</v>
@@ -5515,7 +5562,7 @@
         <v>241</v>
       </c>
       <c r="G62" s="5" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="I62" s="83">
         <v>4</v>
@@ -5535,11 +5582,11 @@
       <c r="O62" s="67" t="s">
         <v>41</v>
       </c>
-      <c r="P62" s="128" t="s">
+      <c r="P62" s="126" t="s">
         <v>98</v>
       </c>
-      <c r="Q62" s="128"/>
-      <c r="R62" s="128"/>
+      <c r="Q62" s="126"/>
+      <c r="R62" s="126"/>
       <c r="S62" s="69" t="s">
         <v>8</v>
       </c>
@@ -5550,19 +5597,19 @@
         <v>46</v>
       </c>
       <c r="C63" s="3" t="s">
-        <v>293</v>
-      </c>
-      <c r="D63" s="90" t="s">
-        <v>57</v>
+        <v>200</v>
+      </c>
+      <c r="D63" s="1">
+        <v>1</v>
       </c>
       <c r="E63" s="1" t="s">
-        <v>44</v>
+        <v>58</v>
       </c>
       <c r="F63" s="2" t="s">
-        <v>43</v>
+        <v>238</v>
       </c>
       <c r="G63" s="5" t="s">
-        <v>61</v>
+        <v>214</v>
       </c>
       <c r="I63" s="83">
         <v>5</v>
@@ -5582,11 +5629,11 @@
       <c r="O63" s="87">
         <v>1</v>
       </c>
-      <c r="P63" s="129" t="s">
+      <c r="P63" s="142" t="s">
         <v>21</v>
       </c>
-      <c r="Q63" s="129"/>
-      <c r="R63" s="129"/>
+      <c r="Q63" s="142"/>
+      <c r="R63" s="142"/>
       <c r="S63" s="88" t="s">
         <v>133</v>
       </c>
@@ -5597,19 +5644,19 @@
         <v>47</v>
       </c>
       <c r="C64" s="3" t="s">
-        <v>244</v>
+        <v>206</v>
       </c>
       <c r="D64" s="1">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="E64" s="1" t="s">
-        <v>44</v>
+        <v>58</v>
       </c>
       <c r="F64" s="2" t="s">
         <v>241</v>
       </c>
       <c r="G64" s="5" t="s">
-        <v>245</v>
+        <v>220</v>
       </c>
       <c r="I64" s="83">
         <v>6</v>
@@ -5629,34 +5676,34 @@
       <c r="O64" s="80">
         <v>2</v>
       </c>
-      <c r="P64" s="119" t="s">
+      <c r="P64" s="124" t="s">
         <v>20</v>
       </c>
-      <c r="Q64" s="119"/>
-      <c r="R64" s="119"/>
+      <c r="Q64" s="124"/>
+      <c r="R64" s="124"/>
       <c r="S64" s="82" t="s">
         <v>134</v>
       </c>
     </row>
-    <row r="65" spans="2:19" ht="33.75" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="65" spans="2:19" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B65" s="33">
         <f t="shared" si="1"/>
         <v>48</v>
       </c>
-      <c r="C65" s="97" t="s">
-        <v>280</v>
-      </c>
-      <c r="D65" s="101" t="s">
-        <v>45</v>
-      </c>
-      <c r="E65" s="33" t="s">
+      <c r="C65" s="3" t="s">
+        <v>293</v>
+      </c>
+      <c r="D65" s="90" t="s">
+        <v>57</v>
+      </c>
+      <c r="E65" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="F65" s="98" t="s">
-        <v>42</v>
-      </c>
-      <c r="G65" s="99" t="s">
-        <v>50</v>
+      <c r="F65" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="G65" s="5" t="s">
+        <v>61</v>
       </c>
       <c r="I65" s="83">
         <v>7</v>
@@ -5695,19 +5742,19 @@
         <v>49</v>
       </c>
       <c r="C66" s="3" t="s">
-        <v>288</v>
-      </c>
-      <c r="D66" s="90" t="s">
-        <v>55</v>
+        <v>244</v>
+      </c>
+      <c r="D66" s="1">
+        <v>6</v>
       </c>
       <c r="E66" s="1" t="s">
         <v>44</v>
       </c>
       <c r="F66" s="2" t="s">
-        <v>58</v>
+        <v>241</v>
       </c>
       <c r="G66" s="5" t="s">
-        <v>59</v>
+        <v>245</v>
       </c>
       <c r="I66" s="83">
         <v>8</v>
@@ -5740,25 +5787,25 @@
         <v>155</v>
       </c>
     </row>
-    <row r="67" spans="2:19" x14ac:dyDescent="0.3">
+    <row r="67" spans="2:19" ht="33" x14ac:dyDescent="0.3">
       <c r="B67" s="33">
         <f t="shared" si="1"/>
         <v>50</v>
       </c>
-      <c r="C67" s="3" t="s">
-        <v>291</v>
-      </c>
-      <c r="D67" s="90" t="s">
-        <v>56</v>
-      </c>
-      <c r="E67" s="1" t="s">
+      <c r="C67" s="97" t="s">
+        <v>280</v>
+      </c>
+      <c r="D67" s="101" t="s">
+        <v>45</v>
+      </c>
+      <c r="E67" s="33" t="s">
         <v>44</v>
       </c>
-      <c r="F67" s="2" t="s">
-        <v>241</v>
-      </c>
-      <c r="G67" s="5" t="s">
-        <v>310</v>
+      <c r="F67" s="98" t="s">
+        <v>42</v>
+      </c>
+      <c r="G67" s="99" t="s">
+        <v>50</v>
       </c>
       <c r="I67" s="83">
         <v>9</v>
@@ -5791,25 +5838,25 @@
         <v>156</v>
       </c>
     </row>
-    <row r="68" spans="2:19" ht="33" x14ac:dyDescent="0.3">
+    <row r="68" spans="2:19" x14ac:dyDescent="0.3">
       <c r="B68" s="33">
         <f t="shared" si="1"/>
         <v>51</v>
       </c>
       <c r="C68" s="3" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="D68" s="90" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="E68" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="F68" s="103" t="s">
-        <v>339</v>
+      <c r="F68" s="2" t="s">
+        <v>58</v>
       </c>
       <c r="G68" s="5" t="s">
-        <v>338</v>
+        <v>59</v>
       </c>
       <c r="I68" s="83">
         <v>10</v>
@@ -5848,7 +5895,7 @@
         <v>52</v>
       </c>
       <c r="C69" s="3" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="D69" s="90" t="s">
         <v>56</v>
@@ -5857,10 +5904,10 @@
         <v>44</v>
       </c>
       <c r="F69" s="2" t="s">
-        <v>62</v>
+        <v>241</v>
       </c>
       <c r="G69" s="5" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="I69" s="83">
         <v>11</v>
@@ -5893,25 +5940,25 @@
         <v>182</v>
       </c>
     </row>
-    <row r="70" spans="2:19" x14ac:dyDescent="0.3">
+    <row r="70" spans="2:19" ht="33" x14ac:dyDescent="0.3">
       <c r="B70" s="33">
         <f t="shared" si="1"/>
         <v>53</v>
       </c>
       <c r="C70" s="3" t="s">
-        <v>292</v>
-      </c>
-      <c r="D70" s="1">
-        <v>5</v>
+        <v>289</v>
+      </c>
+      <c r="D70" s="90" t="s">
+        <v>56</v>
       </c>
       <c r="E70" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="F70" s="2" t="s">
-        <v>64</v>
+      <c r="F70" s="103" t="s">
+        <v>339</v>
       </c>
       <c r="G70" s="5" t="s">
-        <v>60</v>
+        <v>338</v>
       </c>
       <c r="I70" s="83">
         <v>12</v>
@@ -5944,25 +5991,25 @@
         <v>189</v>
       </c>
     </row>
-    <row r="71" spans="2:19" ht="33.75" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="71" spans="2:19" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B71" s="33">
         <f t="shared" si="1"/>
         <v>54</v>
       </c>
       <c r="C71" s="3" t="s">
-        <v>232</v>
-      </c>
-      <c r="D71" s="101" t="s">
-        <v>20</v>
-      </c>
-      <c r="E71" s="102" t="s">
-        <v>284</v>
+        <v>290</v>
+      </c>
+      <c r="D71" s="90" t="s">
+        <v>56</v>
+      </c>
+      <c r="E71" s="1" t="s">
+        <v>44</v>
       </c>
       <c r="F71" s="2" t="s">
-        <v>241</v>
+        <v>62</v>
       </c>
       <c r="G71" s="5" t="s">
-        <v>233</v>
+        <v>311</v>
       </c>
       <c r="I71" s="80">
         <v>13</v>
@@ -6001,58 +6048,58 @@
         <v>55</v>
       </c>
       <c r="C72" s="3" t="s">
-        <v>203</v>
+        <v>292</v>
       </c>
       <c r="D72" s="1">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="E72" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="F72" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="G72" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="I72" s="136" t="s">
+        <v>105</v>
+      </c>
+      <c r="J72" s="137"/>
+      <c r="K72" s="138" t="s">
         <v>58</v>
       </c>
-      <c r="F72" s="114" t="s">
+      <c r="L72" s="139"/>
+      <c r="M72" s="140"/>
+      <c r="O72" s="136" t="s">
+        <v>105</v>
+      </c>
+      <c r="P72" s="137"/>
+      <c r="Q72" s="138" t="s">
+        <v>243</v>
+      </c>
+      <c r="R72" s="139"/>
+      <c r="S72" s="140"/>
+    </row>
+    <row r="73" spans="2:19" ht="33" x14ac:dyDescent="0.3">
+      <c r="B73" s="33">
+        <f t="shared" si="1"/>
+        <v>56</v>
+      </c>
+      <c r="C73" s="3" t="s">
+        <v>232</v>
+      </c>
+      <c r="D73" s="101" t="s">
+        <v>20</v>
+      </c>
+      <c r="E73" s="102" t="s">
+        <v>284</v>
+      </c>
+      <c r="F73" s="2" t="s">
         <v>241</v>
       </c>
-      <c r="G72" s="5" t="s">
-        <v>217</v>
-      </c>
-      <c r="I72" s="123" t="s">
-        <v>105</v>
-      </c>
-      <c r="J72" s="124"/>
-      <c r="K72" s="125" t="s">
-        <v>58</v>
-      </c>
-      <c r="L72" s="126"/>
-      <c r="M72" s="127"/>
-      <c r="O72" s="123" t="s">
-        <v>105</v>
-      </c>
-      <c r="P72" s="124"/>
-      <c r="Q72" s="125" t="s">
-        <v>243</v>
-      </c>
-      <c r="R72" s="126"/>
-      <c r="S72" s="127"/>
-    </row>
-    <row r="73" spans="2:19" x14ac:dyDescent="0.3">
-      <c r="B73" s="33">
-        <f t="shared" si="1"/>
-        <v>56</v>
-      </c>
-      <c r="C73" s="3" t="s">
-        <v>201</v>
-      </c>
-      <c r="D73" s="1">
-        <v>1</v>
-      </c>
-      <c r="E73" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="F73" s="2" t="s">
-        <v>238</v>
-      </c>
       <c r="G73" s="5" t="s">
-        <v>215</v>
+        <v>233</v>
       </c>
     </row>
     <row r="74" spans="2:19" x14ac:dyDescent="0.3">
@@ -6061,7 +6108,7 @@
         <v>57</v>
       </c>
       <c r="C74" s="3" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="D74" s="1">
         <v>1</v>
@@ -6073,7 +6120,7 @@
         <v>241</v>
       </c>
       <c r="G74" s="5" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
     </row>
     <row r="75" spans="2:19" x14ac:dyDescent="0.3">
@@ -6082,19 +6129,19 @@
         <v>58</v>
       </c>
       <c r="C75" s="3" t="s">
-        <v>208</v>
-      </c>
-      <c r="D75" s="90" t="s">
-        <v>20</v>
+        <v>201</v>
+      </c>
+      <c r="D75" s="1">
+        <v>1</v>
       </c>
       <c r="E75" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="F75" s="111" t="s">
+        <v>58</v>
+      </c>
+      <c r="F75" s="2" t="s">
         <v>238</v>
       </c>
       <c r="G75" s="5" t="s">
-        <v>210</v>
+        <v>215</v>
       </c>
     </row>
     <row r="76" spans="2:19" x14ac:dyDescent="0.3">
@@ -6102,20 +6149,20 @@
         <f t="shared" si="1"/>
         <v>59</v>
       </c>
-      <c r="C76" s="112" t="s">
-        <v>209</v>
-      </c>
-      <c r="D76" s="113" t="s">
-        <v>20</v>
+      <c r="C76" s="3" t="s">
+        <v>204</v>
+      </c>
+      <c r="D76" s="1">
+        <v>1</v>
       </c>
       <c r="E76" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="F76" s="111" t="s">
-        <v>238</v>
-      </c>
-      <c r="G76" s="112" t="s">
-        <v>211</v>
+        <v>58</v>
+      </c>
+      <c r="F76" s="114" t="s">
+        <v>241</v>
+      </c>
+      <c r="G76" s="5" t="s">
+        <v>218</v>
       </c>
     </row>
     <row r="77" spans="2:19" x14ac:dyDescent="0.3">
@@ -6124,19 +6171,19 @@
         <v>60</v>
       </c>
       <c r="C77" s="3" t="s">
-        <v>363</v>
-      </c>
-      <c r="D77" s="1">
-        <v>1</v>
+        <v>208</v>
+      </c>
+      <c r="D77" s="90" t="s">
+        <v>20</v>
       </c>
       <c r="E77" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="F77" s="1" t="s">
-        <v>241</v>
+        <v>62</v>
+      </c>
+      <c r="F77" s="111" t="s">
+        <v>238</v>
       </c>
       <c r="G77" s="5" t="s">
-        <v>213</v>
+        <v>210</v>
       </c>
     </row>
     <row r="78" spans="2:19" x14ac:dyDescent="0.3">
@@ -6144,41 +6191,41 @@
         <f t="shared" si="1"/>
         <v>61</v>
       </c>
-      <c r="C78" s="3" t="s">
-        <v>202</v>
-      </c>
-      <c r="D78" s="1">
-        <v>1</v>
+      <c r="C78" s="112" t="s">
+        <v>209</v>
+      </c>
+      <c r="D78" s="113" t="s">
+        <v>20</v>
       </c>
       <c r="E78" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="F78" s="111" t="s">
+        <v>238</v>
+      </c>
+      <c r="G78" s="112" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="79" spans="2:19" x14ac:dyDescent="0.3">
+      <c r="B79" s="33">
+        <f t="shared" si="1"/>
+        <v>62</v>
+      </c>
+      <c r="C79" s="3" t="s">
+        <v>355</v>
+      </c>
+      <c r="D79" s="1">
+        <v>1</v>
+      </c>
+      <c r="E79" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="F78" s="2" t="s">
+      <c r="F79" s="1" t="s">
         <v>241</v>
       </c>
-      <c r="G78" s="5" t="s">
-        <v>216</v>
-      </c>
-    </row>
-    <row r="79" spans="2:19" ht="49.5" x14ac:dyDescent="0.3">
-      <c r="B79" s="33">
-        <f t="shared" si="1"/>
-        <v>62</v>
-      </c>
-      <c r="C79" s="3" t="s">
-        <v>283</v>
-      </c>
-      <c r="D79" s="101" t="s">
-        <v>46</v>
-      </c>
-      <c r="E79" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="F79" s="2" t="s">
-        <v>232</v>
-      </c>
       <c r="G79" s="5" t="s">
-        <v>51</v>
+        <v>213</v>
       </c>
     </row>
     <row r="80" spans="2:19" x14ac:dyDescent="0.3">
@@ -6187,7 +6234,7 @@
         <v>63</v>
       </c>
       <c r="C80" s="3" t="s">
-        <v>207</v>
+        <v>202</v>
       </c>
       <c r="D80" s="1">
         <v>1</v>
@@ -6196,31 +6243,31 @@
         <v>58</v>
       </c>
       <c r="F80" s="2" t="s">
-        <v>43</v>
+        <v>241</v>
       </c>
       <c r="G80" s="5" t="s">
-        <v>221</v>
-      </c>
-    </row>
-    <row r="81" spans="2:7" x14ac:dyDescent="0.3">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="81" spans="2:7" ht="49.5" x14ac:dyDescent="0.3">
       <c r="B81" s="33">
         <f t="shared" si="1"/>
         <v>64</v>
       </c>
       <c r="C81" s="3" t="s">
-        <v>229</v>
-      </c>
-      <c r="D81" s="90" t="s">
-        <v>20</v>
+        <v>283</v>
+      </c>
+      <c r="D81" s="101" t="s">
+        <v>46</v>
       </c>
       <c r="E81" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="F81" s="103" t="s">
-        <v>238</v>
+        <v>42</v>
+      </c>
+      <c r="F81" s="2" t="s">
+        <v>232</v>
       </c>
       <c r="G81" s="5" t="s">
-        <v>227</v>
+        <v>51</v>
       </c>
     </row>
     <row r="82" spans="2:7" x14ac:dyDescent="0.3">
@@ -6228,41 +6275,41 @@
         <f t="shared" si="1"/>
         <v>65</v>
       </c>
-      <c r="C82" s="97" t="s">
-        <v>191</v>
-      </c>
-      <c r="D82" s="90" t="s">
-        <v>21</v>
-      </c>
-      <c r="E82" s="33" t="s">
-        <v>39</v>
-      </c>
-      <c r="F82" s="98" t="s">
-        <v>240</v>
-      </c>
-      <c r="G82" s="99" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="83" spans="2:7" ht="33" x14ac:dyDescent="0.3">
+      <c r="C82" s="3" t="s">
+        <v>207</v>
+      </c>
+      <c r="D82" s="1">
+        <v>1</v>
+      </c>
+      <c r="E82" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="F82" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="G82" s="5" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="83" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B83" s="33">
         <f t="shared" ref="B83:B114" si="2">IF(C83="","",B82+1)</f>
         <v>66</v>
       </c>
-      <c r="C83" s="93" t="s">
-        <v>281</v>
-      </c>
-      <c r="D83" s="94" t="s">
-        <v>21</v>
-      </c>
-      <c r="E83" s="92" t="s">
-        <v>35</v>
-      </c>
-      <c r="F83" s="95" t="s">
-        <v>74</v>
-      </c>
-      <c r="G83" s="96" t="s">
-        <v>37</v>
+      <c r="C83" s="3" t="s">
+        <v>229</v>
+      </c>
+      <c r="D83" s="90" t="s">
+        <v>20</v>
+      </c>
+      <c r="E83" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="F83" s="103" t="s">
+        <v>238</v>
+      </c>
+      <c r="G83" s="5" t="s">
+        <v>227</v>
       </c>
     </row>
     <row r="84" spans="2:7" x14ac:dyDescent="0.3">
@@ -6270,62 +6317,62 @@
         <f t="shared" si="2"/>
         <v>67</v>
       </c>
-      <c r="C84" s="93" t="s">
+      <c r="C84" s="97" t="s">
+        <v>191</v>
+      </c>
+      <c r="D84" s="90" t="s">
+        <v>21</v>
+      </c>
+      <c r="E84" s="33" t="s">
+        <v>39</v>
+      </c>
+      <c r="F84" s="98" t="s">
+        <v>240</v>
+      </c>
+      <c r="G84" s="99" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="85" spans="2:7" ht="33" x14ac:dyDescent="0.3">
+      <c r="B85" s="33">
+        <f t="shared" si="2"/>
+        <v>68</v>
+      </c>
+      <c r="C85" s="93" t="s">
+        <v>281</v>
+      </c>
+      <c r="D85" s="94" t="s">
+        <v>21</v>
+      </c>
+      <c r="E85" s="92" t="s">
+        <v>35</v>
+      </c>
+      <c r="F85" s="95" t="s">
+        <v>74</v>
+      </c>
+      <c r="G85" s="96" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="86" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="B86" s="33">
+        <f t="shared" si="2"/>
+        <v>69</v>
+      </c>
+      <c r="C86" s="93" t="s">
         <v>282</v>
       </c>
-      <c r="D84" s="92">
-        <v>1</v>
-      </c>
-      <c r="E84" s="92" t="s">
+      <c r="D86" s="92">
+        <v>1</v>
+      </c>
+      <c r="E86" s="92" t="s">
         <v>35</v>
       </c>
-      <c r="F84" s="100" t="s">
+      <c r="F86" s="100" t="s">
         <v>11</v>
       </c>
-      <c r="G84" s="96" t="s">
+      <c r="G86" s="96" t="s">
         <v>38</v>
-      </c>
-    </row>
-    <row r="85" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B85" s="33">
-        <f t="shared" si="2"/>
-        <v>68</v>
-      </c>
-      <c r="C85" s="3" t="s">
-        <v>342</v>
-      </c>
-      <c r="D85" s="90" t="s">
-        <v>21</v>
-      </c>
-      <c r="E85" s="1" t="s">
-        <v>343</v>
-      </c>
-      <c r="F85" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="G85" s="5" t="s">
-        <v>344</v>
-      </c>
-    </row>
-    <row r="86" spans="2:7" ht="66" x14ac:dyDescent="0.3">
-      <c r="B86" s="33">
-        <f t="shared" si="2"/>
-        <v>69</v>
-      </c>
-      <c r="C86" s="104" t="s">
-        <v>260</v>
-      </c>
-      <c r="D86" s="109" t="s">
-        <v>20</v>
-      </c>
-      <c r="E86" s="105" t="s">
-        <v>242</v>
-      </c>
-      <c r="F86" s="110" t="s">
-        <v>377</v>
-      </c>
-      <c r="G86" s="107" t="s">
-        <v>263</v>
       </c>
     </row>
     <row r="87" spans="2:7" x14ac:dyDescent="0.3">
@@ -6334,40 +6381,40 @@
         <v>70</v>
       </c>
       <c r="C87" s="3" t="s">
-        <v>315</v>
+        <v>342</v>
       </c>
       <c r="D87" s="90" t="s">
-        <v>56</v>
-      </c>
-      <c r="E87" s="103" t="s">
+        <v>21</v>
+      </c>
+      <c r="E87" s="1" t="s">
+        <v>343</v>
+      </c>
+      <c r="F87" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="G87" s="5" t="s">
+        <v>344</v>
+      </c>
+    </row>
+    <row r="88" spans="2:7" ht="66" x14ac:dyDescent="0.3">
+      <c r="B88" s="33">
+        <f t="shared" si="2"/>
+        <v>71</v>
+      </c>
+      <c r="C88" s="104" t="s">
+        <v>260</v>
+      </c>
+      <c r="D88" s="109" t="s">
+        <v>20</v>
+      </c>
+      <c r="E88" s="105" t="s">
         <v>242</v>
       </c>
-      <c r="F87" s="103" t="s">
-        <v>243</v>
-      </c>
-      <c r="G87" s="5" t="s">
-        <v>320</v>
-      </c>
-    </row>
-    <row r="88" spans="2:7" ht="33" x14ac:dyDescent="0.3">
-      <c r="B88" s="33">
-        <f t="shared" si="2"/>
-        <v>71</v>
-      </c>
-      <c r="C88" s="3" t="s">
-        <v>314</v>
-      </c>
-      <c r="D88" s="90" t="s">
-        <v>56</v>
-      </c>
-      <c r="E88" s="103" t="s">
-        <v>242</v>
-      </c>
-      <c r="F88" s="103" t="s">
-        <v>362</v>
-      </c>
-      <c r="G88" s="5" t="s">
-        <v>319</v>
+      <c r="F88" s="110" t="s">
+        <v>360</v>
+      </c>
+      <c r="G88" s="107" t="s">
+        <v>263</v>
       </c>
     </row>
     <row r="89" spans="2:7" x14ac:dyDescent="0.3">
@@ -6375,62 +6422,62 @@
         <f t="shared" si="2"/>
         <v>72</v>
       </c>
-      <c r="C89" s="104" t="s">
-        <v>254</v>
-      </c>
-      <c r="D89" s="105">
-        <v>1</v>
-      </c>
-      <c r="E89" s="105" t="s">
+      <c r="C89" s="3" t="s">
+        <v>315</v>
+      </c>
+      <c r="D89" s="90" t="s">
+        <v>56</v>
+      </c>
+      <c r="E89" s="103" t="s">
         <v>242</v>
       </c>
-      <c r="F89" s="106" t="s">
-        <v>14</v>
-      </c>
-      <c r="G89" s="107" t="s">
-        <v>256</v>
-      </c>
-    </row>
-    <row r="90" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="F89" s="103" t="s">
+        <v>243</v>
+      </c>
+      <c r="G89" s="5" t="s">
+        <v>320</v>
+      </c>
+    </row>
+    <row r="90" spans="2:7" ht="33" x14ac:dyDescent="0.3">
       <c r="B90" s="33">
         <f t="shared" si="2"/>
         <v>73</v>
       </c>
       <c r="C90" s="3" t="s">
-        <v>271</v>
-      </c>
-      <c r="D90" s="1">
-        <v>1</v>
-      </c>
-      <c r="E90" s="2" t="s">
+        <v>314</v>
+      </c>
+      <c r="D90" s="90" t="s">
+        <v>56</v>
+      </c>
+      <c r="E90" s="103" t="s">
         <v>242</v>
       </c>
-      <c r="F90" s="2" t="s">
-        <v>243</v>
+      <c r="F90" s="103" t="s">
+        <v>387</v>
       </c>
       <c r="G90" s="5" t="s">
-        <v>274</v>
-      </c>
-    </row>
-    <row r="91" spans="2:7" ht="33" x14ac:dyDescent="0.3">
+        <v>319</v>
+      </c>
+    </row>
+    <row r="91" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B91" s="33">
         <f t="shared" si="2"/>
         <v>74</v>
       </c>
-      <c r="C91" s="104" t="s">
-        <v>255</v>
-      </c>
-      <c r="D91" s="105">
-        <v>1</v>
-      </c>
-      <c r="E91" s="105" t="s">
+      <c r="C91" s="3" t="s">
+        <v>365</v>
+      </c>
+      <c r="D91" s="1">
+        <v>1</v>
+      </c>
+      <c r="E91" s="2" t="s">
         <v>242</v>
       </c>
-      <c r="F91" s="108" t="s">
-        <v>73</v>
-      </c>
-      <c r="G91" s="107" t="s">
-        <v>257</v>
+      <c r="F91" s="103" t="s">
+        <v>348</v>
+      </c>
+      <c r="G91" s="5" t="s">
+        <v>382</v>
       </c>
     </row>
     <row r="92" spans="2:7" x14ac:dyDescent="0.3">
@@ -6438,20 +6485,20 @@
         <f t="shared" si="2"/>
         <v>75</v>
       </c>
-      <c r="C92" s="112" t="s">
-        <v>264</v>
-      </c>
-      <c r="D92" s="113" t="s">
-        <v>20</v>
-      </c>
-      <c r="E92" s="111" t="s">
+      <c r="C92" s="104" t="s">
+        <v>254</v>
+      </c>
+      <c r="D92" s="105">
+        <v>1</v>
+      </c>
+      <c r="E92" s="105" t="s">
         <v>242</v>
       </c>
-      <c r="F92" s="118" t="s">
-        <v>355</v>
-      </c>
-      <c r="G92" s="112" t="s">
-        <v>265</v>
+      <c r="F92" s="106" t="s">
+        <v>14</v>
+      </c>
+      <c r="G92" s="107" t="s">
+        <v>256</v>
       </c>
     </row>
     <row r="93" spans="2:7" x14ac:dyDescent="0.3">
@@ -6460,19 +6507,19 @@
         <v>76</v>
       </c>
       <c r="C93" s="3" t="s">
-        <v>364</v>
+        <v>271</v>
       </c>
       <c r="D93" s="1">
         <v>1</v>
       </c>
-      <c r="E93" s="103" t="s">
+      <c r="E93" s="2" t="s">
         <v>242</v>
       </c>
-      <c r="F93" s="103" t="s">
+      <c r="F93" s="2" t="s">
         <v>243</v>
       </c>
       <c r="G93" s="5" t="s">
-        <v>325</v>
+        <v>274</v>
       </c>
     </row>
     <row r="94" spans="2:7" ht="33" x14ac:dyDescent="0.3">
@@ -6480,41 +6527,41 @@
         <f t="shared" si="2"/>
         <v>77</v>
       </c>
-      <c r="C94" s="3" t="s">
-        <v>340</v>
-      </c>
-      <c r="D94" s="90" t="s">
-        <v>56</v>
-      </c>
-      <c r="E94" s="1" t="s">
+      <c r="C94" s="104" t="s">
+        <v>255</v>
+      </c>
+      <c r="D94" s="105">
+        <v>1</v>
+      </c>
+      <c r="E94" s="105" t="s">
         <v>242</v>
       </c>
-      <c r="F94" s="103" t="s">
-        <v>359</v>
-      </c>
-      <c r="G94" s="5" t="s">
-        <v>341</v>
-      </c>
-    </row>
-    <row r="95" spans="2:7" ht="33" x14ac:dyDescent="0.3">
+      <c r="F94" s="108" t="s">
+        <v>73</v>
+      </c>
+      <c r="G94" s="107" t="s">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="95" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B95" s="33">
         <f t="shared" si="2"/>
         <v>78</v>
       </c>
-      <c r="C95" s="3" t="s">
+      <c r="C95" s="112" t="s">
+        <v>264</v>
+      </c>
+      <c r="D95" s="113" t="s">
+        <v>20</v>
+      </c>
+      <c r="E95" s="111" t="s">
+        <v>242</v>
+      </c>
+      <c r="F95" s="143" t="s">
         <v>348</v>
       </c>
-      <c r="D95" s="1">
-        <v>1</v>
-      </c>
-      <c r="E95" s="2" t="s">
-        <v>242</v>
-      </c>
-      <c r="F95" s="103" t="s">
-        <v>349</v>
-      </c>
-      <c r="G95" s="5" t="s">
-        <v>308</v>
+      <c r="G95" s="112" t="s">
+        <v>265</v>
       </c>
     </row>
     <row r="96" spans="2:7" x14ac:dyDescent="0.3">
@@ -6522,62 +6569,62 @@
         <f t="shared" si="2"/>
         <v>79</v>
       </c>
-      <c r="C96" s="104" t="s">
-        <v>354</v>
-      </c>
-      <c r="D96" s="109" t="s">
-        <v>20</v>
-      </c>
-      <c r="E96" s="117" t="s">
-        <v>355</v>
-      </c>
-      <c r="F96" s="106" t="s">
-        <v>17</v>
-      </c>
-      <c r="G96" s="107" t="s">
+      <c r="C96" s="3" t="s">
         <v>356</v>
       </c>
-    </row>
-    <row r="97" spans="2:7" ht="66" x14ac:dyDescent="0.3">
+      <c r="D96" s="1">
+        <v>1</v>
+      </c>
+      <c r="E96" s="103" t="s">
+        <v>242</v>
+      </c>
+      <c r="F96" s="103" t="s">
+        <v>243</v>
+      </c>
+      <c r="G96" s="5" t="s">
+        <v>325</v>
+      </c>
+    </row>
+    <row r="97" spans="2:7" ht="33" x14ac:dyDescent="0.3">
       <c r="B97" s="33">
         <f t="shared" si="2"/>
         <v>80</v>
       </c>
       <c r="C97" s="3" t="s">
-        <v>276</v>
+        <v>340</v>
       </c>
       <c r="D97" s="90" t="s">
-        <v>20</v>
+        <v>56</v>
       </c>
       <c r="E97" s="1" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="F97" s="103" t="s">
-        <v>381</v>
+        <v>352</v>
       </c>
       <c r="G97" s="5" t="s">
-        <v>277</v>
-      </c>
-    </row>
-    <row r="98" spans="2:7" x14ac:dyDescent="0.3">
+        <v>341</v>
+      </c>
+    </row>
+    <row r="98" spans="2:7" ht="33" x14ac:dyDescent="0.3">
       <c r="B98" s="33">
         <f t="shared" si="2"/>
         <v>81</v>
       </c>
       <c r="C98" s="3" t="s">
-        <v>317</v>
-      </c>
-      <c r="D98" s="90" t="s">
-        <v>56</v>
-      </c>
-      <c r="E98" s="103" t="s">
-        <v>243</v>
-      </c>
-      <c r="F98" s="2" t="s">
-        <v>64</v>
+        <v>345</v>
+      </c>
+      <c r="D98" s="1">
+        <v>1</v>
+      </c>
+      <c r="E98" s="2" t="s">
+        <v>242</v>
+      </c>
+      <c r="F98" s="103" t="s">
+        <v>346</v>
       </c>
       <c r="G98" s="5" t="s">
-        <v>322</v>
+        <v>308</v>
       </c>
     </row>
     <row r="99" spans="2:7" x14ac:dyDescent="0.3">
@@ -6585,20 +6632,20 @@
         <f t="shared" si="2"/>
         <v>82</v>
       </c>
-      <c r="C99" s="3" t="s">
-        <v>316</v>
-      </c>
-      <c r="D99" s="90" t="s">
-        <v>56</v>
-      </c>
-      <c r="E99" s="103" t="s">
-        <v>243</v>
-      </c>
-      <c r="F99" s="103" t="s">
-        <v>62</v>
-      </c>
-      <c r="G99" s="5" t="s">
-        <v>321</v>
+      <c r="C99" s="104" t="s">
+        <v>371</v>
+      </c>
+      <c r="D99" s="109" t="s">
+        <v>20</v>
+      </c>
+      <c r="E99" s="117" t="s">
+        <v>348</v>
+      </c>
+      <c r="F99" s="106" t="s">
+        <v>17</v>
+      </c>
+      <c r="G99" s="107" t="s">
+        <v>349</v>
       </c>
     </row>
     <row r="100" spans="2:7" x14ac:dyDescent="0.3">
@@ -6607,40 +6654,40 @@
         <v>83</v>
       </c>
       <c r="C100" s="3" t="s">
-        <v>272</v>
-      </c>
-      <c r="D100" s="1">
-        <v>1</v>
-      </c>
-      <c r="E100" s="2" t="s">
-        <v>243</v>
-      </c>
-      <c r="F100" s="2" t="s">
-        <v>81</v>
+        <v>383</v>
+      </c>
+      <c r="D100" s="90" t="s">
+        <v>20</v>
+      </c>
+      <c r="E100" s="1" t="s">
+        <v>242</v>
+      </c>
+      <c r="F100" s="1" t="s">
+        <v>348</v>
       </c>
       <c r="G100" s="5" t="s">
-        <v>275</v>
-      </c>
-    </row>
-    <row r="101" spans="2:7" x14ac:dyDescent="0.3">
+        <v>395</v>
+      </c>
+    </row>
+    <row r="101" spans="2:7" ht="82.5" x14ac:dyDescent="0.3">
       <c r="B101" s="33">
         <f t="shared" si="2"/>
         <v>84</v>
       </c>
       <c r="C101" s="3" t="s">
-        <v>295</v>
+        <v>276</v>
       </c>
       <c r="D101" s="90" t="s">
         <v>20</v>
       </c>
       <c r="E101" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="F101" s="2" t="s">
-        <v>62</v>
+        <v>243</v>
+      </c>
+      <c r="F101" s="103" t="s">
+        <v>392</v>
       </c>
       <c r="G101" s="5" t="s">
-        <v>296</v>
+        <v>277</v>
       </c>
     </row>
     <row r="102" spans="2:7" x14ac:dyDescent="0.3">
@@ -6649,10 +6696,10 @@
         <v>85</v>
       </c>
       <c r="C102" s="3" t="s">
-        <v>365</v>
-      </c>
-      <c r="D102" s="1">
-        <v>1</v>
+        <v>317</v>
+      </c>
+      <c r="D102" s="90" t="s">
+        <v>56</v>
       </c>
       <c r="E102" s="103" t="s">
         <v>243</v>
@@ -6661,37 +6708,37 @@
         <v>64</v>
       </c>
       <c r="G102" s="5" t="s">
-        <v>326</v>
-      </c>
-    </row>
-    <row r="103" spans="2:7" ht="33" x14ac:dyDescent="0.3">
+        <v>322</v>
+      </c>
+    </row>
+    <row r="103" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B103" s="33">
         <f t="shared" si="2"/>
         <v>86</v>
       </c>
       <c r="C103" s="3" t="s">
-        <v>327</v>
+        <v>316</v>
       </c>
       <c r="D103" s="90" t="s">
         <v>56</v>
       </c>
-      <c r="E103" s="1" t="s">
+      <c r="E103" s="103" t="s">
         <v>243</v>
       </c>
       <c r="F103" s="103" t="s">
-        <v>379</v>
+        <v>62</v>
       </c>
       <c r="G103" s="5" t="s">
-        <v>328</v>
-      </c>
-    </row>
-    <row r="104" spans="2:7" ht="33" x14ac:dyDescent="0.3">
+        <v>321</v>
+      </c>
+    </row>
+    <row r="104" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B104" s="33">
         <f t="shared" si="2"/>
         <v>87</v>
       </c>
       <c r="C104" s="3" t="s">
-        <v>306</v>
+        <v>272</v>
       </c>
       <c r="D104" s="1">
         <v>1</v>
@@ -6699,37 +6746,95 @@
       <c r="E104" s="2" t="s">
         <v>243</v>
       </c>
-      <c r="F104" s="103" t="s">
-        <v>379</v>
+      <c r="F104" s="2" t="s">
+        <v>81</v>
       </c>
       <c r="G104" s="5" t="s">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="105" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="B105" s="33">
+        <f t="shared" si="2"/>
+        <v>88</v>
+      </c>
+      <c r="C105" s="3" t="s">
+        <v>295</v>
+      </c>
+      <c r="D105" s="90" t="s">
+        <v>20</v>
+      </c>
+      <c r="E105" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="F105" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="G105" s="5" t="s">
+        <v>296</v>
+      </c>
+    </row>
+    <row r="106" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="B106" s="33">
+        <f t="shared" si="2"/>
+        <v>89</v>
+      </c>
+      <c r="C106" s="3" t="s">
+        <v>357</v>
+      </c>
+      <c r="D106" s="1">
+        <v>1</v>
+      </c>
+      <c r="E106" s="103" t="s">
+        <v>243</v>
+      </c>
+      <c r="F106" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="G106" s="5" t="s">
+        <v>326</v>
+      </c>
+    </row>
+    <row r="107" spans="2:7" ht="33" x14ac:dyDescent="0.3">
+      <c r="B107" s="33">
+        <f t="shared" si="2"/>
+        <v>90</v>
+      </c>
+      <c r="C107" s="3" t="s">
+        <v>327</v>
+      </c>
+      <c r="D107" s="90" t="s">
+        <v>56</v>
+      </c>
+      <c r="E107" s="1" t="s">
+        <v>243</v>
+      </c>
+      <c r="F107" s="103" t="s">
+        <v>362</v>
+      </c>
+      <c r="G107" s="5" t="s">
+        <v>328</v>
+      </c>
+    </row>
+    <row r="108" spans="2:7" ht="33" x14ac:dyDescent="0.3">
+      <c r="B108" s="33">
+        <f t="shared" si="2"/>
+        <v>91</v>
+      </c>
+      <c r="C108" s="3" t="s">
+        <v>306</v>
+      </c>
+      <c r="D108" s="1">
+        <v>1</v>
+      </c>
+      <c r="E108" s="2" t="s">
+        <v>243</v>
+      </c>
+      <c r="F108" s="103" t="s">
+        <v>362</v>
+      </c>
+      <c r="G108" s="5" t="s">
         <v>309</v>
-      </c>
-    </row>
-    <row r="105" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B105" s="33" t="str">
-        <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="E105" s="102"/>
-    </row>
-    <row r="106" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B106" s="33" t="str">
-        <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="E106" s="102"/>
-    </row>
-    <row r="107" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B107" s="33" t="str">
-        <f t="shared" si="2"/>
-        <v/>
-      </c>
-    </row>
-    <row r="108" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B108" s="33" t="str">
-        <f t="shared" si="2"/>
-        <v/>
       </c>
     </row>
     <row r="109" spans="2:7" x14ac:dyDescent="0.3">
@@ -6931,39 +7036,51 @@
     </sortState>
   </autoFilter>
   <mergeCells count="102">
-    <mergeCell ref="K2:M2"/>
-    <mergeCell ref="I18:J18"/>
-    <mergeCell ref="K18:M18"/>
-    <mergeCell ref="I21:J21"/>
-    <mergeCell ref="K21:M21"/>
-    <mergeCell ref="J22:L22"/>
-    <mergeCell ref="I3:J3"/>
-    <mergeCell ref="K3:M3"/>
-    <mergeCell ref="B2:G2"/>
-    <mergeCell ref="J6:L6"/>
-    <mergeCell ref="J7:L7"/>
-    <mergeCell ref="I5:J5"/>
-    <mergeCell ref="K5:M5"/>
-    <mergeCell ref="I2:J2"/>
-    <mergeCell ref="J23:L23"/>
-    <mergeCell ref="I12:J12"/>
-    <mergeCell ref="K12:M12"/>
-    <mergeCell ref="I4:J4"/>
-    <mergeCell ref="K4:M4"/>
-    <mergeCell ref="I20:J20"/>
-    <mergeCell ref="K20:M20"/>
-    <mergeCell ref="I19:J19"/>
-    <mergeCell ref="K19:M19"/>
-    <mergeCell ref="I41:J41"/>
-    <mergeCell ref="K41:M41"/>
-    <mergeCell ref="J42:L42"/>
-    <mergeCell ref="J43:L43"/>
-    <mergeCell ref="I32:J32"/>
-    <mergeCell ref="K32:M32"/>
-    <mergeCell ref="I38:J38"/>
-    <mergeCell ref="K38:M38"/>
-    <mergeCell ref="I39:J39"/>
-    <mergeCell ref="K39:M39"/>
+    <mergeCell ref="P24:R24"/>
+    <mergeCell ref="O38:P38"/>
+    <mergeCell ref="Q38:S38"/>
+    <mergeCell ref="P44:R44"/>
+    <mergeCell ref="O56:P56"/>
+    <mergeCell ref="Q56:S56"/>
+    <mergeCell ref="P62:R62"/>
+    <mergeCell ref="P63:R63"/>
+    <mergeCell ref="P64:R64"/>
+    <mergeCell ref="O72:P72"/>
+    <mergeCell ref="Q72:S72"/>
+    <mergeCell ref="P8:R8"/>
+    <mergeCell ref="O59:P59"/>
+    <mergeCell ref="Q59:S59"/>
+    <mergeCell ref="O60:P60"/>
+    <mergeCell ref="Q60:S60"/>
+    <mergeCell ref="O61:P61"/>
+    <mergeCell ref="Q61:S61"/>
+    <mergeCell ref="P42:R42"/>
+    <mergeCell ref="P43:R43"/>
+    <mergeCell ref="O58:P58"/>
+    <mergeCell ref="Q58:S58"/>
+    <mergeCell ref="O39:P39"/>
+    <mergeCell ref="Q39:S39"/>
+    <mergeCell ref="O40:P40"/>
+    <mergeCell ref="Q40:S40"/>
+    <mergeCell ref="O41:P41"/>
+    <mergeCell ref="Q41:S41"/>
+    <mergeCell ref="P22:R22"/>
+    <mergeCell ref="P23:R23"/>
+    <mergeCell ref="O36:P36"/>
+    <mergeCell ref="Q36:S36"/>
+    <mergeCell ref="O19:P19"/>
+    <mergeCell ref="Q19:S19"/>
+    <mergeCell ref="O20:P20"/>
+    <mergeCell ref="Q20:S20"/>
+    <mergeCell ref="O21:P21"/>
+    <mergeCell ref="Q21:S21"/>
+    <mergeCell ref="Q5:S5"/>
+    <mergeCell ref="P6:R6"/>
+    <mergeCell ref="P7:R7"/>
+    <mergeCell ref="O16:P16"/>
+    <mergeCell ref="Q16:S16"/>
+    <mergeCell ref="O18:P18"/>
+    <mergeCell ref="Q18:S18"/>
     <mergeCell ref="I72:J72"/>
     <mergeCell ref="K72:M72"/>
     <mergeCell ref="J57:L57"/>
@@ -6988,51 +7105,39 @@
     <mergeCell ref="K52:M52"/>
     <mergeCell ref="I40:J40"/>
     <mergeCell ref="K40:M40"/>
-    <mergeCell ref="Q19:S19"/>
-    <mergeCell ref="O20:P20"/>
-    <mergeCell ref="Q20:S20"/>
-    <mergeCell ref="O21:P21"/>
-    <mergeCell ref="Q21:S21"/>
-    <mergeCell ref="Q5:S5"/>
-    <mergeCell ref="P6:R6"/>
-    <mergeCell ref="P7:R7"/>
-    <mergeCell ref="O16:P16"/>
-    <mergeCell ref="Q16:S16"/>
-    <mergeCell ref="O18:P18"/>
-    <mergeCell ref="Q18:S18"/>
-    <mergeCell ref="O72:P72"/>
-    <mergeCell ref="Q72:S72"/>
-    <mergeCell ref="P8:R8"/>
-    <mergeCell ref="O59:P59"/>
-    <mergeCell ref="Q59:S59"/>
-    <mergeCell ref="O60:P60"/>
-    <mergeCell ref="Q60:S60"/>
-    <mergeCell ref="O61:P61"/>
-    <mergeCell ref="Q61:S61"/>
-    <mergeCell ref="P42:R42"/>
-    <mergeCell ref="P43:R43"/>
-    <mergeCell ref="O58:P58"/>
-    <mergeCell ref="Q58:S58"/>
-    <mergeCell ref="O39:P39"/>
-    <mergeCell ref="Q39:S39"/>
-    <mergeCell ref="O40:P40"/>
-    <mergeCell ref="Q40:S40"/>
-    <mergeCell ref="O41:P41"/>
-    <mergeCell ref="Q41:S41"/>
-    <mergeCell ref="P22:R22"/>
-    <mergeCell ref="P23:R23"/>
-    <mergeCell ref="O36:P36"/>
-    <mergeCell ref="Q36:S36"/>
-    <mergeCell ref="O19:P19"/>
-    <mergeCell ref="P24:R24"/>
-    <mergeCell ref="O38:P38"/>
-    <mergeCell ref="Q38:S38"/>
-    <mergeCell ref="P44:R44"/>
-    <mergeCell ref="O56:P56"/>
-    <mergeCell ref="Q56:S56"/>
-    <mergeCell ref="P62:R62"/>
-    <mergeCell ref="P63:R63"/>
-    <mergeCell ref="P64:R64"/>
+    <mergeCell ref="I41:J41"/>
+    <mergeCell ref="K41:M41"/>
+    <mergeCell ref="J42:L42"/>
+    <mergeCell ref="J43:L43"/>
+    <mergeCell ref="I32:J32"/>
+    <mergeCell ref="K32:M32"/>
+    <mergeCell ref="I38:J38"/>
+    <mergeCell ref="K38:M38"/>
+    <mergeCell ref="I39:J39"/>
+    <mergeCell ref="K39:M39"/>
+    <mergeCell ref="J23:L23"/>
+    <mergeCell ref="I12:J12"/>
+    <mergeCell ref="K12:M12"/>
+    <mergeCell ref="I4:J4"/>
+    <mergeCell ref="K4:M4"/>
+    <mergeCell ref="I20:J20"/>
+    <mergeCell ref="K20:M20"/>
+    <mergeCell ref="I19:J19"/>
+    <mergeCell ref="K19:M19"/>
+    <mergeCell ref="K2:M2"/>
+    <mergeCell ref="I18:J18"/>
+    <mergeCell ref="K18:M18"/>
+    <mergeCell ref="I21:J21"/>
+    <mergeCell ref="K21:M21"/>
+    <mergeCell ref="J22:L22"/>
+    <mergeCell ref="I3:J3"/>
+    <mergeCell ref="K3:M3"/>
+    <mergeCell ref="B2:G2"/>
+    <mergeCell ref="J6:L6"/>
+    <mergeCell ref="J7:L7"/>
+    <mergeCell ref="I5:J5"/>
+    <mergeCell ref="K5:M5"/>
+    <mergeCell ref="I2:J2"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
IDD Update for Load Stall
</commit_message>
<xml_diff>
--- a/Document/IDD.xlsx
+++ b/Document/IDD.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="V:\SoC_Design\Document\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC991E40-4640-4764-8153-C0DB49EDCA9B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E47090BE-DFE7-4CE4-9182-D31A5AA789FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{813C5046-60F0-40FF-AAC7-48B46C31F73B}"/>
+    <workbookView xWindow="17235" yWindow="0" windowWidth="11670" windowHeight="15585" xr2:uid="{813C5046-60F0-40FF-AAC7-48B46C31F73B}"/>
   </bookViews>
   <sheets>
     <sheet name="CPU" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="863" uniqueCount="402">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="844" uniqueCount="395">
   <si>
     <t>top_cpu</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -1269,18 +1269,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>w_mem_dec_rd</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>w_wb_dec_rt</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>w_wb_dec_rd</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>Decoded rd Register (EX)</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -1289,31 +1277,11 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>Decoded rd Register (MEM)</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Decoded rt Register (WB)</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Decoded rd Register (WB)</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>w_ex_ctr_regdst</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>RegDst Flag (EX)</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>RegDst Flag (MEM)</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>RegDst Flag (WB)</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
@@ -1367,11 +1335,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>u_registers
-u_id_ex_bridge</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>w_mem_regdst_mux_reg</t>
   </si>
   <si>
@@ -1422,11 +1385,6 @@
   <si>
     <t>u_alu_forwarding_unit
 u_mem_wb_bridge</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>u_ex_mem_bridge
-u_regdst_mux</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
@@ -1437,14 +1395,6 @@
   </si>
   <si>
     <t>w_id_regdst</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>w_mem_regdst</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>w_wb_regdst</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
@@ -1552,11 +1502,6 @@
   </si>
   <si>
     <t>u_alu_forward_b_mux</t>
-  </si>
-  <si>
-    <t>u_mem_wb_bridge
-u_wdata_forwarding_unit</t>
-    <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>u_wdata_forward_2cycle_mux</t>
@@ -1643,11 +1588,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>u_pc_mux
-u_id_ex_bridge</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>w_id_pc_addr</t>
   </si>
   <si>
@@ -1674,6 +1614,40 @@
   </si>
   <si>
     <t>w_ex_flush</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>u_ex_mem_bridge
+u_load_stall_unit</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>u_registers
+u_id_ex_bridge
+u_load_stall_unit</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>w_load_stall</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>u_load_stall_unit</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Load Stall Flag Signal</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>u_if_id_bridge
+u_id_ex_bridge</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>u_pc_mux
+u_if_id_bridge
+u_id_ex_bridge</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -2657,16 +2631,58 @@
     <xf numFmtId="3" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="6" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="6" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2684,52 +2700,10 @@
     <xf numFmtId="0" fontId="0" fillId="6" borderId="28" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="6" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -3092,31 +3066,31 @@
   <sheetData>
     <row r="1" spans="2:19" ht="17.25" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="2" spans="2:19" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B2" s="141" t="s">
-        <v>0</v>
-      </c>
-      <c r="C2" s="142"/>
-      <c r="D2" s="142"/>
-      <c r="E2" s="142"/>
-      <c r="F2" s="142"/>
-      <c r="G2" s="143"/>
-      <c r="I2" s="120" t="s">
+      <c r="B2" s="133" t="s">
+        <v>0</v>
+      </c>
+      <c r="C2" s="134"/>
+      <c r="D2" s="134"/>
+      <c r="E2" s="134"/>
+      <c r="F2" s="134"/>
+      <c r="G2" s="135"/>
+      <c r="I2" s="119" t="s">
         <v>102</v>
       </c>
       <c r="J2" s="121"/>
-      <c r="K2" s="120" t="s">
+      <c r="K2" s="119" t="s">
         <v>96</v>
       </c>
-      <c r="L2" s="122"/>
+      <c r="L2" s="120"/>
       <c r="M2" s="121"/>
-      <c r="O2" s="120" t="s">
+      <c r="O2" s="119" t="s">
         <v>102</v>
       </c>
       <c r="P2" s="121"/>
-      <c r="Q2" s="120" t="s">
+      <c r="Q2" s="119" t="s">
         <v>149</v>
       </c>
-      <c r="R2" s="122"/>
+      <c r="R2" s="120"/>
       <c r="S2" s="121"/>
     </row>
     <row r="3" spans="2:19" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
@@ -3138,24 +3112,24 @@
       <c r="G3" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="I3" s="130" t="s">
+      <c r="I3" s="128" t="s">
         <v>108</v>
       </c>
-      <c r="J3" s="131"/>
-      <c r="K3" s="132" t="s">
+      <c r="J3" s="129"/>
+      <c r="K3" s="130" t="s">
         <v>109</v>
       </c>
-      <c r="L3" s="133"/>
-      <c r="M3" s="134"/>
-      <c r="O3" s="130" t="s">
+      <c r="L3" s="131"/>
+      <c r="M3" s="132"/>
+      <c r="O3" s="128" t="s">
         <v>108</v>
       </c>
-      <c r="P3" s="131"/>
-      <c r="Q3" s="132" t="s">
+      <c r="P3" s="129"/>
+      <c r="Q3" s="130" t="s">
         <v>233</v>
       </c>
-      <c r="R3" s="133"/>
-      <c r="S3" s="134"/>
+      <c r="R3" s="131"/>
+      <c r="S3" s="132"/>
     </row>
     <row r="4" spans="2:19" x14ac:dyDescent="0.3">
       <c r="B4" s="35">
@@ -3176,24 +3150,24 @@
       <c r="G4" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="I4" s="130" t="s">
+      <c r="I4" s="128" t="s">
         <v>106</v>
       </c>
-      <c r="J4" s="131"/>
-      <c r="K4" s="130" t="s">
+      <c r="J4" s="129"/>
+      <c r="K4" s="128" t="s">
         <v>64</v>
       </c>
-      <c r="L4" s="135"/>
-      <c r="M4" s="131"/>
-      <c r="O4" s="130" t="s">
+      <c r="L4" s="142"/>
+      <c r="M4" s="129"/>
+      <c r="O4" s="128" t="s">
         <v>106</v>
       </c>
-      <c r="P4" s="131"/>
-      <c r="Q4" s="130" t="s">
+      <c r="P4" s="129"/>
+      <c r="Q4" s="128" t="s">
         <v>64</v>
       </c>
-      <c r="R4" s="135"/>
-      <c r="S4" s="131"/>
+      <c r="R4" s="142"/>
+      <c r="S4" s="129"/>
     </row>
     <row r="5" spans="2:19" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B5" s="54">
@@ -3214,24 +3188,24 @@
       <c r="G5" s="14" t="s">
         <v>9</v>
       </c>
-      <c r="I5" s="136" t="s">
+      <c r="I5" s="122" t="s">
         <v>8</v>
       </c>
-      <c r="J5" s="137"/>
-      <c r="K5" s="138" t="s">
+      <c r="J5" s="123"/>
+      <c r="K5" s="124" t="s">
         <v>101</v>
       </c>
-      <c r="L5" s="119"/>
-      <c r="M5" s="139"/>
-      <c r="O5" s="136" t="s">
+      <c r="L5" s="125"/>
+      <c r="M5" s="126"/>
+      <c r="O5" s="122" t="s">
         <v>8</v>
       </c>
-      <c r="P5" s="137"/>
-      <c r="Q5" s="138" t="s">
+      <c r="P5" s="123"/>
+      <c r="Q5" s="124" t="s">
         <v>150</v>
       </c>
-      <c r="R5" s="119"/>
-      <c r="S5" s="139"/>
+      <c r="R5" s="125"/>
+      <c r="S5" s="126"/>
     </row>
     <row r="6" spans="2:19" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B6" s="55">
@@ -3255,22 +3229,22 @@
       <c r="I6" s="67" t="s">
         <v>41</v>
       </c>
-      <c r="J6" s="128" t="s">
+      <c r="J6" s="127" t="s">
         <v>97</v>
       </c>
-      <c r="K6" s="128"/>
-      <c r="L6" s="128"/>
+      <c r="K6" s="127"/>
+      <c r="L6" s="127"/>
       <c r="M6" s="69" t="s">
         <v>8</v>
       </c>
       <c r="O6" s="67" t="s">
         <v>41</v>
       </c>
-      <c r="P6" s="128" t="s">
+      <c r="P6" s="127" t="s">
         <v>97</v>
       </c>
-      <c r="Q6" s="128"/>
-      <c r="R6" s="128"/>
+      <c r="Q6" s="127"/>
+      <c r="R6" s="127"/>
       <c r="S6" s="69" t="s">
         <v>8</v>
       </c>
@@ -3297,22 +3271,22 @@
       <c r="I7" s="70">
         <v>1</v>
       </c>
-      <c r="J7" s="140" t="s">
+      <c r="J7" s="136" t="s">
         <v>21</v>
       </c>
-      <c r="K7" s="140"/>
-      <c r="L7" s="140"/>
+      <c r="K7" s="136"/>
+      <c r="L7" s="136"/>
       <c r="M7" s="71" t="s">
         <v>132</v>
       </c>
       <c r="O7" s="87">
         <v>1</v>
       </c>
-      <c r="P7" s="129" t="s">
+      <c r="P7" s="143" t="s">
         <v>21</v>
       </c>
-      <c r="Q7" s="129"/>
-      <c r="R7" s="129"/>
+      <c r="Q7" s="143"/>
+      <c r="R7" s="143"/>
       <c r="S7" s="88" t="s">
         <v>132</v>
       </c>
@@ -3354,11 +3328,11 @@
       <c r="O8" s="80">
         <v>2</v>
       </c>
-      <c r="P8" s="119" t="s">
+      <c r="P8" s="125" t="s">
         <v>20</v>
       </c>
-      <c r="Q8" s="119"/>
-      <c r="R8" s="119"/>
+      <c r="Q8" s="125"/>
+      <c r="R8" s="125"/>
       <c r="S8" s="82" t="s">
         <v>133</v>
       </c>
@@ -3532,15 +3506,15 @@
       <c r="G12" s="30" t="s">
         <v>29</v>
       </c>
-      <c r="I12" s="123" t="s">
+      <c r="I12" s="137" t="s">
         <v>104</v>
       </c>
-      <c r="J12" s="124"/>
-      <c r="K12" s="125" t="s">
+      <c r="J12" s="138"/>
+      <c r="K12" s="139" t="s">
         <v>105</v>
       </c>
-      <c r="L12" s="126"/>
-      <c r="M12" s="127"/>
+      <c r="L12" s="140"/>
+      <c r="M12" s="141"/>
       <c r="O12" s="72">
         <v>3</v>
       </c>
@@ -3663,15 +3637,15 @@
       </c>
     </row>
     <row r="16" spans="2:19" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="O16" s="123" t="s">
+      <c r="O16" s="137" t="s">
         <v>104</v>
       </c>
-      <c r="P16" s="124"/>
-      <c r="Q16" s="125" t="s">
+      <c r="P16" s="138"/>
+      <c r="Q16" s="139" t="s">
         <v>236</v>
       </c>
-      <c r="R16" s="126"/>
-      <c r="S16" s="127"/>
+      <c r="R16" s="140"/>
+      <c r="S16" s="141"/>
     </row>
     <row r="17" spans="2:19" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B17" s="90" t="s">
@@ -3693,83 +3667,83 @@
         <v>8</v>
       </c>
     </row>
-    <row r="18" spans="2:19" ht="33" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:19" x14ac:dyDescent="0.3">
       <c r="B18" s="33">
         <f>IF(C18="","",1)</f>
         <v>1</v>
       </c>
       <c r="C18" s="3" t="s">
-        <v>398</v>
-      </c>
-      <c r="D18" s="90" t="s">
-        <v>21</v>
-      </c>
-      <c r="E18" s="2" t="s">
-        <v>234</v>
-      </c>
-      <c r="F18" s="103" t="s">
-        <v>255</v>
-      </c>
-      <c r="G18" s="99" t="s">
-        <v>195</v>
-      </c>
-      <c r="I18" s="120" t="s">
+        <v>292</v>
+      </c>
+      <c r="D18" s="1">
+        <v>1</v>
+      </c>
+      <c r="E18" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="F18" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="G18" s="5" t="s">
+        <v>83</v>
+      </c>
+      <c r="I18" s="119" t="s">
         <v>102</v>
       </c>
       <c r="J18" s="121"/>
-      <c r="K18" s="120" t="s">
+      <c r="K18" s="119" t="s">
         <v>103</v>
       </c>
-      <c r="L18" s="122"/>
+      <c r="L18" s="120"/>
       <c r="M18" s="121"/>
-      <c r="O18" s="120" t="s">
+      <c r="O18" s="119" t="s">
         <v>102</v>
       </c>
       <c r="P18" s="121"/>
-      <c r="Q18" s="120" t="s">
+      <c r="Q18" s="119" t="s">
         <v>159</v>
       </c>
-      <c r="R18" s="122"/>
+      <c r="R18" s="120"/>
       <c r="S18" s="121"/>
     </row>
-    <row r="19" spans="2:19" x14ac:dyDescent="0.3">
+    <row r="19" spans="2:19" ht="33" x14ac:dyDescent="0.3">
       <c r="B19" s="33">
         <f t="shared" ref="B19:B50" si="0">IF(C19="","",B18+1)</f>
         <v>2</v>
       </c>
       <c r="C19" s="3" t="s">
-        <v>292</v>
+        <v>288</v>
       </c>
       <c r="D19" s="1">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E19" s="1" t="s">
-        <v>78</v>
-      </c>
-      <c r="F19" s="2" t="s">
-        <v>64</v>
+        <v>74</v>
+      </c>
+      <c r="F19" s="103" t="s">
+        <v>75</v>
       </c>
       <c r="G19" s="5" t="s">
-        <v>83</v>
-      </c>
-      <c r="I19" s="130" t="s">
+        <v>76</v>
+      </c>
+      <c r="I19" s="128" t="s">
         <v>108</v>
       </c>
-      <c r="J19" s="131"/>
-      <c r="K19" s="132" t="s">
+      <c r="J19" s="129"/>
+      <c r="K19" s="130" t="s">
         <v>110</v>
       </c>
-      <c r="L19" s="133"/>
-      <c r="M19" s="134"/>
-      <c r="O19" s="130" t="s">
+      <c r="L19" s="131"/>
+      <c r="M19" s="132"/>
+      <c r="O19" s="128" t="s">
         <v>108</v>
       </c>
-      <c r="P19" s="131"/>
-      <c r="Q19" s="132" t="s">
+      <c r="P19" s="129"/>
+      <c r="Q19" s="130" t="s">
         <v>233</v>
       </c>
-      <c r="R19" s="133"/>
-      <c r="S19" s="134"/>
+      <c r="R19" s="131"/>
+      <c r="S19" s="132"/>
     </row>
     <row r="20" spans="2:19" ht="33" x14ac:dyDescent="0.3">
       <c r="B20" s="33">
@@ -3777,160 +3751,160 @@
         <v>3</v>
       </c>
       <c r="C20" s="3" t="s">
-        <v>288</v>
-      </c>
-      <c r="D20" s="1">
-        <v>4</v>
+        <v>354</v>
+      </c>
+      <c r="D20" s="90" t="s">
+        <v>20</v>
       </c>
       <c r="E20" s="1" t="s">
-        <v>74</v>
+        <v>340</v>
       </c>
       <c r="F20" s="103" t="s">
         <v>75</v>
       </c>
       <c r="G20" s="5" t="s">
-        <v>76</v>
-      </c>
-      <c r="I20" s="130" t="s">
+        <v>355</v>
+      </c>
+      <c r="I20" s="128" t="s">
         <v>106</v>
       </c>
-      <c r="J20" s="131"/>
-      <c r="K20" s="132" t="s">
+      <c r="J20" s="129"/>
+      <c r="K20" s="130" t="s">
         <v>107</v>
       </c>
-      <c r="L20" s="133"/>
-      <c r="M20" s="134"/>
-      <c r="O20" s="130" t="s">
+      <c r="L20" s="131"/>
+      <c r="M20" s="132"/>
+      <c r="O20" s="128" t="s">
         <v>106</v>
       </c>
-      <c r="P20" s="131"/>
-      <c r="Q20" s="130" t="s">
+      <c r="P20" s="129"/>
+      <c r="Q20" s="128" t="s">
         <v>64</v>
       </c>
-      <c r="R20" s="135"/>
-      <c r="S20" s="131"/>
-    </row>
-    <row r="21" spans="2:19" ht="33.75" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="R20" s="142"/>
+      <c r="S20" s="129"/>
+    </row>
+    <row r="21" spans="2:19" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B21" s="33">
         <f t="shared" si="0"/>
         <v>4</v>
       </c>
       <c r="C21" s="3" t="s">
-        <v>366</v>
+        <v>356</v>
       </c>
       <c r="D21" s="90" t="s">
         <v>20</v>
       </c>
       <c r="E21" s="1" t="s">
-        <v>352</v>
+        <v>341</v>
       </c>
       <c r="F21" s="103" t="s">
-        <v>75</v>
+        <v>332</v>
       </c>
       <c r="G21" s="5" t="s">
-        <v>367</v>
-      </c>
-      <c r="I21" s="136" t="s">
+        <v>357</v>
+      </c>
+      <c r="I21" s="122" t="s">
         <v>8</v>
       </c>
-      <c r="J21" s="137"/>
-      <c r="K21" s="138" t="s">
+      <c r="J21" s="123"/>
+      <c r="K21" s="124" t="s">
         <v>124</v>
       </c>
-      <c r="L21" s="119"/>
-      <c r="M21" s="139"/>
-      <c r="O21" s="136" t="s">
+      <c r="L21" s="125"/>
+      <c r="M21" s="126"/>
+      <c r="O21" s="122" t="s">
         <v>8</v>
       </c>
-      <c r="P21" s="137"/>
-      <c r="Q21" s="138" t="s">
+      <c r="P21" s="123"/>
+      <c r="Q21" s="124" t="s">
         <v>160</v>
       </c>
-      <c r="R21" s="119"/>
-      <c r="S21" s="139"/>
-    </row>
-    <row r="22" spans="2:19" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="R21" s="125"/>
+      <c r="S21" s="126"/>
+    </row>
+    <row r="22" spans="2:19" ht="33.75" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B22" s="33">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
       <c r="C22" s="3" t="s">
-        <v>368</v>
+        <v>257</v>
       </c>
       <c r="D22" s="90" t="s">
         <v>20</v>
       </c>
       <c r="E22" s="1" t="s">
-        <v>353</v>
+        <v>78</v>
       </c>
       <c r="F22" s="103" t="s">
-        <v>341</v>
+        <v>370</v>
       </c>
       <c r="G22" s="5" t="s">
-        <v>369</v>
+        <v>258</v>
       </c>
       <c r="I22" s="67" t="s">
         <v>41</v>
       </c>
-      <c r="J22" s="128" t="s">
+      <c r="J22" s="127" t="s">
         <v>97</v>
       </c>
-      <c r="K22" s="128"/>
-      <c r="L22" s="128"/>
+      <c r="K22" s="127"/>
+      <c r="L22" s="127"/>
       <c r="M22" s="69" t="s">
         <v>8</v>
       </c>
       <c r="O22" s="67" t="s">
         <v>41</v>
       </c>
-      <c r="P22" s="128" t="s">
+      <c r="P22" s="127" t="s">
         <v>97</v>
       </c>
-      <c r="Q22" s="128"/>
-      <c r="R22" s="128"/>
+      <c r="Q22" s="127"/>
+      <c r="R22" s="127"/>
       <c r="S22" s="69" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="23" spans="2:19" ht="33.75" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="23" spans="2:19" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B23" s="33">
         <f t="shared" si="0"/>
         <v>6</v>
       </c>
       <c r="C23" s="3" t="s">
-        <v>257</v>
-      </c>
-      <c r="D23" s="90" t="s">
-        <v>20</v>
+        <v>293</v>
+      </c>
+      <c r="D23" s="1">
+        <v>1</v>
       </c>
       <c r="E23" s="1" t="s">
         <v>78</v>
       </c>
-      <c r="F23" s="103" t="s">
-        <v>383</v>
+      <c r="F23" s="2" t="s">
+        <v>298</v>
       </c>
       <c r="G23" s="5" t="s">
-        <v>258</v>
+        <v>84</v>
       </c>
       <c r="I23" s="70">
         <v>1</v>
       </c>
-      <c r="J23" s="140" t="s">
+      <c r="J23" s="136" t="s">
         <v>20</v>
       </c>
-      <c r="K23" s="140"/>
-      <c r="L23" s="140"/>
+      <c r="K23" s="136"/>
+      <c r="L23" s="136"/>
       <c r="M23" s="71" t="s">
         <v>133</v>
       </c>
       <c r="O23" s="87">
         <v>1</v>
       </c>
-      <c r="P23" s="129" t="s">
+      <c r="P23" s="143" t="s">
         <v>21</v>
       </c>
-      <c r="Q23" s="129"/>
-      <c r="R23" s="129"/>
+      <c r="Q23" s="143"/>
+      <c r="R23" s="143"/>
       <c r="S23" s="88" t="s">
         <v>132</v>
       </c>
@@ -3941,19 +3915,19 @@
         <v>7</v>
       </c>
       <c r="C24" s="3" t="s">
-        <v>293</v>
+        <v>244</v>
       </c>
       <c r="D24" s="1">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E24" s="1" t="s">
-        <v>78</v>
+        <v>237</v>
       </c>
       <c r="F24" s="2" t="s">
-        <v>298</v>
+        <v>65</v>
       </c>
       <c r="G24" s="5" t="s">
-        <v>84</v>
+        <v>245</v>
       </c>
       <c r="I24" s="67" t="s">
         <v>41</v>
@@ -3973,34 +3947,34 @@
       <c r="O24" s="80">
         <v>2</v>
       </c>
-      <c r="P24" s="119" t="s">
+      <c r="P24" s="125" t="s">
         <v>20</v>
       </c>
-      <c r="Q24" s="119"/>
-      <c r="R24" s="119"/>
+      <c r="Q24" s="125"/>
+      <c r="R24" s="125"/>
       <c r="S24" s="82" t="s">
         <v>133</v>
       </c>
     </row>
-    <row r="25" spans="2:19" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="25" spans="2:19" ht="33.75" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B25" s="33">
         <f t="shared" si="0"/>
         <v>8</v>
       </c>
       <c r="C25" s="3" t="s">
-        <v>244</v>
-      </c>
-      <c r="D25" s="1">
-        <v>3</v>
+        <v>291</v>
+      </c>
+      <c r="D25" s="90" t="s">
+        <v>20</v>
       </c>
       <c r="E25" s="1" t="s">
-        <v>237</v>
-      </c>
-      <c r="F25" s="2" t="s">
-        <v>65</v>
+        <v>79</v>
+      </c>
+      <c r="F25" s="103" t="s">
+        <v>75</v>
       </c>
       <c r="G25" s="5" t="s">
-        <v>245</v>
+        <v>81</v>
       </c>
       <c r="I25" s="72">
         <v>1</v>
@@ -4033,25 +4007,25 @@
         <v>8</v>
       </c>
     </row>
-    <row r="26" spans="2:19" ht="33" x14ac:dyDescent="0.3">
+    <row r="26" spans="2:19" x14ac:dyDescent="0.3">
       <c r="B26" s="33">
         <f t="shared" si="0"/>
         <v>9</v>
       </c>
       <c r="C26" s="3" t="s">
-        <v>291</v>
-      </c>
-      <c r="D26" s="90" t="s">
-        <v>20</v>
-      </c>
-      <c r="E26" s="1" t="s">
-        <v>79</v>
-      </c>
-      <c r="F26" s="103" t="s">
-        <v>75</v>
+        <v>262</v>
+      </c>
+      <c r="D26" s="1">
+        <v>2</v>
+      </c>
+      <c r="E26" s="2" t="s">
+        <v>237</v>
+      </c>
+      <c r="F26" s="2" t="s">
+        <v>298</v>
       </c>
       <c r="G26" s="5" t="s">
-        <v>81</v>
+        <v>263</v>
       </c>
       <c r="I26" s="76">
         <v>2</v>
@@ -4090,19 +4064,19 @@
         <v>10</v>
       </c>
       <c r="C27" s="3" t="s">
-        <v>262</v>
-      </c>
-      <c r="D27" s="1">
-        <v>2</v>
-      </c>
-      <c r="E27" s="2" t="s">
-        <v>237</v>
+        <v>281</v>
+      </c>
+      <c r="D27" s="90" t="s">
+        <v>20</v>
+      </c>
+      <c r="E27" s="1" t="s">
+        <v>40</v>
       </c>
       <c r="F27" s="2" t="s">
-        <v>298</v>
+        <v>53</v>
       </c>
       <c r="G27" s="5" t="s">
-        <v>263</v>
+        <v>232</v>
       </c>
       <c r="I27" s="83">
         <v>3</v>
@@ -4141,19 +4115,19 @@
         <v>11</v>
       </c>
       <c r="C28" s="3" t="s">
-        <v>281</v>
+        <v>296</v>
       </c>
       <c r="D28" s="90" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="E28" s="1" t="s">
-        <v>40</v>
+        <v>53</v>
       </c>
       <c r="F28" s="2" t="s">
-        <v>53</v>
+        <v>36</v>
       </c>
       <c r="G28" s="5" t="s">
-        <v>232</v>
+        <v>88</v>
       </c>
       <c r="I28" s="83">
         <v>4</v>
@@ -4192,19 +4166,19 @@
         <v>12</v>
       </c>
       <c r="C29" s="3" t="s">
-        <v>296</v>
-      </c>
-      <c r="D29" s="90" t="s">
-        <v>21</v>
+        <v>226</v>
+      </c>
+      <c r="D29" s="1">
+        <v>1</v>
       </c>
       <c r="E29" s="1" t="s">
-        <v>53</v>
+        <v>234</v>
       </c>
       <c r="F29" s="2" t="s">
-        <v>36</v>
+        <v>79</v>
       </c>
       <c r="G29" s="5" t="s">
-        <v>88</v>
+        <v>227</v>
       </c>
       <c r="I29" s="83">
         <v>5</v>
@@ -4237,25 +4211,25 @@
         <v>168</v>
       </c>
     </row>
-    <row r="30" spans="2:19" x14ac:dyDescent="0.3">
+    <row r="30" spans="2:19" ht="33" x14ac:dyDescent="0.3">
       <c r="B30" s="33">
         <f t="shared" si="0"/>
         <v>13</v>
       </c>
       <c r="C30" s="3" t="s">
-        <v>226</v>
+        <v>298</v>
       </c>
       <c r="D30" s="1">
         <v>1</v>
       </c>
-      <c r="E30" s="1" t="s">
-        <v>234</v>
-      </c>
-      <c r="F30" s="2" t="s">
-        <v>79</v>
+      <c r="E30" s="102" t="s">
+        <v>297</v>
+      </c>
+      <c r="F30" s="103" t="s">
+        <v>385</v>
       </c>
       <c r="G30" s="5" t="s">
-        <v>227</v>
+        <v>89</v>
       </c>
       <c r="I30" s="83">
         <v>6</v>
@@ -4294,19 +4268,19 @@
         <v>14</v>
       </c>
       <c r="C31" s="3" t="s">
-        <v>298</v>
+        <v>264</v>
       </c>
       <c r="D31" s="1">
         <v>1</v>
       </c>
-      <c r="E31" s="102" t="s">
-        <v>297</v>
+      <c r="E31" s="2" t="s">
+        <v>237</v>
       </c>
       <c r="F31" s="103" t="s">
-        <v>399</v>
+        <v>386</v>
       </c>
       <c r="G31" s="5" t="s">
-        <v>89</v>
+        <v>265</v>
       </c>
       <c r="I31" s="80">
         <v>7</v>
@@ -4339,35 +4313,35 @@
         <v>169</v>
       </c>
     </row>
-    <row r="32" spans="2:19" ht="33.75" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="32" spans="2:19" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B32" s="33">
         <f t="shared" si="0"/>
         <v>15</v>
       </c>
       <c r="C32" s="3" t="s">
-        <v>264</v>
+        <v>311</v>
       </c>
       <c r="D32" s="1">
         <v>1</v>
       </c>
-      <c r="E32" s="2" t="s">
+      <c r="E32" s="1" t="s">
         <v>237</v>
       </c>
       <c r="F32" s="103" t="s">
-        <v>400</v>
+        <v>63</v>
       </c>
       <c r="G32" s="5" t="s">
-        <v>265</v>
-      </c>
-      <c r="I32" s="123" t="s">
+        <v>312</v>
+      </c>
+      <c r="I32" s="137" t="s">
         <v>104</v>
       </c>
-      <c r="J32" s="124"/>
-      <c r="K32" s="125" t="s">
+      <c r="J32" s="138"/>
+      <c r="K32" s="139" t="s">
         <v>78</v>
       </c>
-      <c r="L32" s="126"/>
-      <c r="M32" s="127"/>
+      <c r="L32" s="140"/>
+      <c r="M32" s="141"/>
       <c r="O32" s="83">
         <v>7</v>
       </c>
@@ -4384,25 +4358,25 @@
         <v>167</v>
       </c>
     </row>
-    <row r="33" spans="2:19" ht="33" x14ac:dyDescent="0.3">
+    <row r="33" spans="2:19" x14ac:dyDescent="0.3">
       <c r="B33" s="33">
         <f t="shared" si="0"/>
         <v>16</v>
       </c>
       <c r="C33" s="3" t="s">
-        <v>317</v>
+        <v>242</v>
       </c>
       <c r="D33" s="1">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="E33" s="1" t="s">
-        <v>237</v>
-      </c>
-      <c r="F33" s="103" t="s">
-        <v>347</v>
+        <v>234</v>
+      </c>
+      <c r="F33" s="2" t="s">
+        <v>65</v>
       </c>
       <c r="G33" s="5" t="s">
-        <v>318</v>
+        <v>243</v>
       </c>
       <c r="O33" s="83">
         <v>8</v>
@@ -4426,19 +4400,19 @@
         <v>17</v>
       </c>
       <c r="C34" s="3" t="s">
-        <v>242</v>
-      </c>
-      <c r="D34" s="1">
-        <v>6</v>
+        <v>307</v>
+      </c>
+      <c r="D34" s="90" t="s">
+        <v>56</v>
       </c>
       <c r="E34" s="1" t="s">
-        <v>234</v>
-      </c>
-      <c r="F34" s="2" t="s">
-        <v>65</v>
+        <v>237</v>
+      </c>
+      <c r="F34" s="103" t="s">
+        <v>63</v>
       </c>
       <c r="G34" s="5" t="s">
-        <v>243</v>
+        <v>309</v>
       </c>
       <c r="O34" s="83">
         <v>9</v>
@@ -4456,13 +4430,13 @@
         <v>171</v>
       </c>
     </row>
-    <row r="35" spans="2:19" ht="33.75" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="35" spans="2:19" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B35" s="33">
         <f t="shared" si="0"/>
         <v>18</v>
       </c>
       <c r="C35" s="3" t="s">
-        <v>307</v>
+        <v>322</v>
       </c>
       <c r="D35" s="90" t="s">
         <v>56</v>
@@ -4471,10 +4445,10 @@
         <v>237</v>
       </c>
       <c r="F35" s="103" t="s">
-        <v>347</v>
+        <v>343</v>
       </c>
       <c r="G35" s="5" t="s">
-        <v>312</v>
+        <v>323</v>
       </c>
       <c r="O35" s="80">
         <v>10</v>
@@ -4492,13 +4466,13 @@
         <v>172</v>
       </c>
     </row>
-    <row r="36" spans="2:19" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="36" spans="2:19" ht="50.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B36" s="33">
         <f t="shared" si="0"/>
         <v>19</v>
       </c>
       <c r="C36" s="3" t="s">
-        <v>330</v>
+        <v>306</v>
       </c>
       <c r="D36" s="90" t="s">
         <v>56</v>
@@ -4507,20 +4481,20 @@
         <v>237</v>
       </c>
       <c r="F36" s="103" t="s">
-        <v>355</v>
+        <v>338</v>
       </c>
       <c r="G36" s="5" t="s">
-        <v>331</v>
-      </c>
-      <c r="O36" s="123" t="s">
+        <v>305</v>
+      </c>
+      <c r="O36" s="137" t="s">
         <v>104</v>
       </c>
-      <c r="P36" s="124"/>
-      <c r="Q36" s="125" t="s">
+      <c r="P36" s="138"/>
+      <c r="Q36" s="139" t="s">
         <v>237</v>
       </c>
-      <c r="R36" s="126"/>
-      <c r="S36" s="127"/>
+      <c r="R36" s="140"/>
+      <c r="S36" s="141"/>
     </row>
     <row r="37" spans="2:19" ht="50.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B37" s="33">
@@ -4528,19 +4502,19 @@
         <v>20</v>
       </c>
       <c r="C37" s="3" t="s">
-        <v>306</v>
-      </c>
-      <c r="D37" s="90" t="s">
-        <v>56</v>
-      </c>
-      <c r="E37" s="1" t="s">
-        <v>237</v>
+        <v>387</v>
+      </c>
+      <c r="D37" s="1">
+        <v>1</v>
+      </c>
+      <c r="E37" s="102" t="s">
+        <v>379</v>
       </c>
       <c r="F37" s="103" t="s">
-        <v>348</v>
+        <v>394</v>
       </c>
       <c r="G37" s="5" t="s">
-        <v>305</v>
+        <v>380</v>
       </c>
     </row>
     <row r="38" spans="2:19" ht="33" x14ac:dyDescent="0.3">
@@ -4549,37 +4523,37 @@
         <v>21</v>
       </c>
       <c r="C38" s="3" t="s">
-        <v>357</v>
+        <v>345</v>
       </c>
       <c r="D38" s="1">
         <v>1</v>
       </c>
       <c r="E38" s="102" t="s">
-        <v>358</v>
+        <v>346</v>
       </c>
       <c r="F38" s="103" t="s">
-        <v>384</v>
+        <v>371</v>
       </c>
       <c r="G38" s="5" t="s">
-        <v>375</v>
-      </c>
-      <c r="I38" s="120" t="s">
+        <v>363</v>
+      </c>
+      <c r="I38" s="119" t="s">
         <v>102</v>
       </c>
       <c r="J38" s="121"/>
-      <c r="K38" s="120" t="s">
+      <c r="K38" s="119" t="s">
         <v>122</v>
       </c>
-      <c r="L38" s="122"/>
+      <c r="L38" s="120"/>
       <c r="M38" s="121"/>
-      <c r="O38" s="120" t="s">
+      <c r="O38" s="119" t="s">
         <v>102</v>
       </c>
       <c r="P38" s="121"/>
-      <c r="Q38" s="120" t="s">
+      <c r="Q38" s="119" t="s">
         <v>173</v>
       </c>
-      <c r="R38" s="122"/>
+      <c r="R38" s="120"/>
       <c r="S38" s="121"/>
     </row>
     <row r="39" spans="2:19" x14ac:dyDescent="0.3">
@@ -4602,24 +4576,24 @@
       <c r="G39" s="5" t="s">
         <v>86</v>
       </c>
-      <c r="I39" s="130" t="s">
+      <c r="I39" s="128" t="s">
         <v>108</v>
       </c>
-      <c r="J39" s="131"/>
-      <c r="K39" s="132" t="s">
+      <c r="J39" s="129"/>
+      <c r="K39" s="130" t="s">
         <v>123</v>
       </c>
-      <c r="L39" s="133"/>
-      <c r="M39" s="134"/>
-      <c r="O39" s="130" t="s">
+      <c r="L39" s="131"/>
+      <c r="M39" s="132"/>
+      <c r="O39" s="128" t="s">
         <v>108</v>
       </c>
-      <c r="P39" s="131"/>
-      <c r="Q39" s="132" t="s">
+      <c r="P39" s="129"/>
+      <c r="Q39" s="130" t="s">
         <v>233</v>
       </c>
-      <c r="R39" s="133"/>
-      <c r="S39" s="134"/>
+      <c r="R39" s="131"/>
+      <c r="S39" s="132"/>
     </row>
     <row r="40" spans="2:19" x14ac:dyDescent="0.3">
       <c r="B40" s="33">
@@ -4641,24 +4615,24 @@
       <c r="G40" s="5" t="s">
         <v>231</v>
       </c>
-      <c r="I40" s="130" t="s">
+      <c r="I40" s="128" t="s">
         <v>106</v>
       </c>
-      <c r="J40" s="131"/>
-      <c r="K40" s="132" t="s">
+      <c r="J40" s="129"/>
+      <c r="K40" s="130" t="s">
         <v>107</v>
       </c>
-      <c r="L40" s="133"/>
-      <c r="M40" s="134"/>
-      <c r="O40" s="130" t="s">
+      <c r="L40" s="131"/>
+      <c r="M40" s="132"/>
+      <c r="O40" s="128" t="s">
         <v>106</v>
       </c>
-      <c r="P40" s="131"/>
-      <c r="Q40" s="130" t="s">
+      <c r="P40" s="129"/>
+      <c r="Q40" s="128" t="s">
         <v>64</v>
       </c>
-      <c r="R40" s="135"/>
-      <c r="S40" s="131"/>
+      <c r="R40" s="142"/>
+      <c r="S40" s="129"/>
     </row>
     <row r="41" spans="2:19" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B41" s="33">
@@ -4675,29 +4649,29 @@
         <v>36</v>
       </c>
       <c r="F41" s="98" t="s">
-        <v>337</v>
+        <v>328</v>
       </c>
       <c r="G41" s="99" t="s">
         <v>275</v>
       </c>
-      <c r="I41" s="136" t="s">
+      <c r="I41" s="122" t="s">
         <v>8</v>
       </c>
-      <c r="J41" s="137"/>
-      <c r="K41" s="138" t="s">
+      <c r="J41" s="123"/>
+      <c r="K41" s="124" t="s">
         <v>125</v>
       </c>
-      <c r="L41" s="119"/>
-      <c r="M41" s="139"/>
-      <c r="O41" s="136" t="s">
+      <c r="L41" s="125"/>
+      <c r="M41" s="126"/>
+      <c r="O41" s="122" t="s">
         <v>8</v>
       </c>
-      <c r="P41" s="137"/>
-      <c r="Q41" s="138" t="s">
+      <c r="P41" s="123"/>
+      <c r="Q41" s="124" t="s">
         <v>174</v>
       </c>
-      <c r="R41" s="119"/>
-      <c r="S41" s="139"/>
+      <c r="R41" s="125"/>
+      <c r="S41" s="126"/>
     </row>
     <row r="42" spans="2:19" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B42" s="33">
@@ -4722,27 +4696,27 @@
       <c r="I42" s="67" t="s">
         <v>41</v>
       </c>
-      <c r="J42" s="128" t="s">
+      <c r="J42" s="127" t="s">
         <v>97</v>
       </c>
-      <c r="K42" s="128"/>
-      <c r="L42" s="128"/>
+      <c r="K42" s="127"/>
+      <c r="L42" s="127"/>
       <c r="M42" s="69" t="s">
         <v>8</v>
       </c>
       <c r="O42" s="67" t="s">
         <v>41</v>
       </c>
-      <c r="P42" s="128" t="s">
+      <c r="P42" s="127" t="s">
         <v>97</v>
       </c>
-      <c r="Q42" s="128"/>
-      <c r="R42" s="128"/>
+      <c r="Q42" s="127"/>
+      <c r="R42" s="127"/>
       <c r="S42" s="69" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="43" spans="2:19" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="43" spans="2:19" ht="33.75" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B43" s="33">
         <f t="shared" si="0"/>
         <v>26</v>
@@ -4756,8 +4730,8 @@
       <c r="E43" s="114" t="s">
         <v>237</v>
       </c>
-      <c r="F43" s="114" t="s">
-        <v>238</v>
+      <c r="F43" s="98" t="s">
+        <v>388</v>
       </c>
       <c r="G43" s="5" t="s">
         <v>248</v>
@@ -4765,22 +4739,22 @@
       <c r="I43" s="70">
         <v>1</v>
       </c>
-      <c r="J43" s="140" t="s">
+      <c r="J43" s="136" t="s">
         <v>20</v>
       </c>
-      <c r="K43" s="140"/>
-      <c r="L43" s="140"/>
+      <c r="K43" s="136"/>
+      <c r="L43" s="136"/>
       <c r="M43" s="71" t="s">
         <v>133</v>
       </c>
       <c r="O43" s="87">
         <v>1</v>
       </c>
-      <c r="P43" s="129" t="s">
+      <c r="P43" s="143" t="s">
         <v>21</v>
       </c>
-      <c r="Q43" s="129"/>
-      <c r="R43" s="129"/>
+      <c r="Q43" s="143"/>
+      <c r="R43" s="143"/>
       <c r="S43" s="88" t="s">
         <v>132</v>
       </c>
@@ -4823,11 +4797,11 @@
       <c r="O44" s="80">
         <v>2</v>
       </c>
-      <c r="P44" s="119" t="s">
+      <c r="P44" s="125" t="s">
         <v>20</v>
       </c>
-      <c r="Q44" s="119"/>
-      <c r="R44" s="119"/>
+      <c r="Q44" s="125"/>
+      <c r="R44" s="125"/>
       <c r="S44" s="82" t="s">
         <v>133</v>
       </c>
@@ -4883,25 +4857,25 @@
         <v>8</v>
       </c>
     </row>
-    <row r="46" spans="2:19" x14ac:dyDescent="0.3">
+    <row r="46" spans="2:19" ht="33" x14ac:dyDescent="0.3">
       <c r="B46" s="33">
         <f t="shared" si="0"/>
         <v>29</v>
       </c>
       <c r="C46" s="3" t="s">
-        <v>218</v>
+        <v>384</v>
       </c>
       <c r="D46" s="90" t="s">
-        <v>20</v>
-      </c>
-      <c r="E46" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="E46" s="2" t="s">
         <v>234</v>
       </c>
       <c r="F46" s="103" t="s">
-        <v>352</v>
-      </c>
-      <c r="G46" s="5" t="s">
-        <v>220</v>
+        <v>255</v>
+      </c>
+      <c r="G46" s="99" t="s">
+        <v>195</v>
       </c>
       <c r="I46" s="76">
         <v>2</v>
@@ -4934,25 +4908,25 @@
         <v>154</v>
       </c>
     </row>
-    <row r="47" spans="2:19" ht="50.25" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="47" spans="2:19" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B47" s="33">
         <f t="shared" si="0"/>
         <v>30</v>
       </c>
-      <c r="C47" s="112" t="s">
-        <v>219</v>
-      </c>
-      <c r="D47" s="113" t="s">
+      <c r="C47" s="3" t="s">
+        <v>218</v>
+      </c>
+      <c r="D47" s="90" t="s">
         <v>20</v>
       </c>
-      <c r="E47" s="111" t="s">
+      <c r="E47" s="1" t="s">
         <v>234</v>
       </c>
-      <c r="F47" s="115" t="s">
-        <v>385</v>
-      </c>
-      <c r="G47" s="112" t="s">
-        <v>221</v>
+      <c r="F47" s="103" t="s">
+        <v>340</v>
+      </c>
+      <c r="G47" s="5" t="s">
+        <v>220</v>
       </c>
       <c r="I47" s="80">
         <v>3</v>
@@ -4985,35 +4959,35 @@
         <v>155</v>
       </c>
     </row>
-    <row r="48" spans="2:19" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="48" spans="2:19" ht="50.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B48" s="33">
         <f t="shared" si="0"/>
         <v>31</v>
       </c>
-      <c r="C48" s="3" t="s">
-        <v>344</v>
-      </c>
-      <c r="D48" s="90" t="s">
-        <v>56</v>
-      </c>
-      <c r="E48" s="1" t="s">
-        <v>63</v>
-      </c>
-      <c r="F48" s="2" t="s">
-        <v>238</v>
-      </c>
-      <c r="G48" s="5" t="s">
-        <v>345</v>
-      </c>
-      <c r="I48" s="123" t="s">
+      <c r="C48" s="112" t="s">
+        <v>219</v>
+      </c>
+      <c r="D48" s="113" t="s">
+        <v>20</v>
+      </c>
+      <c r="E48" s="111" t="s">
+        <v>234</v>
+      </c>
+      <c r="F48" s="115" t="s">
+        <v>372</v>
+      </c>
+      <c r="G48" s="112" t="s">
+        <v>221</v>
+      </c>
+      <c r="I48" s="137" t="s">
         <v>104</v>
       </c>
-      <c r="J48" s="124"/>
-      <c r="K48" s="125" t="s">
+      <c r="J48" s="138"/>
+      <c r="K48" s="139" t="s">
         <v>65</v>
       </c>
-      <c r="L48" s="126"/>
-      <c r="M48" s="127"/>
+      <c r="L48" s="140"/>
+      <c r="M48" s="141"/>
       <c r="O48" s="83">
         <v>3</v>
       </c>
@@ -5030,25 +5004,25 @@
         <v>180</v>
       </c>
     </row>
-    <row r="49" spans="2:19" x14ac:dyDescent="0.3">
+    <row r="49" spans="2:19" ht="33" x14ac:dyDescent="0.3">
       <c r="B49" s="33">
         <f t="shared" si="0"/>
         <v>32</v>
       </c>
       <c r="C49" s="3" t="s">
-        <v>299</v>
-      </c>
-      <c r="D49" s="1">
-        <v>1</v>
-      </c>
-      <c r="E49" s="2" t="s">
-        <v>237</v>
+        <v>335</v>
+      </c>
+      <c r="D49" s="90" t="s">
+        <v>56</v>
+      </c>
+      <c r="E49" s="1" t="s">
+        <v>63</v>
       </c>
       <c r="F49" s="103" t="s">
-        <v>238</v>
+        <v>388</v>
       </c>
       <c r="G49" s="5" t="s">
-        <v>301</v>
+        <v>336</v>
       </c>
       <c r="O49" s="83">
         <v>4</v>
@@ -5072,19 +5046,19 @@
         <v>33</v>
       </c>
       <c r="C50" s="3" t="s">
-        <v>279</v>
-      </c>
-      <c r="D50" s="90" t="s">
-        <v>49</v>
-      </c>
-      <c r="E50" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="F50" s="1" t="s">
-        <v>280</v>
+        <v>299</v>
+      </c>
+      <c r="D50" s="1">
+        <v>1</v>
+      </c>
+      <c r="E50" s="2" t="s">
+        <v>237</v>
+      </c>
+      <c r="F50" s="103" t="s">
+        <v>238</v>
       </c>
       <c r="G50" s="5" t="s">
-        <v>54</v>
+        <v>301</v>
       </c>
       <c r="O50" s="83">
         <v>5</v>
@@ -5108,28 +5082,28 @@
         <v>34</v>
       </c>
       <c r="C51" s="3" t="s">
+        <v>279</v>
+      </c>
+      <c r="D51" s="90" t="s">
+        <v>49</v>
+      </c>
+      <c r="E51" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="F51" s="1" t="s">
         <v>280</v>
       </c>
-      <c r="D51" s="90" t="s">
-        <v>20</v>
-      </c>
-      <c r="E51" s="1" t="s">
-        <v>279</v>
-      </c>
-      <c r="F51" s="2" t="s">
-        <v>40</v>
-      </c>
       <c r="G51" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="I51" s="120" t="s">
+        <v>54</v>
+      </c>
+      <c r="I51" s="119" t="s">
         <v>102</v>
       </c>
       <c r="J51" s="121"/>
-      <c r="K51" s="120" t="s">
+      <c r="K51" s="119" t="s">
         <v>129</v>
       </c>
-      <c r="L51" s="122"/>
+      <c r="L51" s="120"/>
       <c r="M51" s="121"/>
       <c r="O51" s="83">
         <v>6</v>
@@ -5147,35 +5121,35 @@
         <v>168</v>
       </c>
     </row>
-    <row r="52" spans="2:19" ht="33" x14ac:dyDescent="0.3">
+    <row r="52" spans="2:19" x14ac:dyDescent="0.3">
       <c r="B52" s="33">
         <f t="shared" si="1"/>
         <v>35</v>
       </c>
       <c r="C52" s="3" t="s">
-        <v>222</v>
+        <v>280</v>
       </c>
       <c r="D52" s="90" t="s">
         <v>20</v>
       </c>
       <c r="E52" s="1" t="s">
-        <v>234</v>
-      </c>
-      <c r="F52" s="103" t="s">
-        <v>48</v>
+        <v>279</v>
+      </c>
+      <c r="F52" s="2" t="s">
+        <v>40</v>
       </c>
       <c r="G52" s="5" t="s">
-        <v>224</v>
-      </c>
-      <c r="I52" s="130" t="s">
+        <v>52</v>
+      </c>
+      <c r="I52" s="128" t="s">
         <v>108</v>
       </c>
-      <c r="J52" s="131"/>
-      <c r="K52" s="132" t="s">
+      <c r="J52" s="129"/>
+      <c r="K52" s="130" t="s">
         <v>130</v>
       </c>
-      <c r="L52" s="133"/>
-      <c r="M52" s="134"/>
+      <c r="L52" s="131"/>
+      <c r="M52" s="132"/>
       <c r="O52" s="83">
         <v>7</v>
       </c>
@@ -5192,35 +5166,35 @@
         <v>182</v>
       </c>
     </row>
-    <row r="53" spans="2:19" x14ac:dyDescent="0.3">
+    <row r="53" spans="2:19" ht="33" x14ac:dyDescent="0.3">
       <c r="B53" s="33">
         <f t="shared" si="1"/>
         <v>36</v>
       </c>
       <c r="C53" s="3" t="s">
-        <v>387</v>
+        <v>222</v>
       </c>
       <c r="D53" s="90" t="s">
         <v>20</v>
       </c>
       <c r="E53" s="1" t="s">
-        <v>382</v>
-      </c>
-      <c r="F53" s="1" t="s">
-        <v>238</v>
+        <v>234</v>
+      </c>
+      <c r="F53" s="103" t="s">
+        <v>48</v>
       </c>
       <c r="G53" s="5" t="s">
-        <v>388</v>
-      </c>
-      <c r="I53" s="130" t="s">
+        <v>224</v>
+      </c>
+      <c r="I53" s="128" t="s">
         <v>106</v>
       </c>
-      <c r="J53" s="131"/>
-      <c r="K53" s="132" t="s">
+      <c r="J53" s="129"/>
+      <c r="K53" s="130" t="s">
         <v>107</v>
       </c>
-      <c r="L53" s="133"/>
-      <c r="M53" s="134"/>
+      <c r="L53" s="131"/>
+      <c r="M53" s="132"/>
       <c r="O53" s="83">
         <v>8</v>
       </c>
@@ -5243,29 +5217,29 @@
         <v>37</v>
       </c>
       <c r="C54" s="3" t="s">
-        <v>360</v>
-      </c>
-      <c r="D54" s="1">
-        <v>1</v>
-      </c>
-      <c r="E54" s="2" t="s">
-        <v>378</v>
-      </c>
-      <c r="F54" s="2" t="s">
-        <v>379</v>
+        <v>374</v>
+      </c>
+      <c r="D54" s="90" t="s">
+        <v>20</v>
+      </c>
+      <c r="E54" s="1" t="s">
+        <v>369</v>
+      </c>
+      <c r="F54" s="1" t="s">
+        <v>238</v>
       </c>
       <c r="G54" s="5" t="s">
-        <v>370</v>
-      </c>
-      <c r="I54" s="136" t="s">
+        <v>375</v>
+      </c>
+      <c r="I54" s="122" t="s">
         <v>8</v>
       </c>
-      <c r="J54" s="137"/>
-      <c r="K54" s="138" t="s">
+      <c r="J54" s="123"/>
+      <c r="K54" s="124" t="s">
         <v>131</v>
       </c>
-      <c r="L54" s="119"/>
-      <c r="M54" s="139"/>
+      <c r="L54" s="125"/>
+      <c r="M54" s="126"/>
       <c r="O54" s="83">
         <v>9</v>
       </c>
@@ -5288,28 +5262,28 @@
         <v>38</v>
       </c>
       <c r="C55" s="3" t="s">
-        <v>362</v>
+        <v>348</v>
       </c>
       <c r="D55" s="1">
         <v>1</v>
       </c>
       <c r="E55" s="2" t="s">
-        <v>378</v>
+        <v>366</v>
       </c>
       <c r="F55" s="2" t="s">
-        <v>379</v>
+        <v>367</v>
       </c>
       <c r="G55" s="5" t="s">
-        <v>372</v>
+        <v>358</v>
       </c>
       <c r="I55" s="67" t="s">
         <v>41</v>
       </c>
-      <c r="J55" s="128" t="s">
+      <c r="J55" s="127" t="s">
         <v>97</v>
       </c>
-      <c r="K55" s="128"/>
-      <c r="L55" s="128"/>
+      <c r="K55" s="127"/>
+      <c r="L55" s="127"/>
       <c r="M55" s="69" t="s">
         <v>8</v>
       </c>
@@ -5335,40 +5309,40 @@
         <v>39</v>
       </c>
       <c r="C56" s="3" t="s">
-        <v>361</v>
+        <v>350</v>
       </c>
       <c r="D56" s="1">
         <v>1</v>
       </c>
       <c r="E56" s="2" t="s">
-        <v>378</v>
+        <v>366</v>
       </c>
       <c r="F56" s="2" t="s">
-        <v>380</v>
+        <v>367</v>
       </c>
       <c r="G56" s="5" t="s">
-        <v>371</v>
+        <v>360</v>
       </c>
       <c r="I56" s="87">
         <v>1</v>
       </c>
-      <c r="J56" s="129" t="s">
+      <c r="J56" s="143" t="s">
         <v>20</v>
       </c>
-      <c r="K56" s="129"/>
-      <c r="L56" s="129"/>
+      <c r="K56" s="143"/>
+      <c r="L56" s="143"/>
       <c r="M56" s="88" t="s">
         <v>133</v>
       </c>
-      <c r="O56" s="123" t="s">
+      <c r="O56" s="137" t="s">
         <v>104</v>
       </c>
-      <c r="P56" s="124"/>
-      <c r="Q56" s="125" t="s">
+      <c r="P56" s="138"/>
+      <c r="Q56" s="139" t="s">
         <v>238</v>
       </c>
-      <c r="R56" s="126"/>
-      <c r="S56" s="127"/>
+      <c r="R56" s="140"/>
+      <c r="S56" s="141"/>
     </row>
     <row r="57" spans="2:19" ht="33.75" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B57" s="33">
@@ -5376,28 +5350,28 @@
         <v>40</v>
       </c>
       <c r="C57" s="3" t="s">
-        <v>363</v>
+        <v>349</v>
       </c>
       <c r="D57" s="1">
         <v>1</v>
       </c>
       <c r="E57" s="2" t="s">
-        <v>378</v>
+        <v>366</v>
       </c>
       <c r="F57" s="2" t="s">
-        <v>380</v>
+        <v>368</v>
       </c>
       <c r="G57" s="5" t="s">
-        <v>373</v>
+        <v>359</v>
       </c>
       <c r="I57" s="80">
         <v>2</v>
       </c>
-      <c r="J57" s="119" t="s">
+      <c r="J57" s="125" t="s">
         <v>55</v>
       </c>
-      <c r="K57" s="119"/>
-      <c r="L57" s="119"/>
+      <c r="K57" s="125"/>
+      <c r="L57" s="125"/>
       <c r="M57" s="89" t="s">
         <v>134</v>
       </c>
@@ -5408,19 +5382,19 @@
         <v>41</v>
       </c>
       <c r="C58" s="3" t="s">
-        <v>364</v>
-      </c>
-      <c r="D58" s="33">
-        <v>1</v>
-      </c>
-      <c r="E58" s="1" t="s">
-        <v>358</v>
+        <v>351</v>
+      </c>
+      <c r="D58" s="1">
+        <v>1</v>
+      </c>
+      <c r="E58" s="2" t="s">
+        <v>366</v>
       </c>
       <c r="F58" s="2" t="s">
-        <v>342</v>
+        <v>368</v>
       </c>
       <c r="G58" s="5" t="s">
-        <v>374</v>
+        <v>361</v>
       </c>
       <c r="I58" s="67" t="s">
         <v>41</v>
@@ -5437,14 +5411,14 @@
       <c r="M58" s="69" t="s">
         <v>8</v>
       </c>
-      <c r="O58" s="120" t="s">
+      <c r="O58" s="119" t="s">
         <v>102</v>
       </c>
       <c r="P58" s="121"/>
-      <c r="Q58" s="120" t="s">
+      <c r="Q58" s="119" t="s">
         <v>184</v>
       </c>
-      <c r="R58" s="122"/>
+      <c r="R58" s="120"/>
       <c r="S58" s="121"/>
     </row>
     <row r="59" spans="2:19" x14ac:dyDescent="0.3">
@@ -5453,19 +5427,19 @@
         <v>42</v>
       </c>
       <c r="C59" s="3" t="s">
-        <v>192</v>
-      </c>
-      <c r="D59" s="90" t="s">
-        <v>20</v>
+        <v>352</v>
+      </c>
+      <c r="D59" s="33">
+        <v>1</v>
       </c>
       <c r="E59" s="1" t="s">
-        <v>235</v>
+        <v>346</v>
       </c>
       <c r="F59" s="2" t="s">
-        <v>44</v>
+        <v>333</v>
       </c>
       <c r="G59" s="5" t="s">
-        <v>193</v>
+        <v>362</v>
       </c>
       <c r="I59" s="72">
         <v>1</v>
@@ -5482,35 +5456,35 @@
       <c r="M59" s="75" t="s">
         <v>59</v>
       </c>
-      <c r="O59" s="130" t="s">
+      <c r="O59" s="128" t="s">
         <v>108</v>
       </c>
-      <c r="P59" s="131"/>
-      <c r="Q59" s="132" t="s">
+      <c r="P59" s="129"/>
+      <c r="Q59" s="130" t="s">
         <v>233</v>
       </c>
-      <c r="R59" s="133"/>
-      <c r="S59" s="134"/>
-    </row>
-    <row r="60" spans="2:19" ht="33" x14ac:dyDescent="0.3">
+      <c r="R59" s="131"/>
+      <c r="S59" s="132"/>
+    </row>
+    <row r="60" spans="2:19" x14ac:dyDescent="0.3">
       <c r="B60" s="33">
         <f t="shared" si="1"/>
         <v>43</v>
       </c>
       <c r="C60" s="3" t="s">
-        <v>395</v>
+        <v>192</v>
       </c>
       <c r="D60" s="90" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E60" s="1" t="s">
         <v>235</v>
       </c>
-      <c r="F60" s="103" t="s">
-        <v>254</v>
-      </c>
-      <c r="G60" s="99" t="s">
-        <v>194</v>
+      <c r="F60" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="G60" s="5" t="s">
+        <v>193</v>
       </c>
       <c r="I60" s="76">
         <v>2</v>
@@ -5527,15 +5501,15 @@
       <c r="M60" s="79" t="s">
         <v>66</v>
       </c>
-      <c r="O60" s="130" t="s">
+      <c r="O60" s="128" t="s">
         <v>106</v>
       </c>
-      <c r="P60" s="131"/>
-      <c r="Q60" s="130" t="s">
+      <c r="P60" s="129"/>
+      <c r="Q60" s="128" t="s">
         <v>64</v>
       </c>
-      <c r="R60" s="135"/>
-      <c r="S60" s="131"/>
+      <c r="R60" s="142"/>
+      <c r="S60" s="129"/>
     </row>
     <row r="61" spans="2:19" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B61" s="33">
@@ -5572,15 +5546,15 @@
       <c r="M61" s="85" t="s">
         <v>145</v>
       </c>
-      <c r="O61" s="136" t="s">
+      <c r="O61" s="122" t="s">
         <v>8</v>
       </c>
-      <c r="P61" s="137"/>
-      <c r="Q61" s="138" t="s">
+      <c r="P61" s="123"/>
+      <c r="Q61" s="124" t="s">
         <v>185</v>
       </c>
-      <c r="R61" s="119"/>
-      <c r="S61" s="139"/>
+      <c r="R61" s="125"/>
+      <c r="S61" s="126"/>
     </row>
     <row r="62" spans="2:19" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B62" s="33">
@@ -5620,11 +5594,11 @@
       <c r="O62" s="67" t="s">
         <v>41</v>
       </c>
-      <c r="P62" s="128" t="s">
+      <c r="P62" s="127" t="s">
         <v>97</v>
       </c>
-      <c r="Q62" s="128"/>
-      <c r="R62" s="128"/>
+      <c r="Q62" s="127"/>
+      <c r="R62" s="127"/>
       <c r="S62" s="69" t="s">
         <v>8</v>
       </c>
@@ -5667,11 +5641,11 @@
       <c r="O63" s="87">
         <v>1</v>
       </c>
-      <c r="P63" s="129" t="s">
+      <c r="P63" s="143" t="s">
         <v>21</v>
       </c>
-      <c r="Q63" s="129"/>
-      <c r="R63" s="129"/>
+      <c r="Q63" s="143"/>
+      <c r="R63" s="143"/>
       <c r="S63" s="88" t="s">
         <v>132</v>
       </c>
@@ -5682,19 +5656,19 @@
         <v>47</v>
       </c>
       <c r="C64" s="3" t="s">
-        <v>391</v>
-      </c>
-      <c r="D64" s="1">
-        <v>1</v>
+        <v>287</v>
+      </c>
+      <c r="D64" s="90" t="s">
+        <v>57</v>
       </c>
       <c r="E64" s="1" t="s">
-        <v>58</v>
+        <v>44</v>
       </c>
       <c r="F64" s="2" t="s">
-        <v>237</v>
+        <v>43</v>
       </c>
       <c r="G64" s="5" t="s">
-        <v>216</v>
+        <v>61</v>
       </c>
       <c r="I64" s="83">
         <v>6</v>
@@ -5714,11 +5688,11 @@
       <c r="O64" s="80">
         <v>2</v>
       </c>
-      <c r="P64" s="119" t="s">
+      <c r="P64" s="125" t="s">
         <v>20</v>
       </c>
-      <c r="Q64" s="119"/>
-      <c r="R64" s="119"/>
+      <c r="Q64" s="125"/>
+      <c r="R64" s="125"/>
       <c r="S64" s="82" t="s">
         <v>133</v>
       </c>
@@ -5729,19 +5703,19 @@
         <v>48</v>
       </c>
       <c r="C65" s="3" t="s">
-        <v>287</v>
-      </c>
-      <c r="D65" s="90" t="s">
-        <v>57</v>
+        <v>240</v>
+      </c>
+      <c r="D65" s="1">
+        <v>6</v>
       </c>
       <c r="E65" s="1" t="s">
         <v>44</v>
       </c>
       <c r="F65" s="2" t="s">
-        <v>43</v>
+        <v>237</v>
       </c>
       <c r="G65" s="5" t="s">
-        <v>61</v>
+        <v>241</v>
       </c>
       <c r="I65" s="83">
         <v>7</v>
@@ -5774,25 +5748,25 @@
         <v>8</v>
       </c>
     </row>
-    <row r="66" spans="2:19" x14ac:dyDescent="0.3">
+    <row r="66" spans="2:19" ht="33" x14ac:dyDescent="0.3">
       <c r="B66" s="33">
         <f t="shared" si="1"/>
         <v>49</v>
       </c>
-      <c r="C66" s="3" t="s">
-        <v>240</v>
-      </c>
-      <c r="D66" s="1">
-        <v>6</v>
-      </c>
-      <c r="E66" s="1" t="s">
+      <c r="C66" s="97" t="s">
+        <v>276</v>
+      </c>
+      <c r="D66" s="101" t="s">
+        <v>45</v>
+      </c>
+      <c r="E66" s="33" t="s">
         <v>44</v>
       </c>
-      <c r="F66" s="2" t="s">
-        <v>237</v>
-      </c>
-      <c r="G66" s="5" t="s">
-        <v>241</v>
+      <c r="F66" s="98" t="s">
+        <v>42</v>
+      </c>
+      <c r="G66" s="99" t="s">
+        <v>50</v>
       </c>
       <c r="I66" s="83">
         <v>8</v>
@@ -5825,25 +5799,25 @@
         <v>154</v>
       </c>
     </row>
-    <row r="67" spans="2:19" ht="33" x14ac:dyDescent="0.3">
+    <row r="67" spans="2:19" x14ac:dyDescent="0.3">
       <c r="B67" s="33">
         <f t="shared" si="1"/>
         <v>50</v>
       </c>
-      <c r="C67" s="97" t="s">
-        <v>276</v>
-      </c>
-      <c r="D67" s="101" t="s">
-        <v>45</v>
-      </c>
-      <c r="E67" s="33" t="s">
+      <c r="C67" s="3" t="s">
+        <v>282</v>
+      </c>
+      <c r="D67" s="90" t="s">
+        <v>55</v>
+      </c>
+      <c r="E67" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="F67" s="98" t="s">
-        <v>42</v>
-      </c>
-      <c r="G67" s="99" t="s">
-        <v>50</v>
+      <c r="F67" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="G67" s="5" t="s">
+        <v>59</v>
       </c>
       <c r="I67" s="83">
         <v>9</v>
@@ -5882,19 +5856,19 @@
         <v>51</v>
       </c>
       <c r="C68" s="3" t="s">
-        <v>282</v>
+        <v>285</v>
       </c>
       <c r="D68" s="90" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="E68" s="1" t="s">
         <v>44</v>
       </c>
       <c r="F68" s="2" t="s">
-        <v>58</v>
+        <v>237</v>
       </c>
       <c r="G68" s="5" t="s">
-        <v>59</v>
+        <v>304</v>
       </c>
       <c r="I68" s="83">
         <v>10</v>
@@ -5927,13 +5901,13 @@
         <v>28</v>
       </c>
     </row>
-    <row r="69" spans="2:19" x14ac:dyDescent="0.3">
+    <row r="69" spans="2:19" ht="49.5" x14ac:dyDescent="0.3">
       <c r="B69" s="33">
         <f t="shared" si="1"/>
         <v>52</v>
       </c>
       <c r="C69" s="3" t="s">
-        <v>285</v>
+        <v>283</v>
       </c>
       <c r="D69" s="90" t="s">
         <v>56</v>
@@ -5941,11 +5915,11 @@
       <c r="E69" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="F69" s="2" t="s">
-        <v>237</v>
+      <c r="F69" s="103" t="s">
+        <v>389</v>
       </c>
       <c r="G69" s="5" t="s">
-        <v>304</v>
+        <v>324</v>
       </c>
       <c r="I69" s="83">
         <v>11</v>
@@ -5978,13 +5952,13 @@
         <v>181</v>
       </c>
     </row>
-    <row r="70" spans="2:19" ht="33" x14ac:dyDescent="0.3">
+    <row r="70" spans="2:19" ht="49.5" x14ac:dyDescent="0.3">
       <c r="B70" s="33">
         <f t="shared" si="1"/>
         <v>53</v>
       </c>
       <c r="C70" s="3" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="D70" s="90" t="s">
         <v>56</v>
@@ -5993,10 +5967,10 @@
         <v>44</v>
       </c>
       <c r="F70" s="103" t="s">
-        <v>333</v>
+        <v>389</v>
       </c>
       <c r="G70" s="5" t="s">
-        <v>332</v>
+        <v>305</v>
       </c>
       <c r="I70" s="83">
         <v>12</v>
@@ -6035,19 +6009,19 @@
         <v>54</v>
       </c>
       <c r="C71" s="3" t="s">
-        <v>284</v>
-      </c>
-      <c r="D71" s="90" t="s">
-        <v>56</v>
+        <v>286</v>
+      </c>
+      <c r="D71" s="1">
+        <v>5</v>
       </c>
       <c r="E71" s="1" t="s">
         <v>44</v>
       </c>
       <c r="F71" s="2" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="G71" s="5" t="s">
-        <v>305</v>
+        <v>60</v>
       </c>
       <c r="I71" s="80">
         <v>13</v>
@@ -6086,38 +6060,38 @@
         <v>55</v>
       </c>
       <c r="C72" s="3" t="s">
-        <v>286</v>
+        <v>378</v>
       </c>
       <c r="D72" s="1">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="E72" s="1" t="s">
-        <v>44</v>
+        <v>58</v>
       </c>
       <c r="F72" s="2" t="s">
-        <v>64</v>
+        <v>237</v>
       </c>
       <c r="G72" s="5" t="s">
-        <v>60</v>
-      </c>
-      <c r="I72" s="123" t="s">
+        <v>216</v>
+      </c>
+      <c r="I72" s="137" t="s">
         <v>104</v>
       </c>
-      <c r="J72" s="124"/>
-      <c r="K72" s="125" t="s">
+      <c r="J72" s="138"/>
+      <c r="K72" s="139" t="s">
         <v>58</v>
       </c>
-      <c r="L72" s="126"/>
-      <c r="M72" s="127"/>
-      <c r="O72" s="123" t="s">
+      <c r="L72" s="140"/>
+      <c r="M72" s="141"/>
+      <c r="O72" s="137" t="s">
         <v>104</v>
       </c>
-      <c r="P72" s="124"/>
-      <c r="Q72" s="125" t="s">
+      <c r="P72" s="138"/>
+      <c r="Q72" s="139" t="s">
         <v>239</v>
       </c>
-      <c r="R72" s="126"/>
-      <c r="S72" s="127"/>
+      <c r="R72" s="140"/>
+      <c r="S72" s="141"/>
     </row>
     <row r="73" spans="2:19" ht="33" x14ac:dyDescent="0.3">
       <c r="B73" s="33">
@@ -6131,7 +6105,7 @@
         <v>20</v>
       </c>
       <c r="E73" s="102" t="s">
-        <v>396</v>
+        <v>382</v>
       </c>
       <c r="F73" s="2" t="s">
         <v>237</v>
@@ -6203,25 +6177,25 @@
         <v>214</v>
       </c>
     </row>
-    <row r="77" spans="2:19" x14ac:dyDescent="0.3">
+    <row r="77" spans="2:19" ht="33" x14ac:dyDescent="0.3">
       <c r="B77" s="33">
         <f t="shared" si="1"/>
         <v>60</v>
       </c>
       <c r="C77" s="3" t="s">
-        <v>204</v>
+        <v>381</v>
       </c>
       <c r="D77" s="90" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="E77" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="F77" s="111" t="s">
-        <v>234</v>
-      </c>
-      <c r="G77" s="5" t="s">
-        <v>206</v>
+        <v>235</v>
+      </c>
+      <c r="F77" s="103" t="s">
+        <v>254</v>
+      </c>
+      <c r="G77" s="99" t="s">
+        <v>194</v>
       </c>
     </row>
     <row r="78" spans="2:19" x14ac:dyDescent="0.3">
@@ -6229,10 +6203,10 @@
         <f t="shared" si="1"/>
         <v>61</v>
       </c>
-      <c r="C78" s="112" t="s">
-        <v>205</v>
-      </c>
-      <c r="D78" s="113" t="s">
+      <c r="C78" s="3" t="s">
+        <v>204</v>
+      </c>
+      <c r="D78" s="90" t="s">
         <v>20</v>
       </c>
       <c r="E78" s="1" t="s">
@@ -6241,8 +6215,8 @@
       <c r="F78" s="111" t="s">
         <v>234</v>
       </c>
-      <c r="G78" s="112" t="s">
-        <v>207</v>
+      <c r="G78" s="5" t="s">
+        <v>206</v>
       </c>
     </row>
     <row r="79" spans="2:19" x14ac:dyDescent="0.3">
@@ -6250,20 +6224,20 @@
         <f t="shared" si="1"/>
         <v>62</v>
       </c>
-      <c r="C79" s="3" t="s">
-        <v>349</v>
-      </c>
-      <c r="D79" s="1">
-        <v>1</v>
+      <c r="C79" s="112" t="s">
+        <v>205</v>
+      </c>
+      <c r="D79" s="113" t="s">
+        <v>20</v>
       </c>
       <c r="E79" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="F79" s="1" t="s">
-        <v>237</v>
-      </c>
-      <c r="G79" s="5" t="s">
-        <v>209</v>
+        <v>62</v>
+      </c>
+      <c r="F79" s="111" t="s">
+        <v>234</v>
+      </c>
+      <c r="G79" s="112" t="s">
+        <v>207</v>
       </c>
     </row>
     <row r="80" spans="2:19" x14ac:dyDescent="0.3">
@@ -6272,7 +6246,7 @@
         <v>63</v>
       </c>
       <c r="C80" s="3" t="s">
-        <v>199</v>
+        <v>339</v>
       </c>
       <c r="D80" s="1">
         <v>1</v>
@@ -6280,53 +6254,53 @@
       <c r="E80" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="F80" s="2" t="s">
+      <c r="F80" s="1" t="s">
         <v>237</v>
       </c>
       <c r="G80" s="5" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="81" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="B81" s="33">
+        <f t="shared" si="1"/>
+        <v>64</v>
+      </c>
+      <c r="C81" s="3" t="s">
+        <v>199</v>
+      </c>
+      <c r="D81" s="1">
+        <v>1</v>
+      </c>
+      <c r="E81" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="F81" s="2" t="s">
+        <v>237</v>
+      </c>
+      <c r="G81" s="5" t="s">
         <v>212</v>
       </c>
     </row>
-    <row r="81" spans="2:7" ht="49.5" x14ac:dyDescent="0.3">
-      <c r="B81" s="33">
-        <f t="shared" si="1"/>
-        <v>64</v>
-      </c>
-      <c r="C81" s="3" t="s">
+    <row r="82" spans="2:7" ht="49.5" x14ac:dyDescent="0.3">
+      <c r="B82" s="33">
+        <f t="shared" si="1"/>
+        <v>65</v>
+      </c>
+      <c r="C82" s="3" t="s">
         <v>278</v>
       </c>
-      <c r="D81" s="101" t="s">
+      <c r="D82" s="101" t="s">
         <v>46</v>
       </c>
-      <c r="E81" s="1" t="s">
+      <c r="E82" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="F81" s="2" t="s">
+      <c r="F82" s="2" t="s">
         <v>228</v>
       </c>
-      <c r="G81" s="5" t="s">
+      <c r="G82" s="5" t="s">
         <v>51</v>
-      </c>
-    </row>
-    <row r="82" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B82" s="33">
-        <f t="shared" si="1"/>
-        <v>65</v>
-      </c>
-      <c r="C82" s="3" t="s">
-        <v>203</v>
-      </c>
-      <c r="D82" s="1">
-        <v>1</v>
-      </c>
-      <c r="E82" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="F82" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="G82" s="5" t="s">
-        <v>217</v>
       </c>
     </row>
     <row r="83" spans="2:7" x14ac:dyDescent="0.3">
@@ -6335,19 +6309,19 @@
         <v>66</v>
       </c>
       <c r="C83" s="3" t="s">
-        <v>225</v>
-      </c>
-      <c r="D83" s="90" t="s">
-        <v>20</v>
+        <v>203</v>
+      </c>
+      <c r="D83" s="1">
+        <v>1</v>
       </c>
       <c r="E83" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="F83" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="F83" s="103" t="s">
-        <v>234</v>
-      </c>
       <c r="G83" s="5" t="s">
-        <v>223</v>
+        <v>217</v>
       </c>
     </row>
     <row r="84" spans="2:7" x14ac:dyDescent="0.3">
@@ -6355,41 +6329,41 @@
         <f t="shared" si="2"/>
         <v>67</v>
       </c>
-      <c r="C84" s="97" t="s">
+      <c r="C84" s="3" t="s">
+        <v>225</v>
+      </c>
+      <c r="D84" s="90" t="s">
+        <v>20</v>
+      </c>
+      <c r="E84" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="F84" s="103" t="s">
+        <v>234</v>
+      </c>
+      <c r="G84" s="5" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="85" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="B85" s="33">
+        <f t="shared" si="2"/>
+        <v>68</v>
+      </c>
+      <c r="C85" s="97" t="s">
         <v>190</v>
       </c>
-      <c r="D84" s="90" t="s">
+      <c r="D85" s="90" t="s">
         <v>21</v>
       </c>
-      <c r="E84" s="33" t="s">
+      <c r="E85" s="33" t="s">
         <v>39</v>
       </c>
-      <c r="F84" s="98" t="s">
-        <v>337</v>
-      </c>
-      <c r="G84" s="99" t="s">
+      <c r="F85" s="98" t="s">
+        <v>328</v>
+      </c>
+      <c r="G85" s="99" t="s">
         <v>191</v>
-      </c>
-    </row>
-    <row r="85" spans="2:7" ht="49.5" x14ac:dyDescent="0.3">
-      <c r="B85" s="33">
-        <f t="shared" si="2"/>
-        <v>68</v>
-      </c>
-      <c r="C85" s="93" t="s">
-        <v>397</v>
-      </c>
-      <c r="D85" s="94" t="s">
-        <v>21</v>
-      </c>
-      <c r="E85" s="92" t="s">
-        <v>35</v>
-      </c>
-      <c r="F85" s="95" t="s">
-        <v>390</v>
-      </c>
-      <c r="G85" s="96" t="s">
-        <v>37</v>
       </c>
     </row>
     <row r="86" spans="2:7" x14ac:dyDescent="0.3">
@@ -6413,88 +6387,88 @@
         <v>38</v>
       </c>
     </row>
-    <row r="87" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="87" spans="2:7" ht="49.5" x14ac:dyDescent="0.3">
       <c r="B87" s="33">
         <f t="shared" si="2"/>
         <v>70</v>
       </c>
-      <c r="C87" s="3" t="s">
-        <v>336</v>
-      </c>
-      <c r="D87" s="90" t="s">
+      <c r="C87" s="93" t="s">
+        <v>383</v>
+      </c>
+      <c r="D87" s="94" t="s">
         <v>21</v>
       </c>
-      <c r="E87" s="1" t="s">
-        <v>337</v>
-      </c>
-      <c r="F87" s="2" t="s">
+      <c r="E87" s="92" t="s">
         <v>35</v>
       </c>
-      <c r="G87" s="5" t="s">
-        <v>338</v>
-      </c>
-    </row>
-    <row r="88" spans="2:7" ht="66" x14ac:dyDescent="0.3">
+      <c r="F87" s="95" t="s">
+        <v>377</v>
+      </c>
+      <c r="G87" s="96" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="88" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B88" s="33">
         <f t="shared" si="2"/>
         <v>71</v>
       </c>
-      <c r="C88" s="104" t="s">
+      <c r="C88" s="3" t="s">
+        <v>327</v>
+      </c>
+      <c r="D88" s="90" t="s">
+        <v>21</v>
+      </c>
+      <c r="E88" s="1" t="s">
+        <v>328</v>
+      </c>
+      <c r="F88" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="G88" s="5" t="s">
+        <v>329</v>
+      </c>
+    </row>
+    <row r="89" spans="2:7" ht="33" x14ac:dyDescent="0.3">
+      <c r="B89" s="33">
+        <f t="shared" si="2"/>
+        <v>72</v>
+      </c>
+      <c r="C89" s="3" t="s">
+        <v>390</v>
+      </c>
+      <c r="D89" s="1">
+        <v>1</v>
+      </c>
+      <c r="E89" s="1" t="s">
+        <v>391</v>
+      </c>
+      <c r="F89" s="103" t="s">
+        <v>393</v>
+      </c>
+      <c r="G89" s="5" t="s">
+        <v>392</v>
+      </c>
+    </row>
+    <row r="90" spans="2:7" ht="66" x14ac:dyDescent="0.3">
+      <c r="B90" s="33">
+        <f t="shared" si="2"/>
+        <v>73</v>
+      </c>
+      <c r="C90" s="104" t="s">
         <v>256</v>
       </c>
-      <c r="D88" s="109" t="s">
+      <c r="D90" s="109" t="s">
         <v>20</v>
       </c>
-      <c r="E88" s="105" t="s">
+      <c r="E90" s="105" t="s">
         <v>238</v>
       </c>
-      <c r="F88" s="110" t="s">
-        <v>354</v>
-      </c>
-      <c r="G88" s="107" t="s">
+      <c r="F90" s="110" t="s">
+        <v>342</v>
+      </c>
+      <c r="G90" s="107" t="s">
         <v>259</v>
-      </c>
-    </row>
-    <row r="89" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B89" s="33">
-        <f t="shared" si="2"/>
-        <v>72</v>
-      </c>
-      <c r="C89" s="3" t="s">
-        <v>309</v>
-      </c>
-      <c r="D89" s="90" t="s">
-        <v>56</v>
-      </c>
-      <c r="E89" s="103" t="s">
-        <v>238</v>
-      </c>
-      <c r="F89" s="103" t="s">
-        <v>239</v>
-      </c>
-      <c r="G89" s="5" t="s">
-        <v>314</v>
-      </c>
-    </row>
-    <row r="90" spans="2:7" ht="33" x14ac:dyDescent="0.3">
-      <c r="B90" s="33">
-        <f t="shared" si="2"/>
-        <v>73</v>
-      </c>
-      <c r="C90" s="3" t="s">
-        <v>308</v>
-      </c>
-      <c r="D90" s="90" t="s">
-        <v>56</v>
-      </c>
-      <c r="E90" s="103" t="s">
-        <v>238</v>
-      </c>
-      <c r="F90" s="103" t="s">
-        <v>381</v>
-      </c>
-      <c r="G90" s="5" t="s">
-        <v>313</v>
       </c>
     </row>
     <row r="91" spans="2:7" x14ac:dyDescent="0.3">
@@ -6503,19 +6477,19 @@
         <v>74</v>
       </c>
       <c r="C91" s="3" t="s">
-        <v>359</v>
-      </c>
-      <c r="D91" s="1">
-        <v>1</v>
-      </c>
-      <c r="E91" s="2" t="s">
+        <v>308</v>
+      </c>
+      <c r="D91" s="90" t="s">
+        <v>56</v>
+      </c>
+      <c r="E91" s="103" t="s">
         <v>238</v>
       </c>
       <c r="F91" s="103" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="G91" s="5" t="s">
-        <v>376</v>
+        <v>310</v>
       </c>
     </row>
     <row r="92" spans="2:7" x14ac:dyDescent="0.3">
@@ -6523,20 +6497,20 @@
         <f t="shared" si="2"/>
         <v>75</v>
       </c>
-      <c r="C92" s="104" t="s">
-        <v>250</v>
-      </c>
-      <c r="D92" s="105">
-        <v>1</v>
-      </c>
-      <c r="E92" s="105" t="s">
+      <c r="C92" s="3" t="s">
+        <v>347</v>
+      </c>
+      <c r="D92" s="1">
+        <v>1</v>
+      </c>
+      <c r="E92" s="2" t="s">
         <v>238</v>
       </c>
-      <c r="F92" s="106" t="s">
-        <v>14</v>
-      </c>
-      <c r="G92" s="107" t="s">
-        <v>252</v>
+      <c r="F92" s="103" t="s">
+        <v>333</v>
+      </c>
+      <c r="G92" s="5" t="s">
+        <v>364</v>
       </c>
     </row>
     <row r="93" spans="2:7" x14ac:dyDescent="0.3">
@@ -6544,62 +6518,62 @@
         <f t="shared" si="2"/>
         <v>76</v>
       </c>
-      <c r="C93" s="3" t="s">
+      <c r="C93" s="104" t="s">
+        <v>250</v>
+      </c>
+      <c r="D93" s="105">
+        <v>1</v>
+      </c>
+      <c r="E93" s="105" t="s">
+        <v>238</v>
+      </c>
+      <c r="F93" s="106" t="s">
+        <v>14</v>
+      </c>
+      <c r="G93" s="107" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="94" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="B94" s="33">
+        <f t="shared" si="2"/>
+        <v>77</v>
+      </c>
+      <c r="C94" s="3" t="s">
         <v>267</v>
       </c>
-      <c r="D93" s="1">
-        <v>1</v>
-      </c>
-      <c r="E93" s="2" t="s">
+      <c r="D94" s="1">
+        <v>1</v>
+      </c>
+      <c r="E94" s="2" t="s">
         <v>238</v>
       </c>
-      <c r="F93" s="2" t="s">
+      <c r="F94" s="2" t="s">
         <v>239</v>
       </c>
-      <c r="G93" s="5" t="s">
+      <c r="G94" s="5" t="s">
         <v>270</v>
       </c>
     </row>
-    <row r="94" spans="2:7" ht="33" x14ac:dyDescent="0.3">
-      <c r="B94" s="33">
-        <f t="shared" si="2"/>
-        <v>77</v>
-      </c>
-      <c r="C94" s="104" t="s">
+    <row r="95" spans="2:7" ht="33" x14ac:dyDescent="0.3">
+      <c r="B95" s="33">
+        <f t="shared" si="2"/>
+        <v>78</v>
+      </c>
+      <c r="C95" s="104" t="s">
         <v>251</v>
       </c>
-      <c r="D94" s="105">
-        <v>1</v>
-      </c>
-      <c r="E94" s="105" t="s">
+      <c r="D95" s="105">
+        <v>1</v>
+      </c>
+      <c r="E95" s="105" t="s">
         <v>238</v>
       </c>
-      <c r="F94" s="108" t="s">
+      <c r="F95" s="108" t="s">
         <v>73</v>
       </c>
-      <c r="G94" s="107" t="s">
+      <c r="G95" s="107" t="s">
         <v>253</v>
-      </c>
-    </row>
-    <row r="95" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B95" s="33">
-        <f t="shared" si="2"/>
-        <v>78</v>
-      </c>
-      <c r="C95" s="112" t="s">
-        <v>260</v>
-      </c>
-      <c r="D95" s="113" t="s">
-        <v>20</v>
-      </c>
-      <c r="E95" s="111" t="s">
-        <v>238</v>
-      </c>
-      <c r="F95" s="118" t="s">
-        <v>342</v>
-      </c>
-      <c r="G95" s="112" t="s">
-        <v>261</v>
       </c>
     </row>
     <row r="96" spans="2:7" x14ac:dyDescent="0.3">
@@ -6607,20 +6581,20 @@
         <f t="shared" si="2"/>
         <v>79</v>
       </c>
-      <c r="C96" s="3" t="s">
-        <v>350</v>
-      </c>
-      <c r="D96" s="1">
-        <v>1</v>
-      </c>
-      <c r="E96" s="103" t="s">
+      <c r="C96" s="112" t="s">
+        <v>260</v>
+      </c>
+      <c r="D96" s="113" t="s">
+        <v>20</v>
+      </c>
+      <c r="E96" s="111" t="s">
         <v>238</v>
       </c>
-      <c r="F96" s="103" t="s">
-        <v>239</v>
-      </c>
-      <c r="G96" s="5" t="s">
-        <v>319</v>
+      <c r="F96" s="118" t="s">
+        <v>333</v>
+      </c>
+      <c r="G96" s="112" t="s">
+        <v>261</v>
       </c>
     </row>
     <row r="97" spans="2:7" ht="33" x14ac:dyDescent="0.3">
@@ -6629,7 +6603,7 @@
         <v>80</v>
       </c>
       <c r="C97" s="3" t="s">
-        <v>334</v>
+        <v>325</v>
       </c>
       <c r="D97" s="90" t="s">
         <v>56</v>
@@ -6638,10 +6612,10 @@
         <v>238</v>
       </c>
       <c r="F97" s="103" t="s">
-        <v>346</v>
+        <v>337</v>
       </c>
       <c r="G97" s="5" t="s">
-        <v>335</v>
+        <v>326</v>
       </c>
     </row>
     <row r="98" spans="2:7" ht="33" x14ac:dyDescent="0.3">
@@ -6650,7 +6624,7 @@
         <v>81</v>
       </c>
       <c r="C98" s="3" t="s">
-        <v>339</v>
+        <v>330</v>
       </c>
       <c r="D98" s="1">
         <v>1</v>
@@ -6659,7 +6633,7 @@
         <v>238</v>
       </c>
       <c r="F98" s="103" t="s">
-        <v>340</v>
+        <v>331</v>
       </c>
       <c r="G98" s="5" t="s">
         <v>302</v>
@@ -6671,19 +6645,19 @@
         <v>82</v>
       </c>
       <c r="C99" s="104" t="s">
-        <v>365</v>
+        <v>353</v>
       </c>
       <c r="D99" s="109" t="s">
         <v>20</v>
       </c>
       <c r="E99" s="117" t="s">
-        <v>342</v>
+        <v>333</v>
       </c>
       <c r="F99" s="106" t="s">
         <v>17</v>
       </c>
       <c r="G99" s="107" t="s">
-        <v>343</v>
+        <v>334</v>
       </c>
     </row>
     <row r="100" spans="2:7" x14ac:dyDescent="0.3">
@@ -6692,7 +6666,7 @@
         <v>83</v>
       </c>
       <c r="C100" s="3" t="s">
-        <v>377</v>
+        <v>365</v>
       </c>
       <c r="D100" s="90" t="s">
         <v>20</v>
@@ -6701,10 +6675,10 @@
         <v>238</v>
       </c>
       <c r="F100" s="1" t="s">
-        <v>342</v>
+        <v>333</v>
       </c>
       <c r="G100" s="5" t="s">
-        <v>389</v>
+        <v>376</v>
       </c>
     </row>
     <row r="101" spans="2:7" ht="82.5" x14ac:dyDescent="0.3">
@@ -6722,7 +6696,7 @@
         <v>239</v>
       </c>
       <c r="F101" s="103" t="s">
-        <v>386</v>
+        <v>373</v>
       </c>
       <c r="G101" s="5" t="s">
         <v>273</v>
@@ -6734,19 +6708,19 @@
         <v>85</v>
       </c>
       <c r="C102" s="3" t="s">
-        <v>311</v>
-      </c>
-      <c r="D102" s="90" t="s">
-        <v>56</v>
-      </c>
-      <c r="E102" s="103" t="s">
+        <v>268</v>
+      </c>
+      <c r="D102" s="1">
+        <v>1</v>
+      </c>
+      <c r="E102" s="2" t="s">
         <v>239</v>
       </c>
       <c r="F102" s="2" t="s">
-        <v>64</v>
+        <v>80</v>
       </c>
       <c r="G102" s="5" t="s">
-        <v>316</v>
+        <v>271</v>
       </c>
     </row>
     <row r="103" spans="2:7" x14ac:dyDescent="0.3">
@@ -6755,152 +6729,98 @@
         <v>86</v>
       </c>
       <c r="C103" s="3" t="s">
-        <v>310</v>
+        <v>289</v>
       </c>
       <c r="D103" s="90" t="s">
+        <v>20</v>
+      </c>
+      <c r="E103" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="F103" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="G103" s="5" t="s">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="104" spans="2:7" ht="33" x14ac:dyDescent="0.3">
+      <c r="B104" s="33">
+        <f t="shared" si="2"/>
+        <v>87</v>
+      </c>
+      <c r="C104" s="3" t="s">
+        <v>313</v>
+      </c>
+      <c r="D104" s="90" t="s">
         <v>56</v>
       </c>
-      <c r="E103" s="103" t="s">
+      <c r="E104" s="1" t="s">
         <v>239</v>
       </c>
-      <c r="F103" s="103" t="s">
-        <v>62</v>
-      </c>
-      <c r="G103" s="5" t="s">
-        <v>315</v>
-      </c>
-    </row>
-    <row r="104" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B104" s="33">
-        <f t="shared" si="2"/>
-        <v>87</v>
-      </c>
-      <c r="C104" s="3" t="s">
-        <v>268</v>
-      </c>
-      <c r="D104" s="1">
-        <v>1</v>
-      </c>
-      <c r="E104" s="2" t="s">
+      <c r="F104" s="103" t="s">
+        <v>344</v>
+      </c>
+      <c r="G104" s="5" t="s">
+        <v>314</v>
+      </c>
+    </row>
+    <row r="105" spans="2:7" ht="33" x14ac:dyDescent="0.3">
+      <c r="B105" s="33">
+        <f t="shared" si="2"/>
+        <v>88</v>
+      </c>
+      <c r="C105" s="3" t="s">
+        <v>300</v>
+      </c>
+      <c r="D105" s="1">
+        <v>1</v>
+      </c>
+      <c r="E105" s="2" t="s">
         <v>239</v>
       </c>
-      <c r="F104" s="2" t="s">
-        <v>80</v>
-      </c>
-      <c r="G104" s="5" t="s">
-        <v>271</v>
-      </c>
-    </row>
-    <row r="105" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B105" s="33">
-        <f t="shared" si="2"/>
-        <v>88</v>
-      </c>
-      <c r="C105" s="3" t="s">
-        <v>289</v>
-      </c>
-      <c r="D105" s="90" t="s">
-        <v>20</v>
-      </c>
-      <c r="E105" s="1" t="s">
-        <v>80</v>
-      </c>
-      <c r="F105" s="2" t="s">
-        <v>62</v>
+      <c r="F105" s="103" t="s">
+        <v>344</v>
       </c>
       <c r="G105" s="5" t="s">
-        <v>290</v>
+        <v>303</v>
       </c>
     </row>
     <row r="106" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B106" s="33">
-        <f t="shared" si="2"/>
-        <v>89</v>
-      </c>
-      <c r="C106" s="3" t="s">
-        <v>351</v>
-      </c>
-      <c r="D106" s="1">
-        <v>1</v>
-      </c>
-      <c r="E106" s="103" t="s">
-        <v>239</v>
-      </c>
-      <c r="F106" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="G106" s="5" t="s">
-        <v>320</v>
-      </c>
-    </row>
-    <row r="107" spans="2:7" ht="33" x14ac:dyDescent="0.3">
-      <c r="B107" s="33">
-        <f t="shared" si="2"/>
-        <v>90</v>
-      </c>
-      <c r="C107" s="3" t="s">
-        <v>321</v>
-      </c>
-      <c r="D107" s="90" t="s">
-        <v>56</v>
-      </c>
-      <c r="E107" s="1" t="s">
-        <v>239</v>
-      </c>
-      <c r="F107" s="103" t="s">
-        <v>356</v>
-      </c>
-      <c r="G107" s="5" t="s">
-        <v>322</v>
-      </c>
-    </row>
-    <row r="108" spans="2:7" ht="33" x14ac:dyDescent="0.3">
-      <c r="B108" s="33">
-        <f t="shared" si="2"/>
-        <v>91</v>
-      </c>
-      <c r="C108" s="3" t="s">
-        <v>300</v>
-      </c>
-      <c r="D108" s="1">
-        <v>1</v>
-      </c>
-      <c r="E108" s="2" t="s">
-        <v>239</v>
-      </c>
-      <c r="F108" s="103" t="s">
-        <v>356</v>
-      </c>
-      <c r="G108" s="5" t="s">
-        <v>303</v>
-      </c>
-    </row>
-    <row r="109" spans="2:7" ht="33" x14ac:dyDescent="0.3">
-      <c r="B109" s="33">
-        <f t="shared" si="2"/>
-        <v>92</v>
-      </c>
-      <c r="C109" s="3" t="s">
-        <v>401</v>
-      </c>
-      <c r="D109" s="1">
-        <v>1</v>
-      </c>
-      <c r="E109" s="102" t="s">
-        <v>392</v>
-      </c>
-      <c r="F109" s="103" t="s">
-        <v>394</v>
-      </c>
-      <c r="G109" s="5" t="s">
-        <v>393</v>
-      </c>
+      <c r="B106" s="33" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="F106" s="103"/>
+    </row>
+    <row r="107" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="B107" s="33" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="F107" s="103"/>
+    </row>
+    <row r="108" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="B108" s="33" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="E108" s="2"/>
+      <c r="F108" s="103"/>
+    </row>
+    <row r="109" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="B109" s="33" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="F109" s="103"/>
     </row>
     <row r="110" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B110" s="33" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
+      <c r="F110" s="103"/>
     </row>
     <row r="111" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B111" s="33" t="str">
@@ -7089,39 +7009,51 @@
     </sortState>
   </autoFilter>
   <mergeCells count="102">
-    <mergeCell ref="K2:M2"/>
-    <mergeCell ref="I18:J18"/>
-    <mergeCell ref="K18:M18"/>
-    <mergeCell ref="I21:J21"/>
-    <mergeCell ref="K21:M21"/>
-    <mergeCell ref="J22:L22"/>
-    <mergeCell ref="I3:J3"/>
-    <mergeCell ref="K3:M3"/>
-    <mergeCell ref="B2:G2"/>
-    <mergeCell ref="J6:L6"/>
-    <mergeCell ref="J7:L7"/>
-    <mergeCell ref="I5:J5"/>
-    <mergeCell ref="K5:M5"/>
-    <mergeCell ref="I2:J2"/>
-    <mergeCell ref="J23:L23"/>
-    <mergeCell ref="I12:J12"/>
-    <mergeCell ref="K12:M12"/>
-    <mergeCell ref="I4:J4"/>
-    <mergeCell ref="K4:M4"/>
-    <mergeCell ref="I20:J20"/>
-    <mergeCell ref="K20:M20"/>
-    <mergeCell ref="I19:J19"/>
-    <mergeCell ref="K19:M19"/>
-    <mergeCell ref="I41:J41"/>
-    <mergeCell ref="K41:M41"/>
-    <mergeCell ref="J42:L42"/>
-    <mergeCell ref="J43:L43"/>
-    <mergeCell ref="I32:J32"/>
-    <mergeCell ref="K32:M32"/>
-    <mergeCell ref="I38:J38"/>
-    <mergeCell ref="K38:M38"/>
-    <mergeCell ref="I39:J39"/>
-    <mergeCell ref="K39:M39"/>
+    <mergeCell ref="P24:R24"/>
+    <mergeCell ref="O38:P38"/>
+    <mergeCell ref="Q38:S38"/>
+    <mergeCell ref="P44:R44"/>
+    <mergeCell ref="O56:P56"/>
+    <mergeCell ref="Q56:S56"/>
+    <mergeCell ref="P62:R62"/>
+    <mergeCell ref="P63:R63"/>
+    <mergeCell ref="P64:R64"/>
+    <mergeCell ref="O72:P72"/>
+    <mergeCell ref="Q72:S72"/>
+    <mergeCell ref="P8:R8"/>
+    <mergeCell ref="O59:P59"/>
+    <mergeCell ref="Q59:S59"/>
+    <mergeCell ref="O60:P60"/>
+    <mergeCell ref="Q60:S60"/>
+    <mergeCell ref="O61:P61"/>
+    <mergeCell ref="Q61:S61"/>
+    <mergeCell ref="P42:R42"/>
+    <mergeCell ref="P43:R43"/>
+    <mergeCell ref="O58:P58"/>
+    <mergeCell ref="Q58:S58"/>
+    <mergeCell ref="O39:P39"/>
+    <mergeCell ref="Q39:S39"/>
+    <mergeCell ref="O40:P40"/>
+    <mergeCell ref="Q40:S40"/>
+    <mergeCell ref="O41:P41"/>
+    <mergeCell ref="Q41:S41"/>
+    <mergeCell ref="P22:R22"/>
+    <mergeCell ref="P23:R23"/>
+    <mergeCell ref="O36:P36"/>
+    <mergeCell ref="Q36:S36"/>
+    <mergeCell ref="O19:P19"/>
+    <mergeCell ref="Q19:S19"/>
+    <mergeCell ref="O20:P20"/>
+    <mergeCell ref="Q20:S20"/>
+    <mergeCell ref="O21:P21"/>
+    <mergeCell ref="Q21:S21"/>
+    <mergeCell ref="Q5:S5"/>
+    <mergeCell ref="P6:R6"/>
+    <mergeCell ref="P7:R7"/>
+    <mergeCell ref="O16:P16"/>
+    <mergeCell ref="Q16:S16"/>
+    <mergeCell ref="O18:P18"/>
+    <mergeCell ref="Q18:S18"/>
     <mergeCell ref="I72:J72"/>
     <mergeCell ref="K72:M72"/>
     <mergeCell ref="J57:L57"/>
@@ -7146,51 +7078,39 @@
     <mergeCell ref="K52:M52"/>
     <mergeCell ref="I40:J40"/>
     <mergeCell ref="K40:M40"/>
-    <mergeCell ref="Q19:S19"/>
-    <mergeCell ref="O20:P20"/>
-    <mergeCell ref="Q20:S20"/>
-    <mergeCell ref="O21:P21"/>
-    <mergeCell ref="Q21:S21"/>
-    <mergeCell ref="Q5:S5"/>
-    <mergeCell ref="P6:R6"/>
-    <mergeCell ref="P7:R7"/>
-    <mergeCell ref="O16:P16"/>
-    <mergeCell ref="Q16:S16"/>
-    <mergeCell ref="O18:P18"/>
-    <mergeCell ref="Q18:S18"/>
-    <mergeCell ref="O72:P72"/>
-    <mergeCell ref="Q72:S72"/>
-    <mergeCell ref="P8:R8"/>
-    <mergeCell ref="O59:P59"/>
-    <mergeCell ref="Q59:S59"/>
-    <mergeCell ref="O60:P60"/>
-    <mergeCell ref="Q60:S60"/>
-    <mergeCell ref="O61:P61"/>
-    <mergeCell ref="Q61:S61"/>
-    <mergeCell ref="P42:R42"/>
-    <mergeCell ref="P43:R43"/>
-    <mergeCell ref="O58:P58"/>
-    <mergeCell ref="Q58:S58"/>
-    <mergeCell ref="O39:P39"/>
-    <mergeCell ref="Q39:S39"/>
-    <mergeCell ref="O40:P40"/>
-    <mergeCell ref="Q40:S40"/>
-    <mergeCell ref="O41:P41"/>
-    <mergeCell ref="Q41:S41"/>
-    <mergeCell ref="P22:R22"/>
-    <mergeCell ref="P23:R23"/>
-    <mergeCell ref="O36:P36"/>
-    <mergeCell ref="Q36:S36"/>
-    <mergeCell ref="O19:P19"/>
-    <mergeCell ref="P24:R24"/>
-    <mergeCell ref="O38:P38"/>
-    <mergeCell ref="Q38:S38"/>
-    <mergeCell ref="P44:R44"/>
-    <mergeCell ref="O56:P56"/>
-    <mergeCell ref="Q56:S56"/>
-    <mergeCell ref="P62:R62"/>
-    <mergeCell ref="P63:R63"/>
-    <mergeCell ref="P64:R64"/>
+    <mergeCell ref="I41:J41"/>
+    <mergeCell ref="K41:M41"/>
+    <mergeCell ref="J42:L42"/>
+    <mergeCell ref="J43:L43"/>
+    <mergeCell ref="I32:J32"/>
+    <mergeCell ref="K32:M32"/>
+    <mergeCell ref="I38:J38"/>
+    <mergeCell ref="K38:M38"/>
+    <mergeCell ref="I39:J39"/>
+    <mergeCell ref="K39:M39"/>
+    <mergeCell ref="J23:L23"/>
+    <mergeCell ref="I12:J12"/>
+    <mergeCell ref="K12:M12"/>
+    <mergeCell ref="I4:J4"/>
+    <mergeCell ref="K4:M4"/>
+    <mergeCell ref="I20:J20"/>
+    <mergeCell ref="K20:M20"/>
+    <mergeCell ref="I19:J19"/>
+    <mergeCell ref="K19:M19"/>
+    <mergeCell ref="K2:M2"/>
+    <mergeCell ref="I18:J18"/>
+    <mergeCell ref="K18:M18"/>
+    <mergeCell ref="I21:J21"/>
+    <mergeCell ref="K21:M21"/>
+    <mergeCell ref="J22:L22"/>
+    <mergeCell ref="I3:J3"/>
+    <mergeCell ref="K3:M3"/>
+    <mergeCell ref="B2:G2"/>
+    <mergeCell ref="J6:L6"/>
+    <mergeCell ref="J7:L7"/>
+    <mergeCell ref="I5:J5"/>
+    <mergeCell ref="K5:M5"/>
+    <mergeCell ref="I2:J2"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -7212,25 +7132,25 @@
   <sheetData>
     <row r="2" spans="2:8" ht="49.5" x14ac:dyDescent="0.3">
       <c r="B2" s="1" t="s">
-        <v>323</v>
+        <v>315</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>324</v>
+        <v>316</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>325</v>
+        <v>317</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>326</v>
+        <v>318</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>327</v>
+        <v>319</v>
       </c>
       <c r="G2" s="102" t="s">
-        <v>328</v>
+        <v>320</v>
       </c>
       <c r="H2" s="102" t="s">
-        <v>329</v>
+        <v>321</v>
       </c>
     </row>
     <row r="3" spans="2:8" x14ac:dyDescent="0.3">

</xml_diff>